<commit_message>
L32 Moment kinds settled; document the git process
</commit_message>
<xml_diff>
--- a/docs/substrate-lists.xlsx
+++ b/docs/substrate-lists.xlsx
@@ -287,7 +287,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -490,6 +490,15 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -746,7 +755,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:C69"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" style="18" min="1" max="1"/>
     <col width="42" customWidth="1" style="18" min="2" max="2"/>
@@ -1343,7 +1352,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -1726,7 +1735,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -2116,7 +2125,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -2506,7 +2515,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -2896,7 +2905,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -3394,7 +3403,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -3784,7 +3793,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -4167,7 +4176,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -4709,7 +4718,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" style="18" min="1" max="1"/>
     <col width="20" customWidth="1" style="18" min="2" max="2"/>
@@ -5455,7 +5464,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:Q94"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="20" customWidth="1" style="18" min="1" max="1"/>
     <col width="14" customWidth="1" style="18" min="2" max="2"/>
@@ -7707,7 +7716,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:D36"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" style="18" min="1" max="1"/>
     <col width="34" customWidth="1" style="18" min="2" max="2"/>
@@ -7729,6 +7738,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -8252,21 +8262,21 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="A30" s="78" t="inlineStr">
         <is>
           <t>L32 · Moment kinds</t>
         </is>
       </c>
-      <c r="B30" s="18" t="inlineStr">
-        <is>
-          <t>PENDING · BLOCKING · NEXT</t>
-        </is>
-      </c>
-      <c r="C30" s="18">
+      <c r="B30" s="78" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+      <c r="C30" s="78">
         <f>COUNTA('L32 Moment kinds'!A8:A47)</f>
         <v/>
       </c>
-      <c r="D30" s="18">
+      <c r="D30" s="78">
         <f>IF(C30&gt;0,"started","not started")</f>
         <v/>
       </c>
@@ -8287,6 +8297,7 @@
       </c>
       <c r="C32" s="24" t="n"/>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>
@@ -8334,7 +8345,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -8908,7 +8919,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" style="19" min="1" max="1"/>
     <col width="32" customWidth="1" style="19" min="2" max="2"/>
@@ -9457,7 +9468,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" style="19" min="1" max="1"/>
     <col width="44" customWidth="1" style="19" min="2" max="2"/>
@@ -9838,7 +9849,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" style="19" min="1" max="1"/>
     <col width="42" customWidth="1" style="19" min="2" max="2"/>
@@ -10101,7 +10112,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" style="19" min="1" max="1"/>
     <col width="38" customWidth="1" style="19" min="2" max="2"/>
@@ -10558,7 +10569,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:H47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="34" customWidth="1" style="18" min="2" max="2"/>
@@ -11426,7 +11437,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -12052,7 +12063,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" style="19" min="1" max="1"/>
     <col width="46" customWidth="1" style="19" min="2" max="2"/>
@@ -12446,8 +12457,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" style="19" min="1" max="1"/>
     <col width="40" customWidth="1" style="19" min="2" max="2"/>
@@ -12466,7 +12477,7 @@
     <row r="2">
       <c r="A2" s="64" t="inlineStr">
         <is>
-          <t>PENDING · BLOCKING · NEW Aug 2026</t>
+          <t>SETTLED · Aug 2026</t>
         </is>
       </c>
     </row>
@@ -12544,286 +12555,388 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="70" t="inlineStr">
-        <is>
-          <t>turn ownership (mine / not mine)</t>
-        </is>
-      </c>
-      <c r="B8" s="70" t="inlineStr">
-        <is>
-          <t>Whether the current Moment belongs to this Entity</t>
-        </is>
-      </c>
-      <c r="C8" s="70" t="inlineStr">
-        <is>
-          <t>L31 respond, interrupt</t>
-        </is>
-      </c>
-      <c r="D8" s="70" t="inlineStr">
-        <is>
-          <t>SETTLED IN PRINCIPLE</t>
-        </is>
-      </c>
-      <c r="E8" s="70" t="inlineStr">
-        <is>
-          <t>The load-bearing one. Without ownership as a Substrate concept, a reaction cannot be expressed portably at all, and a reaction is not a genre feature.</t>
-        </is>
-      </c>
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>now</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
+        <is>
+          <t>the Moment currently resolving</t>
+        </is>
+      </c>
+      <c r="C8" s="76" t="inlineStr">
+        <is>
+          <t>respond, interrupt</t>
+        </is>
+      </c>
+      <c r="D8" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="E8" s="76" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="70" t="inlineStr">
-        <is>
-          <t>start of my turn</t>
-        </is>
-      </c>
-      <c r="B9" s="70" t="inlineStr"/>
-      <c r="C9" s="70" t="inlineStr">
-        <is>
-          <t>pinning, Budget refresh</t>
-        </is>
-      </c>
-      <c r="D9" s="70" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E9" s="70" t="inlineStr"/>
+      <c r="A9" s="76" t="inlineStr">
+        <is>
+          <t>next</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>the following Moment, whatever it is</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>Loose time</t>
+        </is>
+      </c>
+      <c r="D9" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="E9" s="76" t="inlineStr">
+        <is>
+          <t>The only anchor available when nobody has a turn.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="70" t="inlineStr">
-        <is>
-          <t>end of my turn</t>
-        </is>
-      </c>
-      <c r="B10" s="70" t="inlineStr"/>
-      <c r="C10" s="70" t="inlineStr">
-        <is>
-          <t>pinning, duration</t>
-        </is>
-      </c>
-      <c r="D10" s="70" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E10" s="70" t="inlineStr"/>
+      <c r="A10" s="76" t="inlineStr">
+        <is>
+          <t>turn start (E)</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>the start of Entity E's turn — E MAY BE SELF</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>the workhorse</t>
+        </is>
+      </c>
+      <c r="D10" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="E10" s="76" t="inlineStr">
+        <is>
+          <t>Collapses what were four entries into two. "My turn" is just E = self.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="70" t="inlineStr">
-        <is>
-          <t>start of a named Entity's turn</t>
-        </is>
-      </c>
-      <c r="B11" s="70" t="inlineStr"/>
-      <c r="C11" s="70" t="inlineStr">
-        <is>
-          <t>pinning to someone else</t>
-        </is>
-      </c>
-      <c r="D11" s="70" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E11" s="70" t="inlineStr">
-        <is>
-          <t>A reference, never a computed tick — turn order may change before it arrives.</t>
-        </is>
-      </c>
+      <c r="A11" s="76" t="inlineStr">
+        <is>
+          <t>turn end (E)</t>
+        </is>
+      </c>
+      <c r="B11" s="76" t="inlineStr">
+        <is>
+          <t>the end of Entity E's turn</t>
+        </is>
+      </c>
+      <c r="C11" s="76" t="inlineStr">
+        <is>
+          <t>durations, upkeep</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="E11" s="76" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="70" t="inlineStr">
-        <is>
-          <t>end of a named Entity's turn</t>
-        </is>
-      </c>
-      <c r="B12" s="70" t="inlineStr"/>
-      <c r="C12" s="70" t="inlineStr">
-        <is>
-          <t>pinning to someone else</t>
-        </is>
-      </c>
-      <c r="D12" s="70" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E12" s="70" t="inlineStr"/>
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>round start</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr"/>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>round-scoped effects</t>
+        </is>
+      </c>
+      <c r="D12" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="E12" s="76" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="70" t="inlineStr">
-        <is>
-          <t>start of the round</t>
-        </is>
-      </c>
-      <c r="B13" s="70" t="inlineStr"/>
-      <c r="C13" s="70" t="inlineStr">
-        <is>
-          <t>round-scoped effects</t>
-        </is>
-      </c>
-      <c r="D13" s="70" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E13" s="70" t="inlineStr"/>
+      <c r="A13" s="76" t="inlineStr">
+        <is>
+          <t>round end</t>
+        </is>
+      </c>
+      <c r="B13" s="76" t="inlineStr"/>
+      <c r="C13" s="76" t="inlineStr">
+        <is>
+          <t>round-scoped effects, cap reset</t>
+        </is>
+      </c>
+      <c r="D13" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="E13" s="76" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="70" t="inlineStr">
-        <is>
-          <t>end of the round</t>
-        </is>
-      </c>
-      <c r="B14" s="70" t="inlineStr"/>
-      <c r="C14" s="70" t="inlineStr">
-        <is>
-          <t>round-scoped effects, cap reset</t>
-        </is>
-      </c>
-      <c r="D14" s="70" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E14" s="70" t="inlineStr"/>
+      <c r="A14" s="76" t="inlineStr">
+        <is>
+          <t>ordered entry</t>
+        </is>
+      </c>
+      <c r="B14" s="76" t="inlineStr">
+        <is>
+          <t>the Moment Ordered time begins</t>
+        </is>
+      </c>
+      <c r="C14" s="76" t="inlineStr">
+        <is>
+          <t>"when the fight starts"</t>
+        </is>
+      </c>
+      <c r="D14" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED · PINNABLE</t>
+        </is>
+      </c>
+      <c r="E14" s="76" t="inlineStr">
+        <is>
+          <t>Not merely watchable.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="70" t="inlineStr">
-        <is>
-          <t>immediately</t>
-        </is>
-      </c>
-      <c r="B15" s="70" t="inlineStr">
-        <is>
-          <t>The current Moment</t>
-        </is>
-      </c>
-      <c r="C15" s="70" t="inlineStr">
-        <is>
-          <t>respond, interrupt</t>
-        </is>
-      </c>
-      <c r="D15" s="70" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E15" s="70" t="inlineStr"/>
+      <c r="A15" s="76" t="inlineStr">
+        <is>
+          <t>ordered exit</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>the Moment Ordered time ends</t>
+        </is>
+      </c>
+      <c r="C15" s="76" t="inlineStr">
+        <is>
+          <t>"until the fight is over"</t>
+        </is>
+      </c>
+      <c r="D15" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED · PINNABLE</t>
+        </is>
+      </c>
+      <c r="E15" s="76" t="inlineStr">
+        <is>
+          <t>Forcing this through a Listener would be perverse.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="70" t="inlineStr">
-        <is>
-          <t>entry to Ordered time</t>
-        </is>
-      </c>
-      <c r="B16" s="70" t="inlineStr"/>
-      <c r="C16" s="70" t="inlineStr">
-        <is>
-          <t>Listeners, Budget</t>
-        </is>
-      </c>
-      <c r="D16" s="70" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E16" s="70" t="inlineStr">
-        <is>
-          <t>WHAT causes entry is base Ruleset, not Substrate — three candidate rules were tried in Phase 0 and each failed on a real case.</t>
+      <c r="A16" s="76" t="inlineStr">
+        <is>
+          <t>(round parameter)</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>EVERY reference carries a round. Numbered from 1 at entry to Ordered time; no round 0; absent in Loose time.</t>
+        </is>
+      </c>
+      <c r="C16" s="76" t="inlineStr">
+        <is>
+          <t>all of them</t>
+        </is>
+      </c>
+      <c r="D16" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="E16" s="76" t="inlineStr">
+        <is>
+          <t>Authors write RELATIVE ("+3"); the Ledger stores ABSOLUTE. Safe because ROUNDS NEVER REORDER — turn order within a round does, which is why the Entity half stays symbolic.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="70" t="inlineStr">
-        <is>
-          <t>exit from Ordered time</t>
-        </is>
-      </c>
-      <c r="B17" s="70" t="inlineStr"/>
-      <c r="C17" s="70" t="inlineStr">
-        <is>
-          <t>Listeners, cleanup</t>
-        </is>
-      </c>
-      <c r="D17" s="70" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="E17" s="70" t="inlineStr"/>
+      <c r="A17" s="70" t="n"/>
+      <c r="B17" s="70" t="n"/>
+      <c r="C17" s="70" t="n"/>
+      <c r="D17" s="70" t="n"/>
+      <c r="E17" s="70" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="76" t="inlineStr">
+        <is>
+          <t>A MOMENT KIND SAYS *WHEN*. A LISTENER SAYS *WHETHER*. Never add a Moment kind to express a condition — the Moment list is a frozen coordinate system; the Listener condition set (L26) is the open one and extends forever.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="70" t="inlineStr">
-        <is>
-          <t>ARGUE EACH ONE AGAINST A REAL ABILITY. A Moment kind nobody can name an ability for is a Moment kind that should not be frozen.</t>
+      <c r="A19" s="70" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="71" t="inlineStr">
+        <is>
+          <t>CONSIDERED AND REJECTED</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="71" t="inlineStr">
-        <is>
-          <t>CONSIDERED AND REJECTED</t>
+      <c r="A21" s="77" t="inlineStr">
+        <is>
+          <t>start of MY turn / end of MY turn</t>
+        </is>
+      </c>
+      <c r="B21" s="72" t="inlineStr"/>
+      <c r="C21" s="72" t="inlineStr"/>
+      <c r="D21" s="72" t="inlineStr"/>
+      <c r="E21" s="72" t="inlineStr">
+        <is>
+          <t>COLLAPSED into turn start(E) / turn end(E) with E = self. Four frozen words became two.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="72" t="inlineStr">
         <is>
-          <t>downtime week / season / campaign turn</t>
-        </is>
-      </c>
-      <c r="B22" s="72" t="inlineStr"/>
+          <t>"activate on initiative 10"</t>
+        </is>
+      </c>
+      <c r="B22" s="72" t="inlineStr">
+        <is>
+          <t>a position in the round independent of who occupies it</t>
+        </is>
+      </c>
       <c r="C22" s="72" t="inlineStr"/>
-      <c r="D22" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="D22" s="72" t="inlineStr"/>
       <c r="E22" s="72" t="inlineStr">
         <is>
-          <t>REJECT: Components. A Component ADDS a coarser clock alongside; it never replaces the fine one.</t>
+          <t>COMPONENT — a finer clock. Only exists where turn structure is a COUNT not an ORDERING (Shadowrun passes, Feng Shui shots, Exalted ticks). Freezing "a round has numbered slots" fails the line: PF2e and 5e have no such thing.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="72" t="inlineStr">
         <is>
-          <t>"before the attack resolves"</t>
+          <t>"the next time somebody is attacked"</t>
         </is>
       </c>
       <c r="B23" s="72" t="inlineStr"/>
       <c r="C23" s="72" t="inlineStr"/>
-      <c r="D23" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="D23" s="72" t="inlineStr"/>
       <c r="E23" s="72" t="inlineStr">
         <is>
-          <t>ARGUE: this is what interrupt (L31) means, not a Moment kind. Do not encode it twice.</t>
+          <t>LISTENER — a Resolution Record exists this Moment with target = X, pinned to now.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="72" t="inlineStr">
         <is>
-          <t>tick</t>
+          <t>"when a person takes their reaction"</t>
         </is>
       </c>
       <c r="B24" s="72" t="inlineStr"/>
       <c r="C24" s="72" t="inlineStr"/>
-      <c r="D24" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="D24" s="72" t="inlineStr"/>
       <c r="E24" s="72" t="inlineStr">
         <is>
-          <t>NOT a Moment kind — the Tick is the STAMP on a Moment when it occurs.</t>
-        </is>
-      </c>
-    </row>
+          <t>LISTENER — doubloons spent this Moment by E with timing respond &gt; 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="72" t="inlineStr">
+        <is>
+          <t>"when a spell is cast that meets a condition"</t>
+        </is>
+      </c>
+      <c r="B25" s="72" t="inlineStr"/>
+      <c r="C25" s="72" t="inlineStr"/>
+      <c r="D25" s="72" t="inlineStr"/>
+      <c r="E25" s="72" t="inlineStr">
+        <is>
+          <t>LISTENER — a Resolution Record matching a shape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>downtime week / season / campaign turn</t>
+        </is>
+      </c>
+      <c r="B26" s="72" t="inlineStr"/>
+      <c r="C26" s="72" t="inlineStr"/>
+      <c r="D26" s="72" t="inlineStr"/>
+      <c r="E26" s="72" t="inlineStr">
+        <is>
+          <t>COMPONENT: adds a coarser clock alongside; never replaces the fine one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="72" t="inlineStr">
+        <is>
+          <t>duration ("for 3 rounds")</t>
+        </is>
+      </c>
+      <c r="B27" s="72" t="inlineStr"/>
+      <c r="C27" s="72" t="inlineStr"/>
+      <c r="D27" s="72" t="inlineStr"/>
+      <c r="E27" s="72" t="inlineStr">
+        <is>
+          <t>NOT a Moment kind — a pin to round end with the round parameter, or a State a Listener ends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="72" t="inlineStr">
+        <is>
+          <t>turn ownership (mine / not mine)</t>
+        </is>
+      </c>
+      <c r="B28" s="72" t="inlineStr"/>
+      <c r="C28" s="72" t="inlineStr"/>
+      <c r="D28" s="72" t="inlineStr"/>
+      <c r="E28" s="72" t="inlineStr">
+        <is>
+          <t>NOT a Moment kind — a PREDICATE on the current Moment. Substrate, but a different shelf. L31 respond and interrupt are defined in terms of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="72" t="inlineStr">
+        <is>
+          <t>tick</t>
+        </is>
+      </c>
+      <c r="B29" s="72" t="inlineStr"/>
+      <c r="C29" s="72" t="inlineStr"/>
+      <c r="D29" s="72" t="inlineStr"/>
+      <c r="E29" s="72" t="inlineStr">
+        <is>
+          <t>NOT a Moment kind — the STAMP on a Moment when it occurs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12835,8 +12948,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="20" customWidth="1" style="19" min="1" max="1"/>
     <col width="36" customWidth="1" style="19" min="2" max="2"/>
@@ -13175,7 +13288,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="70" t="inlineStr">
         <is>
@@ -13183,7 +13295,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="71" t="inlineStr">
         <is>
@@ -13236,22 +13347,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13264,7 +13359,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
     <col width="12" customWidth="1" style="19" min="2" max="2"/>
@@ -13701,7 +13796,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -14355,7 +14450,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="20" customWidth="1" style="19" min="1" max="1"/>
     <col width="24" customWidth="1" style="19" min="2" max="2"/>
@@ -15156,7 +15251,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" style="19" min="1" max="1"/>
     <col width="44" customWidth="1" style="19" min="2" max="2"/>
@@ -15519,7 +15614,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>
@@ -15909,7 +16004,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
     <col width="40" customWidth="1" style="18" min="2" max="2"/>

</xml_diff>

<commit_message>
L32: turn count added (nine kinds); L26 composition and firing discipline settled; authoring loop written up
</commit_message>
<xml_diff>
--- a/docs/substrate-lists.xlsx
+++ b/docs/substrate-lists.xlsx
@@ -7738,7 +7738,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -8297,7 +8296,6 @@
       </c>
       <c r="C32" s="24" t="n"/>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>
@@ -9467,7 +9465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" style="19" min="1" max="1"/>
@@ -9699,6 +9697,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="70" t="inlineStr">
         <is>
@@ -9706,6 +9705,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="71" t="inlineStr">
         <is>
@@ -9837,6 +9837,61 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="76" t="inlineStr">
+        <is>
+          <t>conditions compose</t>
+        </is>
+      </c>
+      <c r="B28" s="76" t="inlineStr">
+        <is>
+          <t>and · or · not, over the closed form set</t>
+        </is>
+      </c>
+      <c r="C28" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED Aug 2026</t>
+        </is>
+      </c>
+      <c r="D28" s="76" t="inlineStr">
+        <is>
+          <t>"not" is safe despite the open-world rule: that rule is about absent FIELDS, not unknown STATE, and the Fold has complete state at evaluation. Composition lets "a spell is cast that fulfils a condition" be ONE Listener rather than a family.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="76" t="inlineStr">
+        <is>
+          <t>firing discipline</t>
+        </is>
+      </c>
+      <c r="B29" s="76" t="inlineStr">
+        <is>
+          <t>a REQUIRED field: once | while. NO DEFAULT.</t>
+        </is>
+      </c>
+      <c r="C29" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED Aug 2026</t>
+        </is>
+      </c>
+      <c r="D29" s="76" t="inlineStr">
+        <is>
+          <t>"The next time somebody attacks" is once. "While you are bleeding" is while. No default because the two behave differently enough that a wrong guess is silent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12457,7 +12512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" style="19" min="1" max="1"/>
@@ -12495,6 +12550,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="67" t="inlineStr">
         <is>
@@ -12749,92 +12805,100 @@
     <row r="16">
       <c r="A16" s="76" t="inlineStr">
         <is>
+          <t>turn count (n)</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>the Moment at numeric position n in the order — OCCURRING WHETHER OR NOT AN ENTITY OCCUPIES IT</t>
+        </is>
+      </c>
+      <c r="C16" s="76" t="inlineStr">
+        <is>
+          <t>initiative-count systems</t>
+        </is>
+      </c>
+      <c r="D16" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="E16" s="76" t="inlineStr">
+        <is>
+          <t>Shadowrun passes, Feng Shui shots, Exalted 2e ticks, Fallout-style AP clocks. Substrate does NOT need the direction (countdowns run high-to-low, ordinals low-to-high; count 10 is count 10). Round parameter applies. When an Entity occupies n: turn count(n) fires FIRST, then turn start(E).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="76" t="inlineStr">
+        <is>
           <t>(round parameter)</t>
         </is>
       </c>
-      <c r="B16" s="76" t="inlineStr">
+      <c r="B17" s="76" t="inlineStr">
         <is>
           <t>EVERY reference carries a round. Numbered from 1 at entry to Ordered time; no round 0; absent in Loose time.</t>
         </is>
       </c>
-      <c r="C16" s="76" t="inlineStr">
+      <c r="C17" s="76" t="inlineStr">
         <is>
           <t>all of them</t>
         </is>
       </c>
-      <c r="D16" s="76" t="inlineStr">
+      <c r="D17" s="76" t="inlineStr">
         <is>
           <t>SETTLED</t>
         </is>
       </c>
-      <c r="E16" s="76" t="inlineStr">
+      <c r="E17" s="76" t="inlineStr">
         <is>
           <t>Authors write RELATIVE ("+3"); the Ledger stores ABSOLUTE. Safe because ROUNDS NEVER REORDER — turn order within a round does, which is why the Entity half stays symbolic.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="70" t="n"/>
-      <c r="B17" s="70" t="n"/>
-      <c r="C17" s="70" t="n"/>
-      <c r="D17" s="70" t="n"/>
-      <c r="E17" s="70" t="n"/>
-    </row>
     <row r="18">
-      <c r="A18" s="76" t="inlineStr">
+      <c r="A18" s="70" t="n"/>
+      <c r="B18" s="70" t="n"/>
+      <c r="C18" s="70" t="n"/>
+      <c r="D18" s="70" t="n"/>
+      <c r="E18" s="70" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="76" t="inlineStr">
         <is>
           <t>A MOMENT KIND SAYS *WHEN*. A LISTENER SAYS *WHETHER*. Never add a Moment kind to express a condition — the Moment list is a frozen coordinate system; the Listener condition set (L26) is the open one and extends forever.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="70" t="n"/>
-    </row>
     <row r="20">
-      <c r="A20" s="71" t="inlineStr">
+      <c r="A20" s="70" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="71" t="inlineStr">
         <is>
           <t>CONSIDERED AND REJECTED</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="77" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="77" t="inlineStr">
         <is>
           <t>start of MY turn / end of MY turn</t>
         </is>
       </c>
-      <c r="B21" s="72" t="inlineStr"/>
-      <c r="C21" s="72" t="inlineStr"/>
-      <c r="D21" s="72" t="inlineStr"/>
-      <c r="E21" s="72" t="inlineStr">
-        <is>
-          <t>COLLAPSED into turn start(E) / turn end(E) with E = self. Four frozen words became two.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="72" t="inlineStr">
-        <is>
-          <t>"activate on initiative 10"</t>
-        </is>
-      </c>
-      <c r="B22" s="72" t="inlineStr">
-        <is>
-          <t>a position in the round independent of who occupies it</t>
-        </is>
-      </c>
+      <c r="B22" s="72" t="inlineStr"/>
       <c r="C22" s="72" t="inlineStr"/>
       <c r="D22" s="72" t="inlineStr"/>
       <c r="E22" s="72" t="inlineStr">
         <is>
-          <t>COMPONENT — a finer clock. Only exists where turn structure is a COUNT not an ORDERING (Shadowrun passes, Feng Shui shots, Exalted ticks). Freezing "a round has numbered slots" fails the line: PF2e and 5e have no such thing.</t>
+          <t>COLLAPSED into turn start(E) / turn end(E) with E = self. Four frozen words became two.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="72" t="inlineStr">
         <is>
-          <t>"the next time somebody is attacked"</t>
+          <t>"activate on initiative 10"</t>
         </is>
       </c>
       <c r="B23" s="72" t="inlineStr"/>
@@ -12842,14 +12906,14 @@
       <c r="D23" s="72" t="inlineStr"/>
       <c r="E23" s="72" t="inlineStr">
         <is>
-          <t>LISTENER — a Resolution Record exists this Moment with target = X, pinned to now.</t>
+          <t>NO LONGER REJECTED — became turn count (n), Aug 2026. The earlier "it is a Component clock" answer was WRONG: a Component CANNOT publish a Moment kind. Sending it to a Component would have made a whole family of published initiative systems inexpressible until a Substrate change.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="72" t="inlineStr">
         <is>
-          <t>"when a person takes their reaction"</t>
+          <t>"the next time somebody is attacked"</t>
         </is>
       </c>
       <c r="B24" s="72" t="inlineStr"/>
@@ -12857,14 +12921,14 @@
       <c r="D24" s="72" t="inlineStr"/>
       <c r="E24" s="72" t="inlineStr">
         <is>
-          <t>LISTENER — doubloons spent this Moment by E with timing respond &gt; 0.</t>
+          <t>LISTENER — a Resolution Record exists this Moment with target = X, pinned to now.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="72" t="inlineStr">
         <is>
-          <t>"when a spell is cast that meets a condition"</t>
+          <t>"when a person takes their reaction"</t>
         </is>
       </c>
       <c r="B25" s="72" t="inlineStr"/>
@@ -12872,14 +12936,14 @@
       <c r="D25" s="72" t="inlineStr"/>
       <c r="E25" s="72" t="inlineStr">
         <is>
-          <t>LISTENER — a Resolution Record matching a shape.</t>
+          <t>LISTENER — doubloons spent this Moment by E with timing respond &gt; 0.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="72" t="inlineStr">
         <is>
-          <t>downtime week / season / campaign turn</t>
+          <t>"when a spell is cast that meets a condition"</t>
         </is>
       </c>
       <c r="B26" s="72" t="inlineStr"/>
@@ -12887,14 +12951,14 @@
       <c r="D26" s="72" t="inlineStr"/>
       <c r="E26" s="72" t="inlineStr">
         <is>
-          <t>COMPONENT: adds a coarser clock alongside; never replaces the fine one.</t>
+          <t>LISTENER — a Resolution Record matching a shape.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="72" t="inlineStr">
         <is>
-          <t>duration ("for 3 rounds")</t>
+          <t>downtime week / season / campaign turn</t>
         </is>
       </c>
       <c r="B27" s="72" t="inlineStr"/>
@@ -12902,14 +12966,14 @@
       <c r="D27" s="72" t="inlineStr"/>
       <c r="E27" s="72" t="inlineStr">
         <is>
-          <t>NOT a Moment kind — a pin to round end with the round parameter, or a State a Listener ends.</t>
+          <t>COMPONENT: adds a coarser clock alongside; never replaces the fine one.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="72" t="inlineStr">
         <is>
-          <t>turn ownership (mine / not mine)</t>
+          <t>duration ("for 3 rounds")</t>
         </is>
       </c>
       <c r="B28" s="72" t="inlineStr"/>
@@ -12917,14 +12981,14 @@
       <c r="D28" s="72" t="inlineStr"/>
       <c r="E28" s="72" t="inlineStr">
         <is>
-          <t>NOT a Moment kind — a PREDICATE on the current Moment. Substrate, but a different shelf. L31 respond and interrupt are defined in terms of it.</t>
+          <t>NOT a Moment kind — a pin to round end with the round parameter, or a State a Listener ends.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="72" t="inlineStr">
         <is>
-          <t>tick</t>
+          <t>turn ownership (mine / not mine)</t>
         </is>
       </c>
       <c r="B29" s="72" t="inlineStr"/>
@@ -12932,11 +12996,54 @@
       <c r="D29" s="72" t="inlineStr"/>
       <c r="E29" s="72" t="inlineStr">
         <is>
+          <t>NOT a Moment kind — a PREDICATE on the current Moment. Substrate, but a different shelf. L31 respond and interrupt are defined in terms of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="72" t="inlineStr">
+        <is>
+          <t>tick</t>
+        </is>
+      </c>
+      <c r="B30" s="72" t="inlineStr"/>
+      <c r="C30" s="72" t="inlineStr"/>
+      <c r="D30" s="72" t="inlineStr"/>
+      <c r="E30" s="72" t="inlineStr">
+        <is>
           <t>NOT a Moment kind — the STAMP on a Moment when it occurs.</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
L1/L2/L3 settled: nine Categories that compose, nine universal fields, links replaces part_of, absence is immunity
</commit_message>
<xml_diff>
--- a/docs/substrate-lists.xlsx
+++ b/docs/substrate-lists.xlsx
@@ -35,6 +35,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L30 Instrumentation surfaces" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L31 Timings" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L32 Moment kinds" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L1b Link relations" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -7765,61 +7766,61 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="19">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="73" t="inlineStr">
         <is>
           <t>L1 · Categories</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>PENDING · BLOCKING</t>
-        </is>
-      </c>
-      <c r="C5" s="26">
+      <c r="B5" s="74" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="73">
         <f>COUNTA('L1 Categories'!A8:A47)</f>
         <v/>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="73">
         <f>IF(C5&gt;0,"started","not started")</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="19">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="73" t="inlineStr">
         <is>
           <t>L2 · Universal Attributes</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>PENDING · BLOCKING</t>
-        </is>
-      </c>
-      <c r="C6" s="26">
+      <c r="B6" s="74" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="73">
         <f>COUNTA('L2 Universal Attributes'!A8:A47)</f>
         <v/>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="73">
         <f>IF(C6&gt;0,"started","not started")</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="19">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="73" t="inlineStr">
         <is>
           <t>L3 · Category Attributes</t>
         </is>
       </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>PENDING · BLOCKING</t>
-        </is>
-      </c>
-      <c r="C7" s="26">
+      <c r="B7" s="74" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="73">
         <f>COUNTA('L3 Category Attributes'!A8:A47)</f>
         <v/>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="73">
         <f>IF(C7&gt;0,"started","not started")</f>
         <v/>
       </c>
@@ -12109,7 +12110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="19" min="1" max="1"/>
@@ -12475,23 +12476,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13010,20 +12994,318 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="19" min="1" max="1"/>
+    <col width="14" customWidth="1" style="19" min="2" max="2"/>
+    <col width="30" customWidth="1" style="19" min="3" max="3"/>
+    <col width="28" customWidth="1" style="19" min="4" max="4"/>
+    <col width="80" customWidth="1" style="19" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="63" t="inlineStr">
+        <is>
+          <t>Links · the relations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="64" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026 · five</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="65" t="inlineStr">
+        <is>
+          <t>A link is a (relation, target) pair stored on the HOLDER and named from its point of view. A relation is an ID with declared traits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>A NEW RELATION IS A NEW ID, NOT A NEW FIELD — additive by construction. Flecs and Bevy each shipped a bespoke parent/child field, each hit a second structural relation, and each had to rebuild it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="67" t="inlineStr">
+        <is>
+          <t>Relation</t>
+        </is>
+      </c>
+      <c r="B6" s="67" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C6" s="67" t="inlineStr">
+        <is>
+          <t>Traits</t>
+        </is>
+      </c>
+      <c r="D6" s="67" t="inlineStr">
+        <is>
+          <t>Means</t>
+        </is>
+      </c>
+      <c r="E6" s="67" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="68" t="inlineStr">
+        <is>
+          <t>is_a</t>
+        </is>
+      </c>
+      <c r="B7" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C7" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="68" t="inlineStr">
+        <is>
+          <t>inheritance</t>
+        </is>
+      </c>
+      <c r="E7" s="68" t="inlineStr">
+        <is>
+          <t>REJECTED — a live inheritance link means editing a template retroactively changes folded history. Templates COPY at creation.</t>
+        </is>
+      </c>
+      <c r="F7" s="69" t="inlineStr">
+        <is>
+          <t>← example, not data</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>part_of</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
+        <is>
+          <t>SUBSTRATE</t>
+        </is>
+      </c>
+      <c r="C8" s="76" t="inlineStr">
+        <is>
+          <t>exclusive · acyclic · CASCADES</t>
+        </is>
+      </c>
+      <c r="D8" s="76" t="inlineStr">
+        <is>
+          <t>physical composition</t>
+        </is>
+      </c>
+      <c r="E8" s="76" t="inlineStr">
+        <is>
+          <t>THE ONLY relation the Substrate itself reads, because destruction cascade and Scale legality depend on it. A door is part of a ship. Cascade is a FOLD RULE, not a Verb side-effect — otherwise rule 8a is violated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="76" t="inlineStr">
+        <is>
+          <t>member_of</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>Ruleset</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>many · no cascade</t>
+        </is>
+      </c>
+      <c r="D9" s="76" t="inlineStr">
+        <is>
+          <t>belonging to a Group</t>
+        </is>
+      </c>
+      <c r="E9" s="76" t="inlineStr">
+        <is>
+          <t>A person is NOT part of a guild. Kira can be member_of the Ashfall Company AND member_of Bren's party.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="76" t="inlineStr">
+        <is>
+          <t>carried_by</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>Ruleset</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>exclusive · no cascade</t>
+        </is>
+      </c>
+      <c r="D10" s="76" t="inlineStr">
+        <is>
+          <t>held or carried</t>
+        </is>
+      </c>
+      <c r="E10" s="76" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="76" t="inlineStr">
+        <is>
+          <t>controlled_by</t>
+        </is>
+      </c>
+      <c r="B11" s="76" t="inlineStr">
+        <is>
+          <t>Ruleset</t>
+        </is>
+      </c>
+      <c r="C11" s="76" t="inlineStr">
+        <is>
+          <t>exclusive · no cascade</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr">
+        <is>
+          <t>who decides for it</t>
+        </is>
+      </c>
+      <c r="E11" s="76" t="inlineStr">
+        <is>
+          <t>THIS is how a player character differs from a creature. Not a schema difference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>owned_by</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>Ruleset</t>
+        </is>
+      </c>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>exclusive · no cascade</t>
+        </is>
+      </c>
+      <c r="D12" s="76" t="inlineStr">
+        <is>
+          <t>property</t>
+        </is>
+      </c>
+      <c r="E12" s="76" t="inlineStr">
+        <is>
+          <t>Distinct from carried_by — you can carry what you do not own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="76" t="inlineStr">
+        <is>
+          <t>CONVENTION: named from the holder's point of view and stored on the holder. Always "this thing -&gt; that thing", never a list on the far side. That is what makes every structural change a SINGLE-TARGET Verb, which the Verb shape requires.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="71" t="inlineStr">
+        <is>
+          <t>CONSIDERED AND REJECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="72" t="inlineStr">
+        <is>
+          <t>inside / location</t>
+        </is>
+      </c>
+      <c r="B17" s="72" t="inlineStr"/>
+      <c r="C17" s="72" t="inlineStr"/>
+      <c r="D17" s="72" t="inlineStr"/>
+      <c r="E17" s="72" t="inlineStr">
+        <is>
+          <t>NOT a relation — the PLACE SOCKET's Facet. Only the occupant can say what a position means.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="72" t="inlineStr">
+        <is>
+          <t>sworn_to · knows · docked_to</t>
+        </is>
+      </c>
+      <c r="B18" s="72" t="inlineStr"/>
+      <c r="C18" s="72" t="inlineStr"/>
+      <c r="D18" s="72" t="inlineStr"/>
+      <c r="E18" s="72" t="inlineStr">
+        <is>
+          <t>SETTING-LEVEL. Let the six Settings publish what they actually need; a new relation is an ID, so it costs nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="72" t="inlineStr">
+        <is>
+          <t>a bidirectional pair (parts + part_of)</t>
+        </is>
+      </c>
+      <c r="B19" s="72" t="inlineStr"/>
+      <c r="C19" s="72" t="inlineStr"/>
+      <c r="D19" s="72" t="inlineStr"/>
+      <c r="E19" s="72" t="inlineStr">
+        <is>
+          <t>REJECTED — denormalisation, and denormalisation desyncs. The Fold derives the inverse. Nobody surveyed stores only the downward list.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" style="19" min="1" max="1"/>
-    <col width="36" customWidth="1" style="19" min="2" max="2"/>
-    <col width="42" customWidth="1" style="19" min="3" max="3"/>
-    <col width="16" customWidth="1" style="19" min="4" max="4"/>
-    <col width="74" customWidth="1" style="19" min="5" max="5"/>
+    <col width="16" customWidth="1" style="19" min="1" max="1"/>
+    <col width="14" customWidth="1" style="19" min="2" max="2"/>
+    <col width="34" customWidth="1" style="19" min="3" max="3"/>
+    <col width="46" customWidth="1" style="19" min="4" max="4"/>
+    <col width="72" customWidth="1" style="19" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13036,21 +13318,21 @@
     <row r="2">
       <c r="A2" s="64" t="inlineStr">
         <is>
-          <t>PENDING · BLOCKING · research-seeded Aug 2026</t>
+          <t>SETTLED · Aug 2026 · nine</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="65" t="inlineStr">
         <is>
-          <t>The labels an Entity may carry saying what kind of thing it is. An Entity may carry several at once; each brings its own Attributes.</t>
+          <t>A named bundle of the data a thing needs in order to PARTICIPATE. Not a taxonomy, not a type hierarchy, not a claim about what something is.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="66" t="inlineStr">
         <is>
-          <t>A CATEGORY THAT BRINGS NO ATTRIBUTES IS A TAG. The boundary the whole field draws: exactly one value true and values partition → Category. Any number true at once, minted forever → Tag. One true within an axis, started and ended by a Verb → State.</t>
+          <t>CATEGORIES COMPOSE. An Entity carries as many as apply; the result is the UNION of their bundles. A sentient sword is Item + Creature. An elemental plague is Phenomenon + Creature.</t>
         </is>
       </c>
     </row>
@@ -13062,17 +13344,17 @@
       </c>
       <c r="B6" s="67" t="inlineStr">
         <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C6" s="67" t="inlineStr">
+        <is>
           <t>What it is</t>
         </is>
       </c>
-      <c r="C6" s="67" t="inlineStr">
-        <is>
-          <t>Attributes it adds</t>
-        </is>
-      </c>
       <c r="D6" s="67" t="inlineStr">
         <is>
-          <t>Can it ATTEMPT?</t>
+          <t>Brings (see L3)</t>
         </is>
       </c>
       <c r="E6" s="67" t="inlineStr">
@@ -13084,27 +13366,27 @@
     <row r="7">
       <c r="A7" s="68" t="inlineStr">
         <is>
-          <t>haunted</t>
+          <t>Tangible</t>
         </is>
       </c>
       <c r="B7" s="68" t="inlineStr">
         <is>
-          <t>a place with a ghost</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C7" s="68" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>things you can touch</t>
         </is>
       </c>
       <c r="D7" s="68" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>scale, place, mass, hardness</t>
         </is>
       </c>
       <c r="E7" s="68" t="inlineStr">
         <is>
-          <t>NOT a Category — a Tag. It adds nothing to the sheet.</t>
+          <t>REJECTED — see below. Location and scale do not depend on matter.</t>
         </is>
       </c>
       <c r="F7" s="69" t="inlineStr">
@@ -13114,252 +13396,252 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="70" t="inlineStr">
-        <is>
-          <t>Being</t>
-        </is>
-      </c>
-      <c r="B8" s="70" t="inlineStr">
-        <is>
-          <t>Anything with a body and agency</t>
-        </is>
-      </c>
-      <c r="C8" s="70" t="inlineStr">
-        <is>
-          <t>the attempt Dimensions, the physical/mental Dimensions</t>
-        </is>
-      </c>
-      <c r="D8" s="70" t="inlineStr">
-        <is>
-          <t>yes — nothing gates it</t>
-        </is>
-      </c>
-      <c r="E8" s="70" t="inlineStr">
-        <is>
-          <t>The only Category nobody argues about.</t>
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
+        <is>
+          <t>SUBSTRATE</t>
+        </is>
+      </c>
+      <c r="C8" s="76" t="inlineStr">
+        <is>
+          <t>a pending push</t>
+        </is>
+      </c>
+      <c r="D8" s="76" t="inlineStr">
+        <is>
+          <t>direction · magnitude · target (exactly one) · pin · layer · class</t>
+        </is>
+      </c>
+      <c r="E8" s="76" t="inlineStr">
+        <is>
+          <t>Enforced shape. A pending vector is an Entity and is targetable.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="70" t="inlineStr">
-        <is>
-          <t>Object</t>
-        </is>
-      </c>
-      <c r="B9" s="70" t="inlineStr">
-        <is>
-          <t>A made or found thing</t>
-        </is>
-      </c>
-      <c r="C9" s="70" t="inlineStr">
-        <is>
-          <t>physical Dimensions, Mass/Bulk/Hardness</t>
-        </is>
-      </c>
-      <c r="D9" s="70" t="inlineStr">
-        <is>
-          <t>yes — nothing gates it</t>
-        </is>
-      </c>
-      <c r="E9" s="70" t="inlineStr">
-        <is>
-          <t>"Can be targeted" without "can attempt" is the test that separates L2 from L3.</t>
+      <c r="A9" s="76" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>SUBSTRATE</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>a pending decision</t>
+        </is>
+      </c>
+      <c r="D9" s="76" t="inlineStr">
+        <is>
+          <t>decider · moment · default · subject</t>
+        </is>
+      </c>
+      <c r="E9" s="76" t="inlineStr">
+        <is>
+          <t>Rule 21: a human Decider always carries a Moment and a default.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="70" t="inlineStr">
+      <c r="A10" s="76" t="inlineStr">
+        <is>
+          <t>Relationship</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>SUBSTRATE</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>a stance between participants</t>
+        </is>
+      </c>
+      <c r="D10" s="76" t="inlineStr">
+        <is>
+          <t>one Connection per participant, stored independently</t>
+        </is>
+      </c>
+      <c r="E10" s="76" t="inlineStr">
+        <is>
+          <t>NEVER an edge. 4 of 5 surveyed systems agree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="76" t="inlineStr">
+        <is>
+          <t>Creature</t>
+        </is>
+      </c>
+      <c r="B11" s="76" t="inlineStr">
+        <is>
+          <t>Ruleset</t>
+        </is>
+      </c>
+      <c r="C11" s="76" t="inlineStr">
+        <is>
+          <t>ANYTHING THAT ACTS — rolls, is played, places vectors</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr">
+        <is>
+          <t>attempt Capacities · vitality · posture/awareness/consciousness · Specialisations</t>
+        </is>
+      </c>
+      <c r="E11" s="76" t="inlineStr">
+        <is>
+          <t>NOTHING ABOUT BIOLOGY. A haunted anchor, a sentient storm and a scheming guild are all Creatures, because all three do things.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>Ruleset</t>
+        </is>
+      </c>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>made or found; carried, used, broken</t>
+        </is>
+      </c>
+      <c r="D12" s="76" t="inlineStr">
+        <is>
+          <t>integrity · mass and bulk Tags · Guards</t>
+        </is>
+      </c>
+      <c r="E12" s="76" t="inlineStr">
+        <is>
+          <t>No mental State axes — which IS why a fear vector against a vase lands on nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="76" t="inlineStr">
         <is>
           <t>Place</t>
         </is>
       </c>
-      <c r="B10" s="70" t="inlineStr">
-        <is>
-          <t>A location that can contain things</t>
-        </is>
-      </c>
-      <c r="C10" s="70" t="inlineStr">
-        <is>
-          <t>containment, Scale</t>
-        </is>
-      </c>
-      <c r="D10" s="70" t="inlineStr">
-        <is>
-          <t>yes — nothing gates it</t>
-        </is>
-      </c>
-      <c r="E10" s="70" t="inlineStr">
-        <is>
-          <t>Overlaps the Place Socket. Argue whether this is a Category at all or purely Socket business.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="70" t="inlineStr">
+      <c r="B13" s="76" t="inlineStr">
+        <is>
+          <t>Ruleset</t>
+        </is>
+      </c>
+      <c r="C13" s="76" t="inlineStr">
+        <is>
+          <t>somewhere things are</t>
+        </is>
+      </c>
+      <c r="D13" s="76" t="inlineStr">
+        <is>
+          <t>extent and containment, per the Place Socket</t>
+        </is>
+      </c>
+      <c r="E13" s="76" t="inlineStr">
+        <is>
+          <t>Contents defined by the Socket occupant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="76" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="B11" s="70" t="inlineStr">
-        <is>
-          <t>A faction, crew, guild, household</t>
-        </is>
-      </c>
-      <c r="C11" s="70" t="inlineStr">
-        <is>
-          <t>social Dimensions, standing</t>
-        </is>
-      </c>
-      <c r="D11" s="70" t="inlineStr">
-        <is>
-          <t>yes — nothing gates it</t>
-        </is>
-      </c>
-      <c r="E11" s="70" t="inlineStr">
-        <is>
-          <t>Reign's companies act like characters. Star Trek Adventures' ships do NOT act — they assist. See notes below.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="70" t="inlineStr">
-        <is>
-          <t>Relationship</t>
-        </is>
-      </c>
-      <c r="B12" s="70" t="inlineStr">
-        <is>
-          <t>A Category of Entity holding one CONNECTION per participant</t>
-        </is>
-      </c>
-      <c r="C12" s="70" t="inlineStr">
-        <is>
-          <t>one stance per participant, stored independently</t>
-        </is>
-      </c>
-      <c r="D12" s="70" t="inlineStr">
-        <is>
-          <t>yes — nothing gates it</t>
-        </is>
-      </c>
-      <c r="E12" s="70" t="inlineStr">
-        <is>
-          <t>NEVER an edge. 4 of 5 surveyed systems agree (Exalted Intimacies, DG Bonds, Cortex relationship dice, Monsterhearts strings). Blades faction status is an edge, and Blades' faction game is the part most often houseruled.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="70" t="inlineStr">
-        <is>
-          <t>Knowledge</t>
-        </is>
-      </c>
-      <c r="B13" s="70" t="inlineStr">
-        <is>
-          <t>A rumour, a secret, a piece of lore</t>
-        </is>
-      </c>
-      <c r="C13" s="70" t="inlineStr">
-        <is>
-          <t>provenance, spread</t>
-        </is>
-      </c>
-      <c r="D13" s="70" t="inlineStr">
-        <is>
-          <t>yes — nothing gates it</t>
-        </is>
-      </c>
-      <c r="E13" s="70" t="inlineStr">
-        <is>
-          <t>The hardest test case for L2 — a rumour has almost no attributes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="70" t="inlineStr">
+      <c r="B14" s="76" t="inlineStr">
+        <is>
+          <t>Ruleset</t>
+        </is>
+      </c>
+      <c r="C14" s="76" t="inlineStr">
+        <is>
+          <t>a party, crew, faction, guild</t>
+        </is>
+      </c>
+      <c r="D14" s="76" t="inlineStr">
+        <is>
+          <t>membership · standing · group Resources</t>
+        </is>
+      </c>
+      <c r="E14" s="76" t="inlineStr">
+        <is>
+          <t>Add Creature if it acts. Membership is member_of, NOT part_of.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="76" t="inlineStr">
+        <is>
+          <t>Notion</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>Ruleset</t>
+        </is>
+      </c>
+      <c r="C15" s="76" t="inlineStr">
+        <is>
+          <t>a rumour, secret, law, debt</t>
+        </is>
+      </c>
+      <c r="D15" s="76" t="inlineStr">
+        <is>
+          <t>provenance · spread · credibility</t>
+        </is>
+      </c>
+      <c r="E15" s="76" t="inlineStr">
+        <is>
+          <t>NO location, NO harm pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="76" t="inlineStr">
         <is>
           <t>Phenomenon</t>
         </is>
       </c>
-      <c r="B14" s="70" t="inlineStr">
-        <is>
-          <t>A storm, a fire, a plague</t>
-        </is>
-      </c>
-      <c r="C14" s="70" t="inlineStr">
-        <is>
-          <t>physical Dimensions, Scale</t>
-        </is>
-      </c>
-      <c r="D14" s="70" t="inlineStr">
-        <is>
-          <t>yes — nothing gates it</t>
-        </is>
-      </c>
-      <c r="E14" s="70" t="inlineStr">
-        <is>
-          <t>ATTACK THIS ONE FIRST — it may just be an Object with Tags.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="70" t="inlineStr">
-        <is>
-          <t>Proposal</t>
-        </is>
-      </c>
-      <c r="B15" s="70" t="inlineStr">
-        <is>
-          <t>A pending decision awaiting a Decider</t>
-        </is>
-      </c>
-      <c r="C15" s="70" t="inlineStr">
-        <is>
-          <t>decider, Moment, default</t>
-        </is>
-      </c>
-      <c r="D15" s="70" t="inlineStr">
-        <is>
-          <t>yes — nothing gates it</t>
-        </is>
-      </c>
-      <c r="E15" s="70" t="inlineStr">
-        <is>
-          <t>Ours, not the field's. Rule 21: a human Decider always carries a Moment and a default.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="70" t="inlineStr">
-        <is>
-          <t>Vector</t>
-        </is>
-      </c>
-      <c r="B16" s="70" t="inlineStr">
-        <is>
-          <t>A pending push not yet resolved</t>
-        </is>
-      </c>
-      <c r="C16" s="70" t="inlineStr">
-        <is>
-          <t>direction, magnitude, pin, layer</t>
-        </is>
-      </c>
-      <c r="D16" s="70" t="inlineStr">
-        <is>
-          <t>yes — nothing gates it</t>
-        </is>
-      </c>
-      <c r="E16" s="70" t="inlineStr">
-        <is>
-          <t>Ours. Already an Entity by the dictionary.</t>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>Ruleset</t>
+        </is>
+      </c>
+      <c r="C16" s="76" t="inlineStr">
+        <is>
+          <t>a fire, storm, plague, curse</t>
+        </is>
+      </c>
+      <c r="D16" s="76" t="inlineStr">
+        <is>
+          <t>a standing vector · intensity · a fuel-like Resource</t>
+        </is>
+      </c>
+      <c r="E16" s="76" t="inlineStr">
+        <is>
+          <t>Works because standing vectors already exist. Add Creature if it acts.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="70" t="inlineStr">
-        <is>
-          <t>SETTLED Aug 2026: ANYTHING MAY ATTEMPT. No Category gates it. An Entity with no points in any attempt Dimension simply cannot attempt — 'absent is not zero' already said so, and adding a gate would enforce for free what the open-world reading enforces anyway. Star Trek Adventures' stance (the ship ASSISTS, it never rolls) stays available as CONTENT: a Setting that wants it simply gives ships no attempt Dimensions.</t>
+      <c r="A18" s="76" t="inlineStr">
+        <is>
+          <t>PC AND NPC ARE NOT CATEGORIES. Same fields, same rules, same sheet. The difference is a controlled_by link and a Decider. A character's numbers come from a creation process; a bestiary entry's are typed in. Identical schema, two authoring paths.</t>
         </is>
       </c>
     </row>
@@ -13373,7 +13655,7 @@
     <row r="21">
       <c r="A21" s="72" t="inlineStr">
         <is>
-          <t>Ship / Vehicle</t>
+          <t>Tangible</t>
         </is>
       </c>
       <c r="B21" s="72" t="inlineStr"/>
@@ -13381,14 +13663,14 @@
       <c r="D21" s="72" t="inlineStr"/>
       <c r="E21" s="72" t="inlineStr">
         <is>
-          <t>ARGUE: is this a Category, or an Object with a Group aboard? Traveller, Lancer and Scum &amp; Villainy all give ships their own sheet; STA gives them the SAME six attributes as characters, deliberately.</t>
+          <t>REJECTED. (1) Payload is wrong — BFO sites (a hold, a cockpit, a room) are IMMATERIAL and FULLY LOCATED; Blades factions have Tier and Turf. (2) BFO defers hurricanes/fires/flames to "the next version" and our Substrate is never versioned. (3) schema.org Intangible is the same shape and its maintainer's own bug closed unresolved. (4) OntoClean: a property things gain and lose must not be a backbone class — a ghost that materialises. NOW A TAG.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="72" t="inlineStr">
         <is>
-          <t>Character / NPC</t>
+          <t>Object</t>
         </is>
       </c>
       <c r="B22" s="72" t="inlineStr"/>
@@ -13396,14 +13678,14 @@
       <c r="D22" s="72" t="inlineStr"/>
       <c r="E22" s="72" t="inlineStr">
         <is>
-          <t>REJECT as separate Categories — both are Being. The distinction is a Lens concern.</t>
+          <t>REJECTED — brings nothing. An Entity with no Category is a thing in the world.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="72" t="inlineStr">
         <is>
-          <t>Item / Weapon / Armour</t>
+          <t>Character / NPC</t>
         </is>
       </c>
       <c r="B23" s="72" t="inlineStr"/>
@@ -13411,7 +13693,22 @@
       <c r="D23" s="72" t="inlineStr"/>
       <c r="E23" s="72" t="inlineStr">
         <is>
-          <t>REJECT: all Object. The differences are Tags and Facets.</t>
+          <t>REJECTED as separate from Creature. Who decides is a link, not a schema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="72" t="inlineStr">
+        <is>
+          <t>Being</t>
+        </is>
+      </c>
+      <c r="B24" s="72" t="inlineStr"/>
+      <c r="C24" s="72" t="inlineStr"/>
+      <c r="D24" s="72" t="inlineStr"/>
+      <c r="E24" s="72" t="inlineStr">
+        <is>
+          <t>RENAMED to Creature, and redefined as CAN ACT rather than IS ALIVE.</t>
         </is>
       </c>
     </row>
@@ -13426,15 +13723,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" style="19" min="1" max="1"/>
-    <col width="12" customWidth="1" style="19" min="2" max="2"/>
-    <col width="12" customWidth="1" style="19" min="3" max="3"/>
-    <col width="12" customWidth="1" style="19" min="4" max="4"/>
-    <col width="12" customWidth="1" style="19" min="5" max="5"/>
-    <col width="72" customWidth="1" style="19" min="6" max="6"/>
+    <col width="20" customWidth="1" style="19" min="1" max="1"/>
+    <col width="14" customWidth="1" style="19" min="2" max="2"/>
+    <col width="42" customWidth="1" style="19" min="3" max="3"/>
+    <col width="86" customWidth="1" style="19" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13447,53 +13742,43 @@
     <row r="2">
       <c r="A2" s="64" t="inlineStr">
         <is>
-          <t>PENDING · BLOCKING · research-seeded Aug 2026</t>
+          <t>SETTLED · Aug 2026 · nine</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="65" t="inlineStr">
         <is>
-          <t>What EVERY Entity has. Test each candidate against a rumour, a lock, a faction and a storm. If any of those does not need it, it is a Category Attribute and belongs in L3.</t>
+          <t>What EVERY Entity has, no exceptions. Six structural fields plus one slot per Noun kind.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="66" t="inlineStr">
         <is>
-          <t>L2 SHOULD BE BRUTALLY SHORT — four or five entries. The shortness IS the evidence the model is not a person schema in a costume. If it grows, L29 needs redoing.</t>
+          <t>THE NOUN SLOTS CANNOT LIVE IN FACETS. Rule 1 forbids reading another Component's Facets, but a Listener watching a State, a Guard reading a Resource and a Threshold reading a Capacity all cross Component lines BY DESIGN.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="67" t="inlineStr">
         <is>
-          <t>Candidate</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B6" s="67" t="inlineStr">
         <is>
-          <t>rumour</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="C6" s="67" t="inlineStr">
         <is>
-          <t>lock</t>
+          <t>What it holds</t>
         </is>
       </c>
       <c r="D6" s="67" t="inlineStr">
         <is>
-          <t>faction</t>
-        </is>
-      </c>
-      <c r="E6" s="67" t="inlineStr">
-        <is>
-          <t>storm</t>
-        </is>
-      </c>
-      <c r="F6" s="67" t="inlineStr">
-        <is>
-          <t>Verdict and notes</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -13503,352 +13788,344 @@
           <t>hit points</t>
         </is>
       </c>
-      <c r="B7" s="68" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="B7" s="68" t="inlineStr"/>
       <c r="C7" s="68" t="inlineStr">
         <is>
-          <t>maybe</t>
+          <t>a number</t>
         </is>
       </c>
       <c r="D7" s="68" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="E7" s="68" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F7" s="68" t="inlineStr">
-        <is>
           <t>NOT universal, and not even shipped — the Substrate ships no Resources.</t>
         </is>
       </c>
-      <c r="G7" s="69" t="inlineStr">
+      <c r="E7" s="69" t="inlineStr">
         <is>
           <t>← example, not data</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="70" t="inlineStr">
-        <is>
-          <t>identity (permanent ID)</t>
-        </is>
-      </c>
-      <c r="B8" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="C8" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D8" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E8" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F8" s="70" t="inlineStr">
-        <is>
-          <t>UNIVERSAL. Numeric, permanent, never reused.</t>
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="C8" s="76" t="inlineStr">
+        <is>
+          <t>permanent numeric, never reused</t>
+        </is>
+      </c>
+      <c r="D8" s="76" t="inlineStr">
+        <is>
+          <t>Derived STRUCTURALLY from the creating Record, so two folds of one Ledger allocate identically. A counter would drift.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="70" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B9" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="C9" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D9" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E9" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F9" s="70" t="inlineStr">
-        <is>
-          <t>UNIVERSAL. Multi-select.</t>
+      <c r="A9" s="76" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>zero or more</t>
+        </is>
+      </c>
+      <c r="D9" s="76" t="inlineStr">
+        <is>
+          <t>Composes — the union of the bundles.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="70" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B10" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="C10" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D10" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E10" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F10" s="70" t="inlineStr">
-        <is>
-          <t>UNIVERSAL. Open, optional magnitude.</t>
+      <c r="A10" s="76" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>zero or more, optional magnitude</t>
+        </is>
+      </c>
+      <c r="D10" s="76" t="inlineStr">
+        <is>
+          <t>Open, Component-extensible forever, never implies another Tag. Doubles as the Tag Noun slot.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="70" t="inlineStr">
-        <is>
-          <t>Scale</t>
-        </is>
-      </c>
-      <c r="B11" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="C11" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D11" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E11" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F11" s="70" t="inlineStr">
-        <is>
-          <t>UNIVERSAL — and Scale belongs to PARTS as well as wholes. A Scale-4 ship has Scale-1 doors.</t>
+      <c r="A11" s="76" t="inlineStr">
+        <is>
+          <t>links</t>
+        </is>
+      </c>
+      <c r="B11" s="76" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="C11" s="76" t="inlineStr">
+        <is>
+          <t>zero or more (relation, target) pairs</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr">
+        <is>
+          <t>REPLACED a hard-coded part_of. A relation is an ID with declared traits, so a new one is a new ID not a new field.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="70" t="inlineStr">
-        <is>
-          <t>Facets</t>
-        </is>
-      </c>
-      <c r="B12" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="C12" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D12" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E12" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F12" s="70" t="inlineStr">
-        <is>
-          <t>UNIVERSAL, but it is structure rather than an attribute. Argue whether it belongs on this list at all.</t>
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>scale</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>optional integer</t>
+        </is>
+      </c>
+      <c r="D12" s="76" t="inlineStr">
+        <is>
+          <t>SUBSTRATE, because R-750 and parts legality read it and rule 1 forbids reading Facets. Not gated on tangibility — factions have Tier.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="70" t="inlineStr">
-        <is>
-          <t>Place / containment reference</t>
-        </is>
-      </c>
-      <c r="B13" s="70" t="inlineStr">
-        <is>
-          <t>stretch</t>
-        </is>
-      </c>
-      <c r="C13" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D13" s="70" t="inlineStr">
-        <is>
-          <t>stretch</t>
-        </is>
-      </c>
-      <c r="E13" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F13" s="70" t="inlineStr">
-        <is>
-          <t>ARGUE. A rumour's "place" is where it is believed; a faction's is its turf. Both are real and both are stretched.</t>
+      <c r="A13" s="76" t="inlineStr">
+        <is>
+          <t>facets</t>
+        </is>
+      </c>
+      <c r="B13" s="76" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="C13" s="76" t="inlineStr">
+        <is>
+          <t>per-Component data</t>
+        </is>
+      </c>
+      <c r="D13" s="76" t="inlineStr">
+        <is>
+          <t>The escape hatch: anything that is NOT one of the five Noun kinds. WATCH THIS — anything put here that another Component must read is a missing Noun slot in disguise.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="70" t="inlineStr">
-        <is>
-          <t>the 14 non-attempt Dimensions</t>
-        </is>
-      </c>
-      <c r="B14" s="70" t="inlineStr">
-        <is>
-          <t>stretch</t>
-        </is>
-      </c>
-      <c r="C14" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D14" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E14" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F14" s="70" t="inlineStr">
-        <is>
-          <t>ARGUE. A rumour has no temperature — but "absent is not zero" already covers that, so the cost of including them may be zero.</t>
+      <c r="A14" s="76" t="inlineStr">
+        <is>
+          <t>capacities</t>
+        </is>
+      </c>
+      <c r="B14" s="76" t="inlineStr">
+        <is>
+          <t>Noun slot</t>
+        </is>
+      </c>
+      <c r="C14" s="76" t="inlineStr">
+        <is>
+          <t>Capacity ID -&gt; value</t>
+        </is>
+      </c>
+      <c r="D14" s="76" t="inlineStr">
+        <is>
+          <t>The fifteen attempt Dimensions live here.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="70" t="inlineStr">
-        <is>
-          <t>the 15 attempt Dimensions</t>
-        </is>
-      </c>
-      <c r="B15" s="70" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="C15" s="70" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D15" s="70" t="inlineStr">
-        <is>
-          <t>maybe</t>
-        </is>
-      </c>
-      <c r="E15" s="70" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F15" s="70" t="inlineStr">
-        <is>
-          <t>NOT UNIVERSAL → L3. A building never attempts a grapple; a Relationship never rolls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="70" t="inlineStr">
-        <is>
-          <t>PERSON-ASSUMPTIONS THAT LEAK MOST OFTEN, from the survey: initiative (a rumour does not act) · carrying capacity (a faction does not carry) · movement speed (a lock does not move) · level and advancement (a storm does not learn) · hit points.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="71" t="inlineStr">
+      <c r="A15" s="76" t="inlineStr">
+        <is>
+          <t>states</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>Noun slot</t>
+        </is>
+      </c>
+      <c r="C15" s="76" t="inlineStr">
+        <is>
+          <t>axis -&gt; State ID, optional magnitude</t>
+        </is>
+      </c>
+      <c r="D15" s="76" t="inlineStr">
+        <is>
+          <t>Aggregates by MAX, never sum (PF2e's rule; additive stacking makes any repeatable source unbounded).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="76" t="inlineStr">
+        <is>
+          <t>resources</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>Noun slot</t>
+        </is>
+      </c>
+      <c r="C16" s="76" t="inlineStr">
+        <is>
+          <t>Resource ID -&gt; value, with Thresholds</t>
+        </is>
+      </c>
+      <c r="D16" s="76" t="inlineStr">
+        <is>
+          <t>Aggregates by CLAMP. The Substrate ships none.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="76" t="inlineStr">
+        <is>
+          <t>RELATIONSHIP NEEDS NO SLOT — it is an Entity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="71" t="inlineStr">
         <is>
           <t>CONSIDERED AND REJECTED</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="72" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B20" s="72" t="inlineStr"/>
-      <c r="C20" s="72" t="inlineStr"/>
-      <c r="D20" s="72" t="inlineStr"/>
-      <c r="E20" s="72" t="inlineStr"/>
-      <c r="F20" s="72" t="inlineStr">
-        <is>
-          <t>ARGUE: is a display name Substrate, or a Lens concern? A pending vector has no name anyone says out loud.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="72" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>exists</t>
         </is>
       </c>
       <c r="B21" s="72" t="inlineStr"/>
       <c r="C21" s="72" t="inlineStr"/>
-      <c r="D21" s="72" t="inlineStr"/>
-      <c r="E21" s="72" t="inlineStr"/>
-      <c r="F21" s="72" t="inlineStr">
-        <is>
-          <t>REJECT: that is a Relationship.</t>
+      <c r="D21" s="72" t="inlineStr">
+        <is>
+          <t>SPLIT. Destruction is a STATE on a lifecycle axis; retraction is a COMPENSATING RECORD, so the Entity is simply not produced by the Fold. No boolean, no default, no predicate to forget. Under "absent is not zero" a boolean would be three-valued with an INVERTED safe default.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="72" t="inlineStr">
         <is>
-          <t>initiative</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B22" s="72" t="inlineStr"/>
       <c r="C22" s="72" t="inlineStr"/>
-      <c r="D22" s="72" t="inlineStr"/>
-      <c r="E22" s="72" t="inlineStr"/>
-      <c r="F22" s="72" t="inlineStr">
-        <is>
-          <t>REJECT: person-assumption, and turn order is base Ruleset.</t>
+      <c r="D22" s="72" t="inlineStr">
+        <is>
+          <t>The PLACE SOCKET's Facet. Only the occupant interprets it; the Substrate never needs to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="72" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B23" s="72" t="inlineStr"/>
+      <c r="C23" s="72" t="inlineStr"/>
+      <c r="D23" s="72" t="inlineStr">
+        <is>
+          <t>A LENS concern. Setting-specific, and the likeliest place for rule 10 (PII) to be violated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="72" t="inlineStr">
+        <is>
+          <t>mass / bulk</t>
+        </is>
+      </c>
+      <c r="B24" s="72" t="inlineStr"/>
+      <c r="C24" s="72" t="inlineStr"/>
+      <c r="D24" s="72" t="inlineStr">
+        <is>
+          <t>TAGS, with magnitudes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="72" t="inlineStr">
+        <is>
+          <t>hardness</t>
+        </is>
+      </c>
+      <c r="B25" s="72" t="inlineStr"/>
+      <c r="C25" s="72" t="inlineStr"/>
+      <c r="D25" s="72" t="inlineStr">
+        <is>
+          <t>A FLAT GUARD at R-850. Not an attribute at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>the fourteen Dimensions</t>
+        </is>
+      </c>
+      <c r="B26" s="72" t="inlineStr"/>
+      <c r="C26" s="72" t="inlineStr"/>
+      <c r="D26" s="72" t="inlineStr">
+        <is>
+          <t>Axes a VECTOR travels on, never fields on a target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="72" t="inlineStr">
+        <is>
+          <t>the inverse of any link</t>
+        </is>
+      </c>
+      <c r="B27" s="72" t="inlineStr"/>
+      <c r="C27" s="72" t="inlineStr"/>
+      <c r="D27" s="72" t="inlineStr">
+        <is>
+          <t>DERIVED by the Fold. Writing both directions is denormalisation, and denormalisation desyncs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="72" t="inlineStr">
+        <is>
+          <t>generation / version counter</t>
+        </is>
+      </c>
+      <c r="B28" s="72" t="inlineStr"/>
+      <c r="C28" s="72" t="inlineStr"/>
+      <c r="D28" s="72" t="inlineStr">
+        <is>
+          <t>Not needed — generational indices exist to stop a RECYCLED id pointing at a new entity. Never reusing ids removes the precondition, and a Record from 400 Moments ago then needs one integer rather than two forever.</t>
         </is>
       </c>
     </row>
@@ -13859,655 +14136,381 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" style="18" min="1" max="1"/>
-    <col width="40" customWidth="1" style="18" min="2" max="2"/>
-    <col width="30" customWidth="1" style="18" min="3" max="3"/>
-    <col width="24" customWidth="1" style="18" min="4" max="4"/>
-    <col width="34" customWidth="1" style="18" min="5" max="5"/>
+    <col width="16" customWidth="1" style="19" min="1" max="1"/>
+    <col width="38" customWidth="1" style="19" min="2" max="2"/>
+    <col width="20" customWidth="1" style="19" min="3" max="3"/>
+    <col width="32" customWidth="1" style="19" min="4" max="4"/>
+    <col width="54" customWidth="1" style="19" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.35" customHeight="1" s="19">
-      <c r="A1" s="20" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="63" t="inlineStr">
         <is>
           <t>L3 · Category Attributes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="19">
-      <c r="A2" s="28" t="inlineStr">
-        <is>
-          <t>PENDING · BLOCKING</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1" s="19">
-      <c r="A3" s="21" t="inlineStr">
-        <is>
-          <t>What each Category adds. Fill after L1 and L2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1" s="19">
-      <c r="A4" s="32" t="inlineStr">
-        <is>
-          <t>NOW SEEDABLE — the Dimensions tell you what each Category needs to carry. An Attribute here is what a FORMULA reads to produce a Dimension value or a Threshold.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="19">
-      <c r="A6" s="33" t="inlineStr">
-        <is>
-          <t>Category (L1)</t>
-        </is>
-      </c>
-      <c r="B6" s="33" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="D6" s="33" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
-      <c r="E6" s="33" t="inlineStr">
-        <is>
-          <t>Why this Category needs it</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="19">
-      <c r="A7" s="34" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
-      <c r="B7" s="34" t="inlineStr">
-        <is>
-          <t>allocation points</t>
-        </is>
-      </c>
-      <c r="C7" s="34" t="inlineStr">
-        <is>
-          <t>whole number</t>
-        </is>
-      </c>
-      <c r="D7" s="34" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E7" s="34" t="inlineStr">
-        <is>
-          <t>How finely they can split attention</t>
-        </is>
-      </c>
-      <c r="F7" s="35" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="64" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="65" t="inlineStr">
+        <is>
+          <t>What each Category brings. Substrate Categories bring an ENFORCED shape; Ruleset Categories bring default field presence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>THE ABSENCE OF A ROW IS THE MECHANISM, NOT AN OMISSION. Item has no mental State axes, which is exactly why a fear vector against a vase resolves fully and lands on nothing. A COMPOSED ENTITY TAKES THE UNION.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="67" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B6" s="67" t="inlineStr">
+        <is>
+          <t>Capacities</t>
+        </is>
+      </c>
+      <c r="C6" s="67" t="inlineStr">
+        <is>
+          <t>Resources</t>
+        </is>
+      </c>
+      <c r="D6" s="67" t="inlineStr">
+        <is>
+          <t>State axes</t>
+        </is>
+      </c>
+      <c r="E6" s="67" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="68" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="B7" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C7" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="68" t="inlineStr">
+        <is>
+          <t>No Category. REJECTED in L1.</t>
+        </is>
+      </c>
+      <c r="F7" s="69" t="inlineStr">
         <is>
           <t>← example, not data</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="19">
-      <c r="A8" s="36" t="inlineStr">
-        <is>
-          <t>being</t>
-        </is>
-      </c>
-      <c r="B8" s="36" t="inlineStr">
-        <is>
-          <t>vitality pool</t>
-        </is>
-      </c>
-      <c r="C8" s="36" t="inlineStr">
-        <is>
-          <t>integer Resource</t>
-        </is>
-      </c>
-      <c r="D8" s="36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E8" s="36" t="inlineStr">
-        <is>
-          <t>vitality landings need somewhere to go</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="19">
-      <c r="A9" s="36" t="inlineStr">
-        <is>
-          <t>being</t>
-        </is>
-      </c>
-      <c r="B9" s="36" t="inlineStr">
-        <is>
-          <t>vigor pool</t>
-        </is>
-      </c>
-      <c r="C9" s="36" t="inlineStr">
-        <is>
-          <t>integer Resource</t>
-        </is>
-      </c>
-      <c r="D9" s="36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>exhaustion needs somewhere to go</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="19">
-      <c r="A10" s="36" t="inlineStr">
-        <is>
-          <t>being</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="inlineStr">
-        <is>
-          <t>the three mental pools</t>
-        </is>
-      </c>
-      <c r="C10" s="36" t="inlineStr">
-        <is>
-          <t>integer Resources</t>
-        </is>
-      </c>
-      <c r="D10" s="36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>composure, clarity, will landings</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="19">
-      <c r="A11" s="36" t="inlineStr">
-        <is>
-          <t>being</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="inlineStr">
-        <is>
-          <t>reach / stride</t>
-        </is>
-      </c>
-      <c r="C11" s="36" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="D11" s="36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E11" s="36" t="inlineStr">
-        <is>
-          <t>feeds mobility</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="19">
-      <c r="A12" s="36" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="inlineStr">
-        <is>
-          <t>integrity pool</t>
-        </is>
-      </c>
-      <c r="C12" s="36" t="inlineStr">
-        <is>
-          <t>integer Resource</t>
-        </is>
-      </c>
-      <c r="D12" s="36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E12" s="36" t="inlineStr"/>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="19">
-      <c r="A13" s="36" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="inlineStr">
-        <is>
-          <t>substance pool</t>
-        </is>
-      </c>
-      <c r="C13" s="36" t="inlineStr">
-        <is>
-          <t>integer Resource</t>
-        </is>
-      </c>
-      <c r="D13" s="36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E13" s="36" t="inlineStr"/>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="19">
-      <c r="A14" s="36" t="inlineStr">
-        <is>
-          <t>structure</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="inlineStr">
-        <is>
-          <t>parts</t>
-        </is>
-      </c>
-      <c r="C14" s="36" t="inlineStr">
-        <is>
-          <t>list of Entity ids</t>
-        </is>
-      </c>
-      <c r="D14" s="36" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
-      <c r="E14" s="36" t="inlineStr">
-        <is>
-          <t>each part carries its own Scale and Thresholds</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="19">
-      <c r="A15" s="36" t="inlineStr">
-        <is>
-          <t>place</t>
-        </is>
-      </c>
-      <c r="B15" s="36" t="inlineStr">
-        <is>
-          <t>scope</t>
-        </is>
-      </c>
-      <c r="C15" s="36" t="inlineStr">
-        <is>
-          <t>Place Socket vocabulary</t>
-        </is>
-      </c>
-      <c r="D15" s="36" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E15" s="36" t="inlineStr">
-        <is>
-          <t>what "here" and "near" mean is the Place Socket's job</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="19">
-      <c r="A16" s="36" t="inlineStr">
-        <is>
-          <t>place</t>
-        </is>
-      </c>
-      <c r="B16" s="36" t="inlineStr">
-        <is>
-          <t>connections</t>
-        </is>
-      </c>
-      <c r="C16" s="36" t="inlineStr">
-        <is>
-          <t>list of place ids</t>
-        </is>
-      </c>
-      <c r="D16" s="36" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
-      <c r="E16" s="36" t="inlineStr"/>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="19">
-      <c r="A17" s="36" t="inlineStr">
-        <is>
-          <t>group</t>
-        </is>
-      </c>
-      <c r="B17" s="36" t="inlineStr">
-        <is>
-          <t>membership</t>
-        </is>
-      </c>
-      <c r="C17" s="36" t="inlineStr">
-        <is>
-          <t>list of Entity ids</t>
-        </is>
-      </c>
-      <c r="D17" s="36" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
-      <c r="E17" s="36" t="inlineStr"/>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="19">
-      <c r="A18" s="36" t="inlineStr">
-        <is>
-          <t>group</t>
-        </is>
-      </c>
-      <c r="B18" s="36" t="inlineStr">
-        <is>
-          <t>cohesion</t>
-        </is>
-      </c>
-      <c r="C18" s="36" t="inlineStr">
-        <is>
-          <t>integer Resource</t>
-        </is>
-      </c>
-      <c r="D18" s="36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E18" s="36" t="inlineStr">
-        <is>
-          <t>the group's equivalent of integrity</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="19">
-      <c r="A19" s="36" t="inlineStr">
-        <is>
-          <t>relationship</t>
-        </is>
-      </c>
-      <c r="B19" s="36" t="inlineStr">
-        <is>
-          <t>connections</t>
-        </is>
-      </c>
-      <c r="C19" s="36" t="inlineStr">
-        <is>
-          <t>one Connection per participant</t>
-        </is>
-      </c>
-      <c r="D19" s="36" t="inlineStr">
+      <c r="C8" s="76" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E19" s="36" t="inlineStr">
-        <is>
-          <t>each stance stored INDEPENDENTLY. Never an edge</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="19">
-      <c r="A20" s="36" t="inlineStr">
-        <is>
-          <t>information</t>
-        </is>
-      </c>
-      <c r="B20" s="36" t="inlineStr">
-        <is>
-          <t>truth</t>
-        </is>
-      </c>
-      <c r="C20" s="36" t="inlineStr">
-        <is>
-          <t>boolean or graded</t>
-        </is>
-      </c>
-      <c r="D20" s="36" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="E20" s="36" t="inlineStr">
-        <is>
-          <t>a rumour can be false and still spread</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="19">
-      <c r="A21" s="36" t="inlineStr">
-        <is>
-          <t>occasion</t>
-        </is>
-      </c>
-      <c r="B21" s="36" t="inlineStr">
-        <is>
-          <t>when</t>
-        </is>
-      </c>
-      <c r="C21" s="36" t="inlineStr">
-        <is>
-          <t>a Moment</t>
-        </is>
-      </c>
-      <c r="D21" s="36" t="inlineStr">
+      <c r="D8" s="76" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="36" t="inlineStr"/>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="19">
-      <c r="A22" s="36" t="inlineStr"/>
-      <c r="B22" s="36" t="inlineStr"/>
-      <c r="C22" s="36" t="inlineStr"/>
-      <c r="D22" s="36" t="inlineStr"/>
-      <c r="E22" s="36" t="inlineStr"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="19">
-      <c r="A23" s="36" t="inlineStr">
-        <is>
-          <t>THE OVERLAP TEST: if the same word means the same thing on two Categories, define it once at the most general Category that needs it.</t>
-        </is>
-      </c>
-      <c r="B23" s="36" t="inlineStr"/>
-      <c r="C23" s="36" t="inlineStr"/>
-      <c r="D23" s="36" t="inlineStr"/>
-      <c r="E23" s="36" t="inlineStr"/>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="19">
-      <c r="A24" s="37" t="n"/>
-      <c r="B24" s="37" t="n"/>
-      <c r="C24" s="37" t="n"/>
-      <c r="D24" s="37" t="n"/>
-      <c r="E24" s="37" t="n"/>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="19">
-      <c r="A25" s="37" t="n"/>
-      <c r="B25" s="37" t="n"/>
-      <c r="C25" s="37" t="n"/>
-      <c r="D25" s="37" t="n"/>
-      <c r="E25" s="37" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="19">
-      <c r="A26" s="37" t="n"/>
-      <c r="B26" s="37" t="n"/>
-      <c r="C26" s="37" t="n"/>
-      <c r="D26" s="37" t="n"/>
-      <c r="E26" s="37" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="19">
-      <c r="A27" s="37" t="n"/>
-      <c r="B27" s="37" t="n"/>
-      <c r="C27" s="37" t="n"/>
-      <c r="D27" s="37" t="n"/>
-      <c r="E27" s="37" t="n"/>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="19">
-      <c r="A28" s="37" t="n"/>
-      <c r="B28" s="37" t="n"/>
-      <c r="C28" s="37" t="n"/>
-      <c r="D28" s="37" t="n"/>
-      <c r="E28" s="37" t="n"/>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="19">
-      <c r="A29" s="37" t="n"/>
-      <c r="B29" s="37" t="n"/>
-      <c r="C29" s="37" t="n"/>
-      <c r="D29" s="37" t="n"/>
-      <c r="E29" s="37" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="19">
-      <c r="A30" s="37" t="n"/>
-      <c r="B30" s="37" t="n"/>
-      <c r="C30" s="37" t="n"/>
-      <c r="D30" s="37" t="n"/>
-      <c r="E30" s="37" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="19">
-      <c r="A31" s="37" t="n"/>
-      <c r="B31" s="37" t="n"/>
-      <c r="C31" s="37" t="n"/>
-      <c r="D31" s="37" t="n"/>
-      <c r="E31" s="37" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="19">
-      <c r="A32" s="37" t="n"/>
-      <c r="B32" s="37" t="n"/>
-      <c r="C32" s="37" t="n"/>
-      <c r="D32" s="37" t="n"/>
-      <c r="E32" s="37" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="19">
-      <c r="A33" s="37" t="n"/>
-      <c r="B33" s="37" t="n"/>
-      <c r="C33" s="37" t="n"/>
-      <c r="D33" s="37" t="n"/>
-      <c r="E33" s="37" t="n"/>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="19">
-      <c r="A34" s="37" t="n"/>
-      <c r="B34" s="37" t="n"/>
-      <c r="C34" s="37" t="n"/>
-      <c r="D34" s="37" t="n"/>
-      <c r="E34" s="37" t="n"/>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="19">
-      <c r="A35" s="37" t="n"/>
-      <c r="B35" s="37" t="n"/>
-      <c r="C35" s="37" t="n"/>
-      <c r="D35" s="37" t="n"/>
-      <c r="E35" s="37" t="n"/>
-    </row>
-    <row r="36" ht="15" customHeight="1" s="19">
-      <c r="A36" s="37" t="n"/>
-      <c r="B36" s="37" t="n"/>
-      <c r="C36" s="37" t="n"/>
-      <c r="D36" s="37" t="n"/>
-      <c r="E36" s="37" t="n"/>
-    </row>
-    <row r="37" ht="15" customHeight="1" s="19">
-      <c r="A37" s="37" t="n"/>
-      <c r="B37" s="37" t="n"/>
-      <c r="C37" s="37" t="n"/>
-      <c r="D37" s="37" t="n"/>
-      <c r="E37" s="37" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="19">
-      <c r="A38" s="37" t="n"/>
-      <c r="B38" s="37" t="n"/>
-      <c r="C38" s="37" t="n"/>
-      <c r="D38" s="37" t="n"/>
-      <c r="E38" s="37" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="19">
-      <c r="A39" s="37" t="n"/>
-      <c r="B39" s="37" t="n"/>
-      <c r="C39" s="37" t="n"/>
-      <c r="D39" s="37" t="n"/>
-      <c r="E39" s="37" t="n"/>
-    </row>
-    <row r="40" ht="15" customHeight="1" s="19">
-      <c r="A40" s="37" t="n"/>
-      <c r="B40" s="37" t="n"/>
-      <c r="C40" s="37" t="n"/>
-      <c r="D40" s="37" t="n"/>
-      <c r="E40" s="37" t="n"/>
-    </row>
-    <row r="41" ht="15" customHeight="1" s="19">
-      <c r="A41" s="37" t="n"/>
-      <c r="B41" s="37" t="n"/>
-      <c r="C41" s="37" t="n"/>
-      <c r="D41" s="37" t="n"/>
-      <c r="E41" s="37" t="n"/>
-    </row>
-    <row r="42" ht="15" customHeight="1" s="19">
-      <c r="A42" s="37" t="n"/>
-      <c r="B42" s="37" t="n"/>
-      <c r="C42" s="37" t="n"/>
-      <c r="D42" s="37" t="n"/>
-      <c r="E42" s="37" t="n"/>
-    </row>
-    <row r="43" ht="15" customHeight="1" s="19">
-      <c r="A43" s="37" t="n"/>
-      <c r="B43" s="37" t="n"/>
-      <c r="C43" s="37" t="n"/>
-      <c r="D43" s="37" t="n"/>
-      <c r="E43" s="37" t="n"/>
-    </row>
-    <row r="44" ht="15" customHeight="1" s="19">
-      <c r="A44" s="37" t="n"/>
-      <c r="B44" s="37" t="n"/>
-      <c r="C44" s="37" t="n"/>
-      <c r="D44" s="37" t="n"/>
-      <c r="E44" s="37" t="n"/>
-    </row>
-    <row r="45" ht="15" customHeight="1" s="19">
-      <c r="A45" s="37" t="n"/>
-      <c r="B45" s="37" t="n"/>
-      <c r="C45" s="37" t="n"/>
-      <c r="D45" s="37" t="n"/>
-      <c r="E45" s="37" t="n"/>
-    </row>
-    <row r="46" ht="15" customHeight="1" s="19">
-      <c r="A46" s="37" t="n"/>
-      <c r="B46" s="37" t="n"/>
-      <c r="C46" s="37" t="n"/>
-      <c r="D46" s="37" t="n"/>
-      <c r="E46" s="37" t="n"/>
-    </row>
-    <row r="47" ht="15" customHeight="1" s="19">
-      <c r="A47" s="37" t="n"/>
-      <c r="B47" s="37" t="n"/>
-      <c r="C47" s="37" t="n"/>
-      <c r="D47" s="37" t="n"/>
-      <c r="E47" s="37" t="n"/>
+      <c r="E8" s="76" t="inlineStr">
+        <is>
+          <t>ENFORCED: direction · magnitude · target (exactly one) · pin · layer · class</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="76" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="76" t="inlineStr">
+        <is>
+          <t>ENFORCED: decider · moment · default · subject</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="76" t="inlineStr">
+        <is>
+          <t>Relationship</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="76" t="inlineStr">
+        <is>
+          <t>ENFORCED: connections[] — one per participant: holder · about · stance</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="76" t="inlineStr">
+        <is>
+          <t>Creature</t>
+        </is>
+      </c>
+      <c r="B11" s="76" t="inlineStr">
+        <is>
+          <t>the fifteen attempt Dimensions</t>
+        </is>
+      </c>
+      <c r="C11" s="76" t="inlineStr">
+        <is>
+          <t>vitality</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr">
+        <is>
+          <t>posture · awareness · consciousness</t>
+        </is>
+      </c>
+      <c r="E11" s="76" t="inlineStr">
+        <is>
+          <t>Specialisations</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>integrity</t>
+        </is>
+      </c>
+      <c r="D12" s="76" t="inlineStr">
+        <is>
+          <t>access</t>
+        </is>
+      </c>
+      <c r="E12" s="76" t="inlineStr">
+        <is>
+          <t>mass and bulk Tags; Guards</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="76" t="inlineStr">
+        <is>
+          <t>Place</t>
+        </is>
+      </c>
+      <c r="B13" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C13" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D13" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="76" t="inlineStr">
+        <is>
+          <t>extent and containment, per the Place Socket</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="76" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B14" s="76" t="inlineStr">
+        <is>
+          <t>the attempt Dimensions IF it also carries Creature</t>
+        </is>
+      </c>
+      <c r="C14" s="76" t="inlineStr">
+        <is>
+          <t>standing</t>
+        </is>
+      </c>
+      <c r="D14" s="76" t="inlineStr">
+        <is>
+          <t>posture</t>
+        </is>
+      </c>
+      <c r="E14" s="76" t="inlineStr">
+        <is>
+          <t>membership via member_of</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="76" t="inlineStr">
+        <is>
+          <t>Notion</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C15" s="76" t="inlineStr">
+        <is>
+          <t>credibility</t>
+        </is>
+      </c>
+      <c r="D15" s="76" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="E15" s="76" t="inlineStr">
+        <is>
+          <t>provenance. NO location, NO harm pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="76" t="inlineStr">
+        <is>
+          <t>Phenomenon</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C16" s="76" t="inlineStr">
+        <is>
+          <t>fuel</t>
+        </is>
+      </c>
+      <c r="D16" s="76" t="inlineStr">
+        <is>
+          <t>intensity</t>
+        </is>
+      </c>
+      <c r="E16" s="76" t="inlineStr">
+        <is>
+          <t>a standing vector, scoped by Place</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="76" t="inlineStr">
+        <is>
+          <t>WORKED: a sentient sword is Item + Creature — integrity AND vitality, mass AND attempt Capacities, smashable AND frightenable. An elemental plague is Phenomenon + Creature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="71" t="inlineStr">
+        <is>
+          <t>CONSIDERED AND REJECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="72" t="inlineStr">
+        <is>
+          <t>the three character sheets</t>
+        </is>
+      </c>
+      <c r="B21" s="72" t="inlineStr"/>
+      <c r="C21" s="72" t="inlineStr"/>
+      <c r="D21" s="72" t="inlineStr"/>
+      <c r="E21" s="72" t="inlineStr">
+        <is>
+          <t>DEFERRED, deliberately. Person, ship and faction were to be written here as the test of L1-L3. They wait until CHARACTER CREATION is designed, because what a sheet shows is downstream of how a character is made. Writing it first would bake in an authoring path nobody chose.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
L5 Tracks settled: State and Resource merge into Track; conditions become bands; L18 collapses; tag compilations added
</commit_message>
<xml_diff>
--- a/docs/substrate-lists.xlsx
+++ b/docs/substrate-lists.xlsx
@@ -2904,499 +2904,228 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" style="18" min="1" max="1"/>
-    <col width="40" customWidth="1" style="18" min="2" max="2"/>
-    <col width="30" customWidth="1" style="18" min="3" max="3"/>
-    <col width="24" customWidth="1" style="18" min="4" max="4"/>
-    <col width="34" customWidth="1" style="18" min="5" max="5"/>
+    <col width="18" customWidth="1" style="19" min="1" max="1"/>
+    <col width="34" customWidth="1" style="19" min="2" max="2"/>
+    <col width="34" customWidth="1" style="19" min="3" max="3"/>
+    <col width="80" customWidth="1" style="19" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.35" customHeight="1" s="19">
-      <c r="A1" s="20" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="63" t="inlineStr">
         <is>
           <t>L18 · Aggregation operators</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="19">
-      <c r="A2" s="28" t="inlineStr">
-        <is>
-          <t>PENDING · BLOCKING</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1" s="19">
-      <c r="A3" s="21" t="inlineStr">
-        <is>
-          <t>How multiple contributions to one value combine. Declared per Noun kind, overridable only from this closed list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1" s="19">
-      <c r="A4" s="32" t="inlineStr">
-        <is>
-          <t>REVISED. Everything on the resolution path is settled; what remains is the other Noun kinds. NOTE: this is a DIFFERENT question from how a THRESHOLD reads multiple contributors (sum / highest / each), which was settled in L29.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="19">
-      <c r="A6" s="33" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="64" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="65" t="inlineStr">
+        <is>
+          <t>How multiple contributions to one value combine, for the Noun kinds outside the resolution path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>THE TRACK MERGE COLLAPSED MOST OF THIS LIST. Four Noun kinds, four rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="67" t="inlineStr">
+        <is>
+          <t>Noun kind</t>
+        </is>
+      </c>
+      <c r="B6" s="67" t="inlineStr">
         <is>
           <t>Operator</t>
         </is>
       </c>
-      <c r="B6" s="33" t="inlineStr">
-        <is>
-          <t>Applies to which Noun kinds</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>Behaviour</t>
-        </is>
-      </c>
-      <c r="D6" s="33" t="inlineStr">
-        <is>
-          <t>Default for</t>
-        </is>
-      </c>
-      <c r="E6" s="33" t="inlineStr">
+      <c r="C6" s="67" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="D6" s="67" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="19">
-      <c r="A7" s="34" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="68" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B7" s="68" t="inlineStr">
         <is>
           <t>max</t>
         </is>
       </c>
-      <c r="B7" s="34" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="C7" s="34" t="inlineStr">
-        <is>
-          <t>Highest applicable wins</t>
-        </is>
-      </c>
-      <c r="D7" s="34" t="inlineStr">
-        <is>
-          <t>States within an axis</t>
-        </is>
-      </c>
-      <c r="E7" s="34" t="inlineStr">
-        <is>
-          <t>Removes an entire bug class versus sum</t>
-        </is>
-      </c>
-      <c r="F7" s="35" t="inlineStr">
+      <c r="C7" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="68" t="inlineStr">
+        <is>
+          <t>GONE — merged into Track, Aug 2026.</t>
+        </is>
+      </c>
+      <c r="E7" s="69" t="inlineStr">
         <is>
           <t>← example, not data</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="19">
-      <c r="A8" s="36" t="inlineStr">
-        <is>
-          <t>sum</t>
-        </is>
-      </c>
-      <c r="B8" s="36" t="inlineStr">
-        <is>
-          <t>Capacity, Channel values, percentages</t>
-        </is>
-      </c>
-      <c r="C8" s="36" t="inlineStr">
-        <is>
-          <t>add, then clamp</t>
-        </is>
-      </c>
-      <c r="D8" s="36" t="inlineStr">
-        <is>
-          <t>everything on the resolution path</t>
-        </is>
-      </c>
-      <c r="E8" s="36" t="inlineStr">
-        <is>
-          <t>SETTLED in Phase 0. Percentages sum, nothing compounds</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="19">
-      <c r="A9" s="36" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="B9" s="36" t="inlineStr">
-        <is>
-          <t>State magnitude within an axis; Baseline</t>
-        </is>
-      </c>
-      <c r="C9" s="36" t="inlineStr">
-        <is>
-          <t>take the highest</t>
-        </is>
-      </c>
-      <c r="D9" s="36" t="inlineStr">
-        <is>
-          <t>States, Baselines</t>
-        </is>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>PROPOSED. Order-free, therefore safe</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="19">
-      <c r="A10" s="36" t="inlineStr">
-        <is>
-          <t>union</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
+        <is>
+          <t>clamp to its bounds</t>
+        </is>
+      </c>
+      <c r="C8" s="76" t="inlineStr">
+        <is>
+          <t>one kind, one rule</t>
+        </is>
+      </c>
+      <c r="D8" s="76" t="inlineStr">
+        <is>
+          <t>Absorbed State's max and Resource's clamp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="76" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="C10" s="36" t="inlineStr">
-        <is>
-          <t>set union by ID</t>
-        </is>
-      </c>
-      <c r="D10" s="36" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>PROPOSED. Order-free</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="19">
-      <c r="A11" s="36" t="inlineStr">
-        <is>
-          <t>clamp</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="inlineStr">
-        <is>
-          <t>Resource</t>
-        </is>
-      </c>
-      <c r="C11" s="36" t="inlineStr">
-        <is>
-          <t>add, then bound at min and max</t>
-        </is>
-      </c>
-      <c r="D11" s="36" t="inlineStr">
-        <is>
-          <t>Resources</t>
-        </is>
-      </c>
-      <c r="E11" s="36" t="inlineStr">
-        <is>
-          <t>PROPOSED</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="19">
-      <c r="A12" s="36" t="inlineStr">
-        <is>
-          <t>per-Connection</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="inlineStr">
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>union for membership; magnitudes ADD</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>two torches make a brighter room</t>
+        </is>
+      </c>
+      <c r="D9" s="76" t="inlineStr">
+        <is>
+          <t>A Tag that should NOT add is a PROPERTY, and properties are SET at creation rather than GRANTED by effects. Mass is set; illumination is granted. So no per-Tag operator is needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="76" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>none needed</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>increases are Modifiers</t>
+        </is>
+      </c>
+      <c r="D10" s="76" t="inlineStr">
+        <is>
+          <t>Handled at R-300 and R-500.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="76" t="inlineStr">
         <is>
           <t>Relationship</t>
         </is>
       </c>
-      <c r="C12" s="36" t="inlineStr">
-        <is>
-          <t>NEVER merge — each participant's stance stands alone</t>
-        </is>
-      </c>
-      <c r="D12" s="36" t="inlineStr">
-        <is>
-          <t>Relationships</t>
-        </is>
-      </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>PROPOSED. This is why a Relationship is a Category of Entity rather than an edge</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="19">
-      <c r="A13" s="36" t="inlineStr"/>
-      <c r="B13" s="36" t="inlineStr"/>
-      <c r="C13" s="36" t="inlineStr"/>
-      <c r="D13" s="36" t="inlineStr"/>
-      <c r="E13" s="36" t="inlineStr"/>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="19">
-      <c r="A14" s="36" t="inlineStr">
-        <is>
-          <t>THE TEST: apply each operator to the same three inputs in six different orders. Any operator that gives different answers is wrong.</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="inlineStr"/>
-      <c r="C14" s="36" t="inlineStr"/>
-      <c r="D14" s="36" t="inlineStr"/>
-      <c r="E14" s="36" t="inlineStr"/>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="19">
-      <c r="A15" s="36" t="inlineStr">
-        <is>
-          <t>Named in the architecture as the single most likely source of "the same Ledger produced different state".</t>
-        </is>
-      </c>
-      <c r="B15" s="36" t="inlineStr"/>
-      <c r="C15" s="36" t="inlineStr"/>
-      <c r="D15" s="36" t="inlineStr"/>
-      <c r="E15" s="36" t="inlineStr"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="19">
-      <c r="A16" s="37" t="n"/>
-      <c r="B16" s="37" t="n"/>
-      <c r="C16" s="37" t="n"/>
-      <c r="D16" s="37" t="n"/>
-      <c r="E16" s="37" t="n"/>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="19">
-      <c r="A17" s="37" t="n"/>
-      <c r="B17" s="37" t="n"/>
-      <c r="C17" s="37" t="n"/>
-      <c r="D17" s="37" t="n"/>
-      <c r="E17" s="37" t="n"/>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="19">
-      <c r="A18" s="37" t="n"/>
-      <c r="B18" s="37" t="n"/>
-      <c r="C18" s="37" t="n"/>
-      <c r="D18" s="37" t="n"/>
-      <c r="E18" s="37" t="n"/>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="19">
-      <c r="A19" s="37" t="n"/>
-      <c r="B19" s="37" t="n"/>
-      <c r="C19" s="37" t="n"/>
-      <c r="D19" s="37" t="n"/>
-      <c r="E19" s="37" t="n"/>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="19">
-      <c r="A20" s="37" t="n"/>
-      <c r="B20" s="37" t="n"/>
-      <c r="C20" s="37" t="n"/>
-      <c r="D20" s="37" t="n"/>
-      <c r="E20" s="37" t="n"/>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="19">
-      <c r="A21" s="37" t="n"/>
-      <c r="B21" s="37" t="n"/>
-      <c r="C21" s="37" t="n"/>
-      <c r="D21" s="37" t="n"/>
-      <c r="E21" s="37" t="n"/>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="19">
-      <c r="A22" s="37" t="n"/>
-      <c r="B22" s="37" t="n"/>
-      <c r="C22" s="37" t="n"/>
-      <c r="D22" s="37" t="n"/>
-      <c r="E22" s="37" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="19">
-      <c r="A23" s="37" t="n"/>
-      <c r="B23" s="37" t="n"/>
-      <c r="C23" s="37" t="n"/>
-      <c r="D23" s="37" t="n"/>
-      <c r="E23" s="37" t="n"/>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="19">
-      <c r="A24" s="37" t="n"/>
-      <c r="B24" s="37" t="n"/>
-      <c r="C24" s="37" t="n"/>
-      <c r="D24" s="37" t="n"/>
-      <c r="E24" s="37" t="n"/>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="19">
-      <c r="A25" s="37" t="n"/>
-      <c r="B25" s="37" t="n"/>
-      <c r="C25" s="37" t="n"/>
-      <c r="D25" s="37" t="n"/>
-      <c r="E25" s="37" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="19">
-      <c r="A26" s="37" t="n"/>
-      <c r="B26" s="37" t="n"/>
-      <c r="C26" s="37" t="n"/>
-      <c r="D26" s="37" t="n"/>
-      <c r="E26" s="37" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="19">
-      <c r="A27" s="37" t="n"/>
-      <c r="B27" s="37" t="n"/>
-      <c r="C27" s="37" t="n"/>
-      <c r="D27" s="37" t="n"/>
-      <c r="E27" s="37" t="n"/>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="19">
-      <c r="A28" s="37" t="n"/>
-      <c r="B28" s="37" t="n"/>
-      <c r="C28" s="37" t="n"/>
-      <c r="D28" s="37" t="n"/>
-      <c r="E28" s="37" t="n"/>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="19">
-      <c r="A29" s="37" t="n"/>
-      <c r="B29" s="37" t="n"/>
-      <c r="C29" s="37" t="n"/>
-      <c r="D29" s="37" t="n"/>
-      <c r="E29" s="37" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="19">
-      <c r="A30" s="37" t="n"/>
-      <c r="B30" s="37" t="n"/>
-      <c r="C30" s="37" t="n"/>
-      <c r="D30" s="37" t="n"/>
-      <c r="E30" s="37" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="19">
-      <c r="A31" s="37" t="n"/>
-      <c r="B31" s="37" t="n"/>
-      <c r="C31" s="37" t="n"/>
-      <c r="D31" s="37" t="n"/>
-      <c r="E31" s="37" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="19">
-      <c r="A32" s="37" t="n"/>
-      <c r="B32" s="37" t="n"/>
-      <c r="C32" s="37" t="n"/>
-      <c r="D32" s="37" t="n"/>
-      <c r="E32" s="37" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="19">
-      <c r="A33" s="37" t="n"/>
-      <c r="B33" s="37" t="n"/>
-      <c r="C33" s="37" t="n"/>
-      <c r="D33" s="37" t="n"/>
-      <c r="E33" s="37" t="n"/>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="19">
-      <c r="A34" s="37" t="n"/>
-      <c r="B34" s="37" t="n"/>
-      <c r="C34" s="37" t="n"/>
-      <c r="D34" s="37" t="n"/>
-      <c r="E34" s="37" t="n"/>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="19">
-      <c r="A35" s="37" t="n"/>
-      <c r="B35" s="37" t="n"/>
-      <c r="C35" s="37" t="n"/>
-      <c r="D35" s="37" t="n"/>
-      <c r="E35" s="37" t="n"/>
-    </row>
-    <row r="36" ht="15" customHeight="1" s="19">
-      <c r="A36" s="37" t="n"/>
-      <c r="B36" s="37" t="n"/>
-      <c r="C36" s="37" t="n"/>
-      <c r="D36" s="37" t="n"/>
-      <c r="E36" s="37" t="n"/>
-    </row>
-    <row r="37" ht="15" customHeight="1" s="19">
-      <c r="A37" s="37" t="n"/>
-      <c r="B37" s="37" t="n"/>
-      <c r="C37" s="37" t="n"/>
-      <c r="D37" s="37" t="n"/>
-      <c r="E37" s="37" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="19">
-      <c r="A38" s="37" t="n"/>
-      <c r="B38" s="37" t="n"/>
-      <c r="C38" s="37" t="n"/>
-      <c r="D38" s="37" t="n"/>
-      <c r="E38" s="37" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="19">
-      <c r="A39" s="37" t="n"/>
-      <c r="B39" s="37" t="n"/>
-      <c r="C39" s="37" t="n"/>
-      <c r="D39" s="37" t="n"/>
-      <c r="E39" s="37" t="n"/>
-    </row>
-    <row r="40" ht="15" customHeight="1" s="19">
-      <c r="A40" s="37" t="n"/>
-      <c r="B40" s="37" t="n"/>
-      <c r="C40" s="37" t="n"/>
-      <c r="D40" s="37" t="n"/>
-      <c r="E40" s="37" t="n"/>
-    </row>
-    <row r="41" ht="15" customHeight="1" s="19">
-      <c r="A41" s="37" t="n"/>
-      <c r="B41" s="37" t="n"/>
-      <c r="C41" s="37" t="n"/>
-      <c r="D41" s="37" t="n"/>
-      <c r="E41" s="37" t="n"/>
-    </row>
-    <row r="42" ht="15" customHeight="1" s="19">
-      <c r="A42" s="37" t="n"/>
-      <c r="B42" s="37" t="n"/>
-      <c r="C42" s="37" t="n"/>
-      <c r="D42" s="37" t="n"/>
-      <c r="E42" s="37" t="n"/>
-    </row>
-    <row r="43" ht="15" customHeight="1" s="19">
-      <c r="A43" s="37" t="n"/>
-      <c r="B43" s="37" t="n"/>
-      <c r="C43" s="37" t="n"/>
-      <c r="D43" s="37" t="n"/>
-      <c r="E43" s="37" t="n"/>
-    </row>
-    <row r="44" ht="15" customHeight="1" s="19">
-      <c r="A44" s="37" t="n"/>
-      <c r="B44" s="37" t="n"/>
-      <c r="C44" s="37" t="n"/>
-      <c r="D44" s="37" t="n"/>
-      <c r="E44" s="37" t="n"/>
-    </row>
-    <row r="45" ht="15" customHeight="1" s="19">
-      <c r="A45" s="37" t="n"/>
-      <c r="B45" s="37" t="n"/>
-      <c r="C45" s="37" t="n"/>
-      <c r="D45" s="37" t="n"/>
-      <c r="E45" s="37" t="n"/>
-    </row>
-    <row r="46" ht="15" customHeight="1" s="19">
-      <c r="A46" s="37" t="n"/>
-      <c r="B46" s="37" t="n"/>
-      <c r="C46" s="37" t="n"/>
-      <c r="D46" s="37" t="n"/>
-      <c r="E46" s="37" t="n"/>
-    </row>
-    <row r="47" ht="15" customHeight="1" s="19">
-      <c r="A47" s="37" t="n"/>
-      <c r="B47" s="37" t="n"/>
-      <c r="C47" s="37" t="n"/>
-      <c r="D47" s="37" t="n"/>
-      <c r="E47" s="37" t="n"/>
+      <c r="B11" s="76" t="inlineStr">
+        <is>
+          <t>NEVER MERGE</t>
+        </is>
+      </c>
+      <c r="C11" s="76" t="inlineStr">
+        <is>
+          <t>each stance stands alone</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr">
+        <is>
+          <t>The whole reason a Relationship is an Entity and not an edge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="76" t="inlineStr">
+        <is>
+          <t>THE TEST: apply each operator to the same three inputs in SIX different orders. Any operator that gives different answers is wrong. This list is named in the architecture as the single most likely source of "the same Ledger produced different state."</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="71" t="inlineStr">
+        <is>
+          <t>CONSIDERED AND REJECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="72" t="inlineStr">
+        <is>
+          <t>lowest (for Thresholds)</t>
+        </is>
+      </c>
+      <c r="B16" s="72" t="inlineStr"/>
+      <c r="C16" s="72" t="inlineStr"/>
+      <c r="D16" s="72" t="inlineStr">
+        <is>
+          <t>REJECTED in Phase 0 — a weakest-link rule punishes the party for letting anyone participate. Threshold modes are sum, highest and each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="72" t="inlineStr">
+        <is>
+          <t>compounding percentages</t>
+        </is>
+      </c>
+      <c r="B17" s="72" t="inlineStr"/>
+      <c r="C17" s="72" t="inlineStr"/>
+      <c r="D17" s="72" t="inlineStr">
+        <is>
+          <t>REJECTED in Phase 0 — percentages SUM and apply once. Nothing compounds anywhere.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -7846,21 +7575,21 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="19">
-      <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t>L5 · State axes</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>PENDING · BLOCKING</t>
-        </is>
-      </c>
-      <c r="C9" s="26">
+      <c r="A9" s="73" t="inlineStr">
+        <is>
+          <t>L5 · Tracks</t>
+        </is>
+      </c>
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="73">
         <f>COUNTA('L5 State axes'!A8:A47)</f>
         <v/>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="73">
         <f>IF(C9&gt;0,"started","not started")</f>
         <v/>
       </c>
@@ -7986,21 +7715,21 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="19">
-      <c r="A16" s="26" t="inlineStr">
+      <c r="A16" s="73" t="inlineStr">
         <is>
           <t>L18 · Aggregation operators</t>
         </is>
       </c>
-      <c r="B16" s="30" t="inlineStr">
-        <is>
-          <t>PENDING · BLOCKING</t>
-        </is>
-      </c>
-      <c r="C16" s="26">
+      <c r="B16" s="74" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+      <c r="C16" s="73">
         <f>COUNTA('L18 Aggregation operators'!A8:A47)</f>
         <v/>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="73">
         <f>IF(C16&gt;0,"started","not started")</f>
         <v/>
       </c>
@@ -15321,75 +15050,75 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" style="19" min="1" max="1"/>
-    <col width="44" customWidth="1" style="19" min="2" max="2"/>
-    <col width="20" customWidth="1" style="19" min="3" max="3"/>
-    <col width="64" customWidth="1" style="19" min="4" max="4"/>
-    <col width="34" customWidth="1" style="19" min="5" max="5"/>
+    <col width="26" customWidth="1" style="19" min="1" max="1"/>
+    <col width="28" customWidth="1" style="19" min="2" max="2"/>
+    <col width="52" customWidth="1" style="19" min="3" max="3"/>
+    <col width="34" customWidth="1" style="19" min="4" max="4"/>
+    <col width="12" customWidth="1" style="19" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="63" t="inlineStr">
         <is>
-          <t>L5 · State axes</t>
+          <t>L5 · Tracks   (was: State axes)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="64" t="inlineStr">
         <is>
-          <t>PENDING · BLOCKING · research-seeded Aug 2026</t>
+          <t>SETTLED · Aug 2026 · fourteen</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="65" t="inlineStr">
         <is>
-          <t>The shape, not the contents. What axes the base Ruleset ships, and what fields a State definition carries. Most States live in Components.</t>
+          <t>A Track is a bounded value with a MAXIMUM, a CURRENT and NAMED BANDS. It is the persistent counterpart of a Dimension: the Dimension is the axis a vector travels on, the Track is the standing value on that axis.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="66" t="inlineStr">
         <is>
-          <t>THE DECISION IS AXES, NOT CONDITIONS. The test: can two members be true at once? If yes, they are two axes, or they are Tags.</t>
+          <t>INFLICTING CHARM IS NO DIFFERENT FROM THROWING A FIREBALL. Same machinery, different axis. MAX IS GOOD, ZERO IS COMPROMISED — except the two BIPOLAR axes, where the MIDDLE is good and both ends are bad.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="67" t="inlineStr">
         <is>
-          <t>Axis</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="B6" s="67" t="inlineStr">
         <is>
-          <t>Members (illustrative — Components fill these)</t>
+          <t>Pushed by (Dimension)</t>
         </is>
       </c>
       <c r="C6" s="67" t="inlineStr">
         <is>
-          <t>Genuinely exclusive?</t>
+          <t>Bands, max -&gt; 0</t>
         </is>
       </c>
       <c r="D6" s="67" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Carried by</t>
         </is>
       </c>
       <c r="E6" s="67" t="inlineStr">
         <is>
-          <t>Precedent</t>
+          <t>Payable?</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="68" t="inlineStr">
         <is>
-          <t>poisoned</t>
+          <t>prone</t>
         </is>
       </c>
       <c r="B7" s="68" t="inlineStr">
@@ -15399,279 +15128,491 @@
       </c>
       <c r="C7" s="68" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="68" t="inlineStr">
+        <is>
+          <t>NOT A TRACK. "Prone" is a BAND on mobility. There is no prone State.</t>
+        </is>
+      </c>
+      <c r="F7" s="69" t="inlineStr">
+        <is>
+          <t>← example, not data</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>vitality</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
+        <is>
+          <t>vitality · integrity</t>
+        </is>
+      </c>
+      <c r="C8" s="76" t="inlineStr">
+        <is>
+          <t>hale · hurt · wounded · grave · dying</t>
+        </is>
+      </c>
+      <c r="D8" s="76" t="inlineStr">
+        <is>
+          <t>Creature · Group (cohesion)</t>
+        </is>
+      </c>
+      <c r="E8" s="76" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="D7" s="68" t="inlineStr">
-        <is>
-          <t>NOT an axis — you can be poisoned and prone and blind. That is a State on its own axis, or a Resource.</t>
-        </is>
-      </c>
-      <c r="E7" s="68" t="inlineStr">
-        <is>
-          <t>5e poisoned</t>
-        </is>
-      </c>
-      <c r="F7" s="69" t="inlineStr">
-        <is>
-          <t>← example, not data</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="70" t="inlineStr">
-        <is>
-          <t>posture</t>
-        </is>
-      </c>
-      <c r="B8" s="70" t="inlineStr">
-        <is>
-          <t>standing · prone · seated · airborne</t>
-        </is>
-      </c>
-      <c r="C8" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D8" s="70" t="inlineStr">
-        <is>
-          <t>You cannot be both prone and airborne</t>
-        </is>
-      </c>
-      <c r="E8" s="70" t="inlineStr">
-        <is>
-          <t>5e prone · WFRP Prone</t>
-        </is>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="70" t="inlineStr">
-        <is>
-          <t>restraint</t>
-        </is>
-      </c>
-      <c r="B9" s="70" t="inlineStr">
-        <is>
-          <t>free · grabbed · restrained · immobilised</t>
-        </is>
-      </c>
-      <c r="C9" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D9" s="70" t="inlineStr">
-        <is>
-          <t>PF2e and 5e both treat these as a ladder</t>
-        </is>
-      </c>
-      <c r="E9" s="70" t="inlineStr">
-        <is>
-          <t>5e grappled/restrained · Lancer Immobilized</t>
+      <c r="A9" s="76" t="inlineStr">
+        <is>
+          <t>vigor</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>vigor · temperature (extremes)</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>fresh · tired · weary · spent · collapsed</t>
+        </is>
+      </c>
+      <c r="D9" s="76" t="inlineStr">
+        <is>
+          <t>Creature · Phenomenon (its fuel)</t>
+        </is>
+      </c>
+      <c r="E9" s="76" t="inlineStr">
+        <is>
+          <t>maybe</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="70" t="inlineStr">
-        <is>
-          <t>consciousness</t>
-        </is>
-      </c>
-      <c r="B10" s="70" t="inlineStr">
-        <is>
-          <t>awake · asleep · unconscious</t>
-        </is>
-      </c>
-      <c r="C10" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D10" s="70" t="inlineStr"/>
-      <c r="E10" s="70" t="inlineStr">
-        <is>
-          <t>5e unconscious · WFRP</t>
+      <c r="A10" s="76" t="inlineStr">
+        <is>
+          <t>mobility</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>mobility</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>free · slowed · hobbled · pinned · immobile</t>
+        </is>
+      </c>
+      <c r="D10" s="76" t="inlineStr">
+        <is>
+          <t>Creature</t>
+        </is>
+      </c>
+      <c r="E10" s="76" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="70" t="inlineStr">
-        <is>
-          <t>awareness</t>
-        </is>
-      </c>
-      <c r="B11" s="70" t="inlineStr">
-        <is>
-          <t>aware · surprised · unaware</t>
-        </is>
-      </c>
-      <c r="C11" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D11" s="70" t="inlineStr"/>
-      <c r="E11" s="70" t="inlineStr">
-        <is>
-          <t>5e surprised · PF2e</t>
+      <c r="A11" s="76" t="inlineStr">
+        <is>
+          <t>acuity</t>
+        </is>
+      </c>
+      <c r="B11" s="76" t="inlineStr">
+        <is>
+          <t>acuity</t>
+        </is>
+      </c>
+      <c r="C11" s="76" t="inlineStr">
+        <is>
+          <t>sharp · dulled · clouded · blind</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr">
+        <is>
+          <t>Creature</t>
+        </is>
+      </c>
+      <c r="E11" s="76" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="70" t="inlineStr">
-        <is>
-          <t>visibility</t>
-        </is>
-      </c>
-      <c r="B12" s="70" t="inlineStr">
-        <is>
-          <t>seen · concealed · hidden · unseen</t>
-        </is>
-      </c>
-      <c r="C12" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D12" s="70" t="inlineStr">
-        <is>
-          <t>PF2e's four-step ladder is the best-specified version in print</t>
-        </is>
-      </c>
-      <c r="E12" s="70" t="inlineStr">
-        <is>
-          <t>PF2e concealed/hidden/undetected</t>
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>integrity</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>integrity · substance · temperature</t>
+        </is>
+      </c>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>intact · marred · damaged · failing · ruined</t>
+        </is>
+      </c>
+      <c r="D12" s="76" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E12" s="76" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="70" t="inlineStr">
-        <is>
-          <t>animacy</t>
-        </is>
-      </c>
-      <c r="B13" s="70" t="inlineStr">
-        <is>
-          <t>living · dying · dead</t>
-        </is>
-      </c>
-      <c r="C13" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D13" s="70" t="inlineStr">
-        <is>
-          <t>PF2e dying/wounded is really a track, not a condition — watch for that</t>
-        </is>
-      </c>
-      <c r="E13" s="70" t="inlineStr">
-        <is>
-          <t>PF2e dying + wounded</t>
+      <c r="A13" s="76" t="inlineStr">
+        <is>
+          <t>substance</t>
+        </is>
+      </c>
+      <c r="B13" s="76" t="inlineStr">
+        <is>
+          <t>substance</t>
+        </is>
+      </c>
+      <c r="C13" s="76" t="inlineStr">
+        <is>
+          <t>whole · pitted · eaten · consumed</t>
+        </is>
+      </c>
+      <c r="D13" s="76" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E13" s="76" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="70" t="inlineStr">
-        <is>
-          <t>containment</t>
-        </is>
-      </c>
-      <c r="B14" s="70" t="inlineStr">
-        <is>
-          <t>free · contained · submerged</t>
-        </is>
-      </c>
-      <c r="C14" s="70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="D14" s="70" t="inlineStr">
-        <is>
-          <t>Overlaps Place; argue whether it belongs to the Place Socket instead</t>
-        </is>
-      </c>
-      <c r="E14" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="A14" s="76" t="inlineStr">
+        <is>
+          <t>composure</t>
+        </is>
+      </c>
+      <c r="B14" s="76" t="inlineStr">
+        <is>
+          <t>composure</t>
+        </is>
+      </c>
+      <c r="C14" s="76" t="inlineStr">
+        <is>
+          <t>steady · rattled · shaken · panicked · broken</t>
+        </is>
+      </c>
+      <c r="D14" s="76" t="inlineStr">
+        <is>
+          <t>Creature</t>
+        </is>
+      </c>
+      <c r="E14" s="76" t="inlineStr">
+        <is>
+          <t>maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="76" t="inlineStr">
+        <is>
+          <t>clarity</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>clarity</t>
+        </is>
+      </c>
+      <c r="C15" s="76" t="inlineStr">
+        <is>
+          <t>lucid · muddled · confused · senseless</t>
+        </is>
+      </c>
+      <c r="D15" s="76" t="inlineStr">
+        <is>
+          <t>Creature</t>
+        </is>
+      </c>
+      <c r="E15" s="76" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="70" t="inlineStr">
-        <is>
-          <t>FIELDS A STATE DEFINITION CARRIES: name · axis · optional magnitude · optional MAXIMUM · what it does · how it ends. FORGETTING THE MAX IS THE MISTAKE — values add by default, so without a ceiling "poisoned 47" is reachable.</t>
+      <c r="A16" s="76" t="inlineStr">
+        <is>
+          <t>will</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>will</t>
+        </is>
+      </c>
+      <c r="C16" s="76" t="inlineStr">
+        <is>
+          <t>resolute · wavering · yielding · dominated</t>
+        </is>
+      </c>
+      <c r="D16" s="76" t="inlineStr">
+        <is>
+          <t>Creature</t>
+        </is>
+      </c>
+      <c r="E16" s="76" t="inlineStr">
+        <is>
+          <t>maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="76" t="inlineStr">
+        <is>
+          <t>standing</t>
+        </is>
+      </c>
+      <c r="B17" s="76" t="inlineStr">
+        <is>
+          <t>standing</t>
+        </is>
+      </c>
+      <c r="C17" s="76" t="inlineStr">
+        <is>
+          <t>renowned · respected · known · disregarded · disgraced</t>
+        </is>
+      </c>
+      <c r="D17" s="76" t="inlineStr">
+        <is>
+          <t>Group · Notion (how believed)</t>
+        </is>
+      </c>
+      <c r="E17" s="76" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="71" t="inlineStr">
+      <c r="A18" s="76" t="inlineStr">
+        <is>
+          <t>regard</t>
+        </is>
+      </c>
+      <c r="B18" s="76" t="inlineStr">
+        <is>
+          <t>regard</t>
+        </is>
+      </c>
+      <c r="C18" s="76" t="inlineStr">
+        <is>
+          <t>devoted · warm · civil · cool · hostile</t>
+        </is>
+      </c>
+      <c r="D18" s="76" t="inlineStr">
+        <is>
+          <t>HELD ON A CONNECTION, never on the target</t>
+        </is>
+      </c>
+      <c r="E18" s="76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="76" t="inlineStr">
+        <is>
+          <t>essence</t>
+        </is>
+      </c>
+      <c r="B19" s="76" t="inlineStr">
+        <is>
+          <t>essence</t>
+        </is>
+      </c>
+      <c r="C19" s="76" t="inlineStr">
+        <is>
+          <t>whole · thinned · frayed · hollow</t>
+        </is>
+      </c>
+      <c r="D19" s="76" t="inlineStr">
+        <is>
+          <t>Creature (mystic Settings)</t>
+        </is>
+      </c>
+      <c r="E19" s="76" t="inlineStr">
+        <is>
+          <t>maybe</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="76" t="inlineStr">
+        <is>
+          <t>temperature  ** BIPOLAR **</t>
+        </is>
+      </c>
+      <c r="B20" s="76" t="inlineStr">
+        <is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="C20" s="76" t="inlineStr">
+        <is>
+          <t>scorched · seared · hot · TEMPERATE · cold · chilled · frozen</t>
+        </is>
+      </c>
+      <c r="D20" s="76" t="inlineStr">
+        <is>
+          <t>Creature · Item · Place</t>
+        </is>
+      </c>
+      <c r="E20" s="76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="76" t="inlineStr">
+        <is>
+          <t>working  ** BIPOLAR **</t>
+        </is>
+      </c>
+      <c r="B21" s="76" t="inlineStr">
+        <is>
+          <t>working</t>
+        </is>
+      </c>
+      <c r="C21" s="76" t="inlineStr">
+        <is>
+          <t>surging · charged · QUIET · dampened · sealed</t>
+        </is>
+      </c>
+      <c r="D21" s="76" t="inlineStr">
+        <is>
+          <t>Creature · Phenomenon (if magical)</t>
+        </is>
+      </c>
+      <c r="E21" s="76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="76" t="inlineStr">
+        <is>
+          <t>EVERY DIMENSION PUSHES AT LEAST ONE TRACK — a CI invariant, not a coincidence. A Dimension with nothing to land on is a dead axis, which is the failure that leaves a quarter of a published bestiary immune to poison and nothing at all resisting force. BANDS ARE RULESET CONTENT; Tracks and Thresholds are Substrate. A Setting may band and name differently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="71" t="inlineStr">
         <is>
           <t>CONSIDERED AND REJECTED</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="72" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>posture · awareness · consciousness · access · spread · intensity</t>
+        </is>
+      </c>
+      <c r="B26" s="72" t="inlineStr"/>
+      <c r="C26" s="72" t="inlineStr"/>
+      <c r="D26" s="72" t="inlineStr"/>
+      <c r="E26" s="72" t="inlineStr">
+        <is>
+          <t>COLLAPSED. Each was an invented axis that turns out to be a band on a Dimension Track. Posture is low mobility — being knocked down IS a mobility push, and standing up is a Verb that restores it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="72" t="inlineStr">
+        <is>
+          <t>enumerated members (standing / prone / seated)</t>
+        </is>
+      </c>
+      <c r="B27" s="72" t="inlineStr"/>
+      <c r="C27" s="72" t="inlineStr"/>
+      <c r="D27" s="72" t="inlineStr"/>
+      <c r="E27" s="72" t="inlineStr">
+        <is>
+          <t>REJECTED. A State is a MAGNITUDE. The named condition is a label on a range of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="72" t="inlineStr">
         <is>
           <t>additive magnitudes</t>
         </is>
       </c>
-      <c r="B19" s="72" t="inlineStr"/>
-      <c r="C19" s="72" t="inlineStr"/>
-      <c r="D19" s="72" t="inlineStr">
-        <is>
-          <t>REJECT. PF2e takes the HIGHER value when a numeric condition is applied twice, never the sum. Additive stacking makes any repeatable source unbounded. This settles L18: the operator for States is max.</t>
-        </is>
-      </c>
-      <c r="E19" s="72" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="72" t="inlineStr">
+      <c r="B28" s="72" t="inlineStr"/>
+      <c r="C28" s="72" t="inlineStr"/>
+      <c r="D28" s="72" t="inlineStr"/>
+      <c r="E28" s="72" t="inlineStr">
+        <is>
+          <t>REJECTED — a Track CLAMPS to its bounds. Additive stacking makes any repeatable source unbounded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="72" t="inlineStr">
         <is>
           <t>conditions that imply other conditions</t>
         </is>
       </c>
-      <c r="B20" s="72" t="inlineStr"/>
-      <c r="C20" s="72" t="inlineStr"/>
-      <c r="D20" s="72" t="inlineStr">
-        <is>
-          <t>REJECT, and it is a live maintenance cost in a shipping product: 5e paralyzed/stunned/unconscious all include incapacitated, and the 2024 revision had to widen incapacitated, which cascaded to all three. Same failure as tag hierarchy.</t>
-        </is>
-      </c>
-      <c r="E20" s="72" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="72" t="inlineStr">
+      <c r="B29" s="72" t="inlineStr"/>
+      <c r="C29" s="72" t="inlineStr"/>
+      <c r="D29" s="72" t="inlineStr"/>
+      <c r="E29" s="72" t="inlineStr">
+        <is>
+          <t>REJECTED. Same failure as tag hierarchy — 5e paralyzed/stunned/unconscious all include incapacitated, and the 2024 revision had to widen incapacitated, cascading to all three.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="72" t="inlineStr">
         <is>
           <t>intrinsic durations (save-ends, N rounds)</t>
         </is>
       </c>
-      <c r="B21" s="72" t="inlineStr"/>
-      <c r="C21" s="72" t="inlineStr"/>
-      <c r="D21" s="72" t="inlineStr">
-        <is>
-          <t>ARGUE. 5e conditions have NO intrinsic duration — they end because the effect that imposed them ends, or a named action ends them. That is already our design, validated at the largest scale in the hobby. 4e layered durations on top and the tracking load is its most-cited failure.</t>
-        </is>
-      </c>
-      <c r="E21" s="72" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="72" t="inlineStr">
-        <is>
-          <t>a long condition list</t>
-        </is>
-      </c>
-      <c r="B22" s="72" t="inlineStr"/>
-      <c r="C22" s="72" t="inlineStr"/>
-      <c r="D22" s="72" t="inlineStr">
-        <is>
-          <t>3e/PF1 carried 34+. 4e carried more. 5e cut to 15. NOBODY HAS GROWN A CONDITION LIST AND BEEN GLAD.</t>
-        </is>
-      </c>
-      <c r="E22" s="72" t="inlineStr"/>
+      <c r="B30" s="72" t="inlineStr"/>
+      <c r="C30" s="72" t="inlineStr"/>
+      <c r="D30" s="72" t="inlineStr"/>
+      <c r="E30" s="72" t="inlineStr">
+        <is>
+          <t>REJECTED. A Track changes only by a Verb. 5e conditions have no intrinsic duration either, and it is the most-played RPG in the world.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
L25 Landing and L7 Layers settled; M- and X- regions added
</commit_message>
<xml_diff>
--- a/docs/substrate-lists.xlsx
+++ b/docs/substrate-lists.xlsx
@@ -7555,21 +7555,21 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="19">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="73" t="inlineStr">
         <is>
           <t>L4 · Core Tag vocabulary</t>
         </is>
       </c>
-      <c r="B8" s="30" t="inlineStr">
-        <is>
-          <t>PENDING · BLOCKING</t>
-        </is>
-      </c>
-      <c r="C8" s="26">
+      <c r="B8" s="74" t="inlineStr">
+        <is>
+          <t>PROVISIONAL · 22 chosen</t>
+        </is>
+      </c>
+      <c r="C8" s="73">
         <f>COUNTA('L4 Core Tag vocabulary'!A8:A47)</f>
         <v/>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="73">
         <f>IF(C8&gt;0,"started","not started")</f>
         <v/>
       </c>
@@ -7615,21 +7615,21 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="19">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="73" t="inlineStr">
         <is>
           <t>L7 · Layers</t>
         </is>
       </c>
-      <c r="B11" s="30" t="inlineStr">
-        <is>
-          <t>PARTIAL · BLOCKING</t>
-        </is>
-      </c>
-      <c r="C11" s="26">
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="73">
         <f>COUNTA('L7 Layers'!A8:A47)</f>
         <v/>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="73">
         <f>IF(C11&gt;0,"started","not started")</f>
         <v/>
       </c>
@@ -7855,21 +7855,21 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="19">
-      <c r="A23" s="26" t="inlineStr">
-        <is>
-          <t>L25 · Transient-to-Persistent conversions</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="inlineStr">
-        <is>
-          <t>PENDING · BLOCKING</t>
-        </is>
-      </c>
-      <c r="C23" s="26">
+      <c r="A23" s="73" t="inlineStr">
+        <is>
+          <t>L25 · Landing</t>
+        </is>
+      </c>
+      <c r="B23" s="74" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+      <c r="C23" s="73">
         <f>COUNTA('L25 Transient-to-Persistent con'!A8:A47)</f>
         <v/>
       </c>
-      <c r="D23" s="26">
+      <c r="D23" s="73">
         <f>IF(C23&gt;0,"started","not started")</f>
         <v/>
       </c>
@@ -8651,41 +8651,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="19" min="1" max="1"/>
-    <col width="32" customWidth="1" style="19" min="2" max="2"/>
-    <col width="40" customWidth="1" style="19" min="3" max="3"/>
-    <col width="42" customWidth="1" style="19" min="4" max="4"/>
-    <col width="66" customWidth="1" style="19" min="5" max="5"/>
+    <col width="26" customWidth="1" style="19" min="1" max="1"/>
+    <col width="30" customWidth="1" style="19" min="2" max="2"/>
+    <col width="26" customWidth="1" style="19" min="3" max="3"/>
+    <col width="86" customWidth="1" style="19" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="63" t="inlineStr">
         <is>
-          <t>L25 · Transient-to-Persistent conversions</t>
+          <t>L25 · Landing</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="64" t="inlineStr">
         <is>
-          <t>PENDING · BLOCKING · research-seeded Aug 2026</t>
+          <t>SETTLED · Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="65" t="inlineStr">
         <is>
-          <t>What a vector that survives Guards actually does. This IS the Landing Socket Vocabulary. Fourteen rows, one per non-attempt Dimension.</t>
+          <t>What a vector that survives Guards actually does. This IS the Landing Socket Vocabulary.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="66" t="inlineStr">
         <is>
-          <t>THE UNIVERSAL ARCHITECTURE IS BUFFER → CONVERT → NAME. Fate, Blades, Lancer, Delta Green, Mouse Guard all do it. So Landing is a PIPELINE SHAPE, not one step — and the buffer belongs to the Component, never the Substrate.</t>
+          <t>DEFAULT LANDING IS ONE LINE: subtract the resolved value from the Track the Dimension names, clamped to its bounds. Three of the eleven landing models researched (pool / track / bar-and-name) are ALL JUST A TRACK.</t>
         </is>
       </c>
     </row>
@@ -8697,22 +8696,17 @@
       </c>
       <c r="B6" s="67" t="inlineStr">
         <is>
-          <t>Proposed landing model</t>
+          <t>Lands on</t>
         </is>
       </c>
       <c r="C6" s="67" t="inlineStr">
         <is>
-          <t>What it means</t>
+          <t>Restores</t>
         </is>
       </c>
       <c r="D6" s="67" t="inlineStr">
         <is>
-          <t>Precedent</t>
-        </is>
-      </c>
-      <c r="E6" s="67" t="inlineStr">
-        <is>
-          <t>Notes and hazards</t>
+          <t>Special</t>
         </is>
       </c>
     </row>
@@ -8724,412 +8718,325 @@
       </c>
       <c r="B7" s="68" t="inlineStr">
         <is>
-          <t>L1 deplete a pool</t>
+          <t>a pool</t>
         </is>
       </c>
       <c r="C7" s="68" t="inlineStr">
         <is>
-          <t>subtract and check zero</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D7" s="68" t="inlineStr">
         <is>
-          <t>D&amp;D</t>
-        </is>
-      </c>
-      <c r="E7" s="68" t="inlineStr">
-        <is>
-          <t>NOT assumed. The Substrate ships no Resources; a Setting may legitimately have none. Masks and Mouse Guard are shipping proof.</t>
-        </is>
-      </c>
-      <c r="F7" s="69" t="inlineStr">
+          <t>NOT assumed. A Setting may ship NO Tracks at all — Masks has five conditions and no numbers; Mouse Guard has six. Both are shipping proof.</t>
+        </is>
+      </c>
+      <c r="E7" s="69" t="inlineStr">
         <is>
           <t>← example, not data</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="70" t="inlineStr">
-        <is>
-          <t>temperature (bipolar)</t>
-        </is>
-      </c>
-      <c r="B8" s="70" t="inlineStr">
-        <is>
-          <t>L11 bank + L6 convert</t>
-        </is>
-      </c>
-      <c r="C8" s="70" t="inlineStr">
-        <is>
-          <t>Accumulate a signed heat value; discharge at a bar</t>
-        </is>
-      </c>
-      <c r="D8" s="70" t="inlineStr">
-        <is>
-          <t>Lancer Heat · WFRP Ablaze · Rolemaster Heat/Cold tables</t>
-        </is>
-      </c>
-      <c r="E8" s="70" t="inlineStr">
-        <is>
-          <t>BIPOLAR needs TWO bars, one per sign. No complete precedent exists — Lancer only implements the hot end.</t>
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>vitality</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
+        <is>
+          <t>vitality</t>
+        </is>
+      </c>
+      <c r="C8" s="76" t="inlineStr">
+        <is>
+          <t>assisted</t>
+        </is>
+      </c>
+      <c r="D8" s="76" t="inlineStr">
+        <is>
+          <t>At zero the Setting decides — death, dying, or a Threshold to something else.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="70" t="inlineStr">
+      <c r="A9" s="76" t="inlineStr">
+        <is>
+          <t>vigor</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>vigor</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>naturally</t>
+        </is>
+      </c>
+      <c r="D9" s="76" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="76" t="inlineStr">
+        <is>
+          <t>mobility</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>mobility</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>naturally, and by a Verb</t>
+        </is>
+      </c>
+      <c r="D10" s="76" t="inlineStr">
+        <is>
+          <t>Standing up is a VERB, not a timer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="76" t="inlineStr">
+        <is>
+          <t>acuity</t>
+        </is>
+      </c>
+      <c r="B11" s="76" t="inlineStr">
+        <is>
+          <t>acuity</t>
+        </is>
+      </c>
+      <c r="C11" s="76" t="inlineStr">
+        <is>
+          <t>naturally</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="76" t="inlineStr">
         <is>
           <t>integrity</t>
         </is>
       </c>
-      <c r="B9" s="70" t="inlineStr">
-        <is>
-          <t>L1 pool + L6 convert at zero</t>
-        </is>
-      </c>
-      <c r="C9" s="70" t="inlineStr">
-        <is>
-          <t>Pool is a DISPOSABLE buffer; its only durable effect is the conversion</t>
-        </is>
-      </c>
-      <c r="D9" s="70" t="inlineStr">
-        <is>
-          <t>Lancer HP→Structure (HP resets to full) · Mörk Borg 0 HP→d4 Broken</t>
-        </is>
-      </c>
-      <c r="E9" s="70" t="inlineStr">
-        <is>
-          <t>The buffer is not durable state and should not survive a Moment as a Facet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="70" t="inlineStr">
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>integrity</t>
+        </is>
+      </c>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>ONLY BY REPAIR</t>
+        </is>
+      </c>
+      <c r="D12" s="76" t="inlineStr">
+        <is>
+          <t>At zero, Item typically converts to a destroyed band.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="76" t="inlineStr">
         <is>
           <t>substance</t>
         </is>
       </c>
-      <c r="B10" s="70" t="inlineStr">
-        <is>
-          <t>L8 permanent scalar edit</t>
-        </is>
-      </c>
-      <c r="C10" s="70" t="inlineStr">
-        <is>
-          <t>Matter removed is matter gone; no recovery without an explicit Verb</t>
-        </is>
-      </c>
-      <c r="D10" s="70" t="inlineStr">
-        <is>
-          <t>Twilight 2000 attribute loss · GURPS DR degradation</t>
-        </is>
-      </c>
-      <c r="E10" s="70" t="inlineStr">
-        <is>
-          <t>Needs an explicit restoration path — L8 has no natural inverse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="70" t="inlineStr">
-        <is>
-          <t>vitality</t>
-        </is>
-      </c>
-      <c r="B11" s="70" t="inlineStr">
-        <is>
-          <t>L3 bar → named condition, read HIGHEST</t>
-        </is>
-      </c>
-      <c r="C11" s="70" t="inlineStr">
-        <is>
-          <t>A single blow's magnitude, not the sum, decides the wound</t>
-        </is>
-      </c>
-      <c r="D11" s="70" t="inlineStr">
-        <is>
-          <t>GURPS major wound (&gt;HP/2) · Mythras Serious/Major · Ars Magica</t>
-        </is>
-      </c>
-      <c r="E11" s="70" t="inlineStr">
-        <is>
-          <t>Reading HIGHEST *is* the all-in incentive. Pair with a residue accumulator or small hits are worthless.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="70" t="inlineStr">
-        <is>
-          <t>vigor</t>
-        </is>
-      </c>
-      <c r="B12" s="70" t="inlineStr">
-        <is>
-          <t>L2 track, non-linear boxes</t>
-        </is>
-      </c>
-      <c r="C12" s="70" t="inlineStr">
-        <is>
-          <t>Fatigue is the archetypal graded track</t>
-        </is>
-      </c>
-      <c r="D12" s="70" t="inlineStr">
-        <is>
-          <t>5e exhaustion · GURPS FP · Ars Magica Fatigue</t>
-        </is>
-      </c>
-      <c r="E12" s="70" t="inlineStr">
-        <is>
-          <t>Non-linear box counts per severity stop minor harm accumulating at the same rate as major.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="70" t="inlineStr">
-        <is>
-          <t>mobility</t>
-        </is>
-      </c>
-      <c r="B13" s="70" t="inlineStr">
-        <is>
-          <t>L3 bar → condition, exclusive within an axis</t>
-        </is>
-      </c>
-      <c r="C13" s="70" t="inlineStr">
-        <is>
-          <t>Below the bar, nothing</t>
-        </is>
-      </c>
-      <c r="D13" s="70" t="inlineStr">
-        <is>
-          <t>WFRP Prone/Entangled · Lancer Immobilized/Slowed</t>
-        </is>
-      </c>
-      <c r="E13" s="70" t="inlineStr">
-        <is>
-          <t>Nothing in the field uses an ablative pool for a CAPABILITY axis — 4 of 7 movement is meaningless.</t>
+      <c r="B13" s="76" t="inlineStr">
+        <is>
+          <t>substance</t>
+        </is>
+      </c>
+      <c r="C13" s="76" t="inlineStr">
+        <is>
+          <t>NEVER</t>
+        </is>
+      </c>
+      <c r="D13" s="76" t="inlineStr">
+        <is>
+          <t>Matter removed is gone. Needs an explicit restoration Verb.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="70" t="inlineStr">
-        <is>
-          <t>acuity</t>
-        </is>
-      </c>
-      <c r="B14" s="70" t="inlineStr">
-        <is>
-          <t>L3 bar → named condition</t>
-        </is>
-      </c>
-      <c r="C14" s="70" t="inlineStr">
-        <is>
-          <t>Optionally L7 table to pick which sense</t>
-        </is>
-      </c>
-      <c r="D14" s="70" t="inlineStr">
-        <is>
-          <t>WFRP Blinded/Deafened · GURPS stunning</t>
-        </is>
-      </c>
-      <c r="E14" s="70" t="inlineStr">
-        <is>
-          <t>Same capability-axis argument as mobility.</t>
+      <c r="A14" s="76" t="inlineStr">
+        <is>
+          <t>composure</t>
+        </is>
+      </c>
+      <c r="B14" s="76" t="inlineStr">
+        <is>
+          <t>composure</t>
+        </is>
+      </c>
+      <c r="C14" s="76" t="inlineStr">
+        <is>
+          <t>naturally, fast</t>
+        </is>
+      </c>
+      <c r="D14" s="76" t="inlineStr">
+        <is>
+          <t>The buffer-like axis — empties and refills within a scene.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="70" t="inlineStr">
-        <is>
-          <t>composure</t>
-        </is>
-      </c>
-      <c r="B15" s="70" t="inlineStr">
-        <is>
-          <t>L0 buffer + L6 convert at the cap</t>
-        </is>
-      </c>
-      <c r="C15" s="70" t="inlineStr">
-        <is>
-          <t>An evaporating in-scene buffer, then a named durable thing</t>
-        </is>
-      </c>
-      <c r="D15" s="70" t="inlineStr">
-        <is>
-          <t>Blades stress 0–9 → Trauma · Fate mental stress → consequence</t>
-        </is>
-      </c>
-      <c r="E15" s="70" t="inlineStr">
-        <is>
-          <t>The buffer belongs to the Landing Component, never the Substrate.</t>
-        </is>
-      </c>
+      <c r="A15" s="76" t="inlineStr">
+        <is>
+          <t>clarity</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>clarity</t>
+        </is>
+      </c>
+      <c r="C15" s="76" t="inlineStr">
+        <is>
+          <t>naturally</t>
+        </is>
+      </c>
+      <c r="D15" s="76" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="70" t="inlineStr">
-        <is>
-          <t>clarity</t>
-        </is>
-      </c>
-      <c r="B16" s="70" t="inlineStr">
-        <is>
-          <t>L3 MOVING bar + L7 table draw</t>
-        </is>
-      </c>
-      <c r="C16" s="70" t="inlineStr">
-        <is>
-          <t>The bar itself moves after each crossing</t>
-        </is>
-      </c>
-      <c r="D16" s="70" t="inlineStr">
-        <is>
-          <t>Delta Green Breaking Point (resets to new SAN − POW) · CoC</t>
-        </is>
-      </c>
-      <c r="E16" s="70" t="inlineStr">
-        <is>
-          <t>A MOVING bar is the best mechanism found for having thresholds without the all-in incentive.</t>
+      <c r="A16" s="76" t="inlineStr">
+        <is>
+          <t>will</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>will</t>
+        </is>
+      </c>
+      <c r="C16" s="76" t="inlineStr">
+        <is>
+          <t>naturally</t>
+        </is>
+      </c>
+      <c r="D16" s="76" t="inlineStr">
+        <is>
+          <t>HARDEN. Resisting notches a counter making future resistance easier; failing notches the other way. THE ONE GENUINELY NEW MECHANISM — no physical system makes you harder to injure by injuring you; every serious mental system does (Unknown Armies, Delta Green, CoC).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="70" t="inlineStr">
-        <is>
-          <t>will</t>
-        </is>
-      </c>
-      <c r="B17" s="70" t="inlineStr">
-        <is>
-          <t>L9 HARDEN + L3 bar</t>
-        </is>
-      </c>
-      <c r="C17" s="70" t="inlineStr">
-        <is>
-          <t>Resisting notches you toward immunity; failing notches you toward collapse</t>
-        </is>
-      </c>
-      <c r="D17" s="70" t="inlineStr">
-        <is>
-          <t>Unknown Armies hardened/failed notches · DG Adaptation</t>
-        </is>
-      </c>
-      <c r="E17" s="70" t="inlineStr">
-        <is>
-          <t>The mental block wants a two-signed axis the physical block does not. No physical system makes you harder to injure by injuring you; every serious mental system does.</t>
+      <c r="A17" s="76" t="inlineStr">
+        <is>
+          <t>standing</t>
+        </is>
+      </c>
+      <c r="B17" s="76" t="inlineStr">
+        <is>
+          <t>standing</t>
+        </is>
+      </c>
+      <c r="C17" s="76" t="inlineStr">
+        <is>
+          <t>NEVER on its own</t>
+        </is>
+      </c>
+      <c r="D17" s="76" t="inlineStr">
+        <is>
+          <t>Eroded only by GROWING A DIFFERENT REPUTATION — the Ars Magica rule.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="70" t="inlineStr">
+      <c r="A18" s="76" t="inlineStr">
         <is>
           <t>regard</t>
         </is>
       </c>
-      <c r="B18" s="70" t="inlineStr">
-        <is>
-          <t>L10 land on a CONNECTION</t>
-        </is>
-      </c>
-      <c r="C18" s="70" t="inlineStr">
-        <is>
-          <t>Never on the target Entity. Adjusts the HOLDER's stance, per participant</t>
-        </is>
-      </c>
-      <c r="D18" s="70" t="inlineStr">
-        <is>
-          <t>Exalted 3e Intimacies · Delta Green Bonds</t>
-        </is>
-      </c>
-      <c r="E18" s="70" t="inlineStr">
-        <is>
-          <t>Exalted: nothing is possible without exploiting an Intimacy. Landing must be able to REJECT a packet for lack of a Connection — and the rejection must be a Record, not a silent drop.</t>
+      <c r="B18" s="76" t="inlineStr">
+        <is>
+          <t>regard, ON A CONNECTION</t>
+        </is>
+      </c>
+      <c r="C18" s="76" t="inlineStr">
+        <is>
+          <t>never on its own</t>
+        </is>
+      </c>
+      <c r="D18" s="76" t="inlineStr">
+        <is>
+          <t>LANDS ON THE HOLDER'S CONNECTION, never on the target. If no Connection exists the packet is REJECTED and the rejection is a RECORD.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="70" t="inlineStr">
-        <is>
-          <t>standing</t>
-        </is>
-      </c>
-      <c r="B19" s="70" t="inlineStr">
-        <is>
-          <t>L11 bank and discharge</t>
-        </is>
-      </c>
-      <c r="C19" s="70" t="inlineStr">
-        <is>
-          <t>Accumulate; convert at a bar into a discrete level; carry the remainder</t>
-        </is>
-      </c>
-      <c r="D19" s="70" t="inlineStr">
-        <is>
-          <t>Ars Magica Reputation (10 pts = +1 level) · Blades Heat→Wanted</t>
-        </is>
-      </c>
-      <c r="E19" s="70" t="inlineStr">
-        <is>
-          <t>Ars Magica: a bad reputation is eroded only by growing a good one, never by subtraction.</t>
+      <c r="A19" s="76" t="inlineStr">
+        <is>
+          <t>essence</t>
+        </is>
+      </c>
+      <c r="B19" s="76" t="inlineStr">
+        <is>
+          <t>essence</t>
+        </is>
+      </c>
+      <c r="C19" s="76" t="inlineStr">
+        <is>
+          <t>NEVER</t>
+        </is>
+      </c>
+      <c r="D19" s="76" t="inlineStr">
+        <is>
+          <t>The axis that does not come back. A Setting that wants it to must supply a Verb.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="70" t="inlineStr">
-        <is>
-          <t>working (bipolar)</t>
-        </is>
-      </c>
-      <c r="B20" s="70" t="inlineStr">
-        <is>
-          <t>L11 bank, discharge at BOTH bars</t>
-        </is>
-      </c>
-      <c r="C20" s="70" t="inlineStr">
-        <is>
-          <t>Two bars, one per sign</t>
-        </is>
-      </c>
-      <c r="D20" s="70" t="inlineStr">
-        <is>
-          <t>Lancer Heat (one end only) · Ars Magica Twilight · Mage Paradox</t>
-        </is>
-      </c>
-      <c r="E20" s="70" t="inlineStr">
-        <is>
-          <t>No complete precedent. Expect to invent here.</t>
+      <c r="A20" s="76" t="inlineStr">
+        <is>
+          <t>temperature  BIPOLAR</t>
+        </is>
+      </c>
+      <c r="B20" s="76" t="inlineStr">
+        <is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="C20" s="76" t="inlineStr">
+        <is>
+          <t>naturally, toward the centre</t>
+        </is>
+      </c>
+      <c r="D20" s="76" t="inlineStr">
+        <is>
+          <t>Pushes move toward or away from temperate. Both ends have Thresholds.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="70" t="inlineStr">
-        <is>
-          <t>essence</t>
-        </is>
-      </c>
-      <c r="B21" s="70" t="inlineStr">
-        <is>
-          <t>L8 + L3 at zero</t>
-        </is>
-      </c>
-      <c r="C21" s="70" t="inlineStr">
-        <is>
-          <t>The axis you never get back</t>
-        </is>
-      </c>
-      <c r="D21" s="70" t="inlineStr">
-        <is>
-          <t>Ars Magica Warping · Vampire Humanity · DG POW loss</t>
-        </is>
-      </c>
-      <c r="E21" s="70" t="inlineStr">
-        <is>
-          <t>Needs an explicit restoration path.</t>
+      <c r="A21" s="76" t="inlineStr">
+        <is>
+          <t>working  BIPOLAR</t>
+        </is>
+      </c>
+      <c r="B21" s="76" t="inlineStr">
+        <is>
+          <t>working</t>
+        </is>
+      </c>
+      <c r="C21" s="76" t="inlineStr">
+        <is>
+          <t>naturally, toward the centre</t>
+        </is>
+      </c>
+      <c r="D21" s="76" t="inlineStr">
+        <is>
+          <t>Same shape.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="70" t="inlineStr">
-        <is>
-          <t>ELEVEN MODELS EXIST (see lists-research.md §4): L0 evaporate · L1 pool · L2 track · L3 bar→condition · L4 phrase in a graded slot · L5 clock · L6 convert to another axis · L7 table draw · L8 scalar edit · L9 harden · L10 land on a Relationship · L11 bank and discharge.</t>
+      <c r="A23" s="76" t="inlineStr">
+        <is>
+          <t>A TRACK HAS NO DEAD ZONE, AND THAT DISSOLVES THE FIELD'S WORST RECORDED PROBLEM. Bar-based landing is a magnitude-concentration incentive — Mythras ships 40 special effects and players use the three that shove one blow over a bar, because harm below the bar did NOTHING. Every point of a push moves a Track even when it does not change the band, so small hits accumulate. THE INCENTIVE RETURNS ONLY WHERE A THRESHOLD READS "highest" — still useful, now OPT-IN, and the Vocabulary must say so where an author reads it.</t>
         </is>
       </c>
     </row>
@@ -9143,49 +9050,42 @@
     <row r="26">
       <c r="A26" s="72" t="inlineStr">
         <is>
-          <t>ONE AXIS, TWO MODELS BY MAGNITUDE</t>
+          <t>a silent drop</t>
         </is>
       </c>
       <c r="B26" s="72" t="inlineStr"/>
       <c r="C26" s="72" t="inlineStr"/>
-      <c r="D26" s="72" t="inlineStr"/>
-      <c r="E26" s="72" t="inlineStr">
-        <is>
-          <t>THE HAZARD TO DECIDE. If vitality lands as a pool below a bar and a condition above it, the answer depends on HOW the total was assembled — which the packet no longer knows. Either Landing reads only the packet (one contributor-reading per Dimension) or it must be handed the contributor list, which is a SUBSTRATE FINDING. Lancer has an open issue on exactly this.</t>
+      <c r="D26" s="72" t="inlineStr">
+        <is>
+          <t>REJECTED. A packet with nowhere to go is a RECORD. "Nothing happened" must never be indistinguishable from a bug.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="72" t="inlineStr">
         <is>
-          <t>assume health</t>
+          <t>freeform phrase landing (Blades-style)</t>
         </is>
       </c>
       <c r="B27" s="72" t="inlineStr"/>
       <c r="C27" s="72" t="inlineStr"/>
-      <c r="D27" s="72" t="inlineStr"/>
-      <c r="E27" s="72" t="inlineStr">
-        <is>
-          <t>REJECT: the Substrate ships no Resources. Health is one answer among several.</t>
+      <c r="D27" s="72" t="inlineStr">
+        <is>
+          <t>AVAILABLE to a Landing occupant, but NOT the default: a phrase is not machine-readable, so the Fold cannot reason about it, and it requires a Person Decider (rule 21). A table draw can be Auto.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="72" t="inlineStr">
         <is>
-          <t>freeform phrase for everything</t>
+          <t>assume health</t>
         </is>
       </c>
       <c r="B28" s="72" t="inlineStr"/>
       <c r="C28" s="72" t="inlineStr"/>
       <c r="D28" s="72" t="inlineStr">
         <is>
-          <t>Blades harm</t>
-        </is>
-      </c>
-      <c r="E28" s="72" t="inlineStr">
-        <is>
-          <t>ARGUE: L4 is not machine-readable, so the Fold cannot reason about "Broken Leg". A phrase-returning Landing needs a Person Decider (rule 21); a table-returning one can be Auto.</t>
+          <t>REJECTED — the Substrate ships no Tracks. Health is one answer among several.</t>
         </is>
       </c>
     </row>
@@ -16011,542 +15911,530 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" style="18" min="1" max="1"/>
-    <col width="40" customWidth="1" style="18" min="2" max="2"/>
-    <col width="30" customWidth="1" style="18" min="3" max="3"/>
-    <col width="24" customWidth="1" style="18" min="4" max="4"/>
-    <col width="34" customWidth="1" style="18" min="5" max="5"/>
+    <col width="22" customWidth="1" style="19" min="1" max="1"/>
+    <col width="10" customWidth="1" style="19" min="2" max="2"/>
+    <col width="32" customWidth="1" style="19" min="3" max="3"/>
+    <col width="26" customWidth="1" style="19" min="4" max="4"/>
+    <col width="86" customWidth="1" style="19" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.35" customHeight="1" s="19">
-      <c r="A1" s="20" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="63" t="inlineStr">
         <is>
           <t>L7 · Layers</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="19">
-      <c r="A2" s="28" t="inlineStr">
-        <is>
-          <t>PARTIAL · BLOCKING</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1" s="19">
-      <c r="A3" s="21" t="inlineStr">
-        <is>
-          <t>The precedence lattice. Resolution region is drafted (E-/C-/R-). What is open is everything outside resolution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1" s="19">
-      <c r="A4" s="32" t="inlineStr">
-        <is>
-          <t>REVISED — the resolution region is now THIRTY slots (E×5, C×6, R×19) after Phase 0 and the L21–L23 work. What remains is everything OUTSIDE resolution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="19">
-      <c r="A6" s="33" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="64" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026 · five regions, 41 slots</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="65" t="inlineStr">
+        <is>
+          <t>The fixed precedence lattice. A Component never says "I modify speed" — it says "I modify speed at R-500."</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>EACH LAYER MAY DEPEND ONLY ON LAYERS BEFORE IT. Fixed and permanent, numbered with gaps of 100. AN UNUSED SLOT COSTS NOTHING; A MISSING ONE IS A FOUNDATION BREAK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="67" t="inlineStr">
         <is>
           <t>Slot</t>
         </is>
       </c>
-      <c r="B6" s="33" t="inlineStr">
+      <c r="B6" s="67" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="D6" s="33" t="inlineStr">
-        <is>
-          <t>What belongs here</t>
-        </is>
-      </c>
-      <c r="E6" s="33" t="inlineStr">
-        <is>
-          <t>May depend on (earlier slots only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="23.85" customHeight="1" s="19">
-      <c r="A7" s="34" t="inlineStr">
-        <is>
-          <t>R-400</t>
-        </is>
-      </c>
-      <c r="B7" s="34" t="inlineStr">
-        <is>
-          <t>Resolution</t>
-        </is>
-      </c>
-      <c r="C7" s="34" t="inlineStr">
-        <is>
-          <t>Apply percentage</t>
-        </is>
-      </c>
-      <c r="D7" s="34" t="inlineStr">
-        <is>
-          <t>The one multiplication; truncate toward zero</t>
-        </is>
-      </c>
-      <c r="E7" s="34" t="inlineStr">
-        <is>
-          <t>R-300, R-350</t>
-        </is>
-      </c>
-      <c r="F7" s="35" t="inlineStr">
+      <c r="C6" s="67" t="inlineStr">
+        <is>
+          <t>What belongs there</t>
+        </is>
+      </c>
+      <c r="D6" s="67" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E6" s="67" t="inlineStr">
+        <is>
+          <t>Why it is here</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="68" t="inlineStr">
+        <is>
+          <t>R-450</t>
+        </is>
+      </c>
+      <c r="B7" s="68" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C7" s="68" t="inlineStr">
+        <is>
+          <t>something between apply and absolutes</t>
+        </is>
+      </c>
+      <c r="D7" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="68" t="inlineStr">
+        <is>
+          <t>There is no R-450. Gaps exist so one CAN be inserted.</t>
+        </is>
+      </c>
+      <c r="F7" s="69" t="inlineStr">
         <is>
           <t>← example, not data</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="19">
-      <c r="A8" s="36" t="inlineStr">
-        <is>
-          <t>E-100 … E-500</t>
-        </is>
-      </c>
-      <c r="B8" s="36" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="C8" s="36" t="inlineStr">
-        <is>
-          <t>preparing an Entity</t>
-        </is>
-      </c>
-      <c r="D8" s="36" t="inlineStr">
-        <is>
-          <t>existence, Categories, its own numbers, its ceilings</t>
-        </is>
-      </c>
-      <c r="E8" s="36" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="19">
-      <c r="A9" s="36" t="inlineStr">
-        <is>
-          <t>C-100 … C-600</t>
-        </is>
-      </c>
-      <c r="B9" s="36" t="inlineStr">
-        <is>
-          <t>creation</t>
-        </is>
-      </c>
-      <c r="C9" s="36" t="inlineStr">
-        <is>
-          <t>creating a vector</t>
-        </is>
-      </c>
-      <c r="D9" s="36" t="inlineStr">
-        <is>
-          <t>everything the source contributes, collapsed to a direction and four numbers</t>
-        </is>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>E-region</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="19">
-      <c r="A10" s="36" t="inlineStr">
-        <is>
-          <t>R-100 … R-1400</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="inlineStr">
-        <is>
-          <t>resolution</t>
-        </is>
-      </c>
-      <c r="C10" s="36" t="inlineStr">
-        <is>
-          <t>resolving at a Moment</t>
-        </is>
-      </c>
-      <c r="D10" s="36" t="inlineStr">
-        <is>
-          <t>gather · ambient · percentages · capacity clamp · apply · absolutes · vector clamp · resolve · SCALE (R-750) · standing cap (R-780, reserved) · combine per source · FLAT GUARDS per source (R-850) · combine across sources (R-1000) · PROPORTIONAL GUARDS (R-1050) · target clamp · land · RESTORE (R-1250) · record · listeners</t>
-        </is>
-      </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>E and C regions</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="19">
-      <c r="A11" s="36" t="inlineStr"/>
-      <c r="B11" s="36" t="inlineStr"/>
-      <c r="C11" s="36" t="inlineStr"/>
-      <c r="D11" s="36" t="inlineStr"/>
-      <c r="E11" s="36" t="inlineStr"/>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="19">
-      <c r="A12" s="36" t="inlineStr">
-        <is>
-          <t>STILL EMPTY — the regions outside resolution:</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="inlineStr"/>
-      <c r="C12" s="36" t="inlineStr"/>
-      <c r="D12" s="36" t="inlineStr"/>
-      <c r="E12" s="36" t="inlineStr"/>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="19">
-      <c r="A13" s="36" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="inlineStr">
-        <is>
-          <t>progression</t>
-        </is>
-      </c>
-      <c r="C13" s="36" t="inlineStr">
-        <is>
-          <t>how a character changes over time</t>
-        </is>
-      </c>
-      <c r="D13" s="36" t="inlineStr"/>
-      <c r="E13" s="36" t="inlineStr">
-        <is>
-          <t>needs its own region</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="19">
-      <c r="A14" s="36" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="inlineStr">
-        <is>
-          <t>economy</t>
-        </is>
-      </c>
-      <c r="C14" s="36" t="inlineStr">
-        <is>
-          <t>Budget refresh, upkeep, costs</t>
-        </is>
-      </c>
-      <c r="D14" s="36" t="inlineStr"/>
-      <c r="E14" s="36" t="inlineStr">
-        <is>
-          <t>the A2 upkeep answer lives here</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="19">
-      <c r="A15" s="36" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="B15" s="36" t="inlineStr">
-        <is>
-          <t>movement</t>
-        </is>
-      </c>
-      <c r="C15" s="36" t="inlineStr">
-        <is>
-          <t>position, travel, pursuit</t>
-        </is>
-      </c>
-      <c r="D15" s="36" t="inlineStr"/>
-      <c r="E15" s="36" t="inlineStr">
-        <is>
-          <t>interacts with the new mobility Dimension</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="19">
-      <c r="A16" s="36" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="B16" s="36" t="inlineStr">
-        <is>
-          <t>knowledge</t>
-        </is>
-      </c>
-      <c r="C16" s="36" t="inlineStr">
-        <is>
-          <t>what is known, by whom, when</t>
-        </is>
-      </c>
-      <c r="D16" s="36" t="inlineStr"/>
-      <c r="E16" s="36" t="inlineStr">
-        <is>
-          <t>Almanac</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="19">
-      <c r="A17" s="36" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="B17" s="36" t="inlineStr">
-        <is>
-          <t>social standing</t>
-        </is>
-      </c>
-      <c r="C17" s="36" t="inlineStr">
-        <is>
-          <t>reputation over time, decay</t>
-        </is>
-      </c>
-      <c r="D17" s="36" t="inlineStr"/>
-      <c r="E17" s="36" t="inlineStr">
-        <is>
-          <t>interacts with the new standing Dimension</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="19">
-      <c r="A18" s="36" t="inlineStr"/>
-      <c r="B18" s="36" t="inlineStr"/>
-      <c r="C18" s="36" t="inlineStr"/>
-      <c r="D18" s="36" t="inlineStr"/>
-      <c r="E18" s="36" t="inlineStr"/>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="19">
-      <c r="A19" s="36" t="inlineStr">
-        <is>
-          <t>THE TEST: take a mechanic you want. Write out what must already be settled before it can be computed. If no existing slot supplies it, that is a new slot.</t>
-        </is>
-      </c>
-      <c r="B19" s="36" t="inlineStr"/>
-      <c r="C19" s="36" t="inlineStr"/>
-      <c r="D19" s="36" t="inlineStr"/>
-      <c r="E19" s="36" t="inlineStr"/>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="19">
-      <c r="A20" s="36" t="inlineStr">
-        <is>
-          <t>ERR HIGH. Gaps of 100 so 650 can be inserted. An unused slot costs nothing; a missing one is a foundation break.</t>
-        </is>
-      </c>
-      <c r="B20" s="36" t="inlineStr"/>
-      <c r="C20" s="36" t="inlineStr"/>
-      <c r="D20" s="36" t="inlineStr"/>
-      <c r="E20" s="36" t="inlineStr"/>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="19">
-      <c r="A21" s="37" t="n"/>
-      <c r="B21" s="37" t="n"/>
-      <c r="C21" s="37" t="n"/>
-      <c r="D21" s="37" t="n"/>
-      <c r="E21" s="37" t="n"/>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="19">
-      <c r="A22" s="37" t="n"/>
-      <c r="B22" s="37" t="n"/>
-      <c r="C22" s="37" t="n"/>
-      <c r="D22" s="37" t="n"/>
-      <c r="E22" s="37" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="19">
-      <c r="A23" s="37" t="n"/>
-      <c r="B23" s="37" t="n"/>
-      <c r="C23" s="37" t="n"/>
-      <c r="D23" s="37" t="n"/>
-      <c r="E23" s="37" t="n"/>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="19">
-      <c r="A24" s="37" t="n"/>
-      <c r="B24" s="37" t="n"/>
-      <c r="C24" s="37" t="n"/>
-      <c r="D24" s="37" t="n"/>
-      <c r="E24" s="37" t="n"/>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="19">
-      <c r="A25" s="37" t="n"/>
-      <c r="B25" s="37" t="n"/>
-      <c r="C25" s="37" t="n"/>
-      <c r="D25" s="37" t="n"/>
-      <c r="E25" s="37" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="19">
-      <c r="A26" s="37" t="n"/>
-      <c r="B26" s="37" t="n"/>
-      <c r="C26" s="37" t="n"/>
-      <c r="D26" s="37" t="n"/>
-      <c r="E26" s="37" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="19">
-      <c r="A27" s="37" t="n"/>
-      <c r="B27" s="37" t="n"/>
-      <c r="C27" s="37" t="n"/>
-      <c r="D27" s="37" t="n"/>
-      <c r="E27" s="37" t="n"/>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="19">
-      <c r="A28" s="37" t="n"/>
-      <c r="B28" s="37" t="n"/>
-      <c r="C28" s="37" t="n"/>
-      <c r="D28" s="37" t="n"/>
-      <c r="E28" s="37" t="n"/>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="19">
-      <c r="A29" s="37" t="n"/>
-      <c r="B29" s="37" t="n"/>
-      <c r="C29" s="37" t="n"/>
-      <c r="D29" s="37" t="n"/>
-      <c r="E29" s="37" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="19">
-      <c r="A30" s="37" t="n"/>
-      <c r="B30" s="37" t="n"/>
-      <c r="C30" s="37" t="n"/>
-      <c r="D30" s="37" t="n"/>
-      <c r="E30" s="37" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="19">
-      <c r="A31" s="37" t="n"/>
-      <c r="B31" s="37" t="n"/>
-      <c r="C31" s="37" t="n"/>
-      <c r="D31" s="37" t="n"/>
-      <c r="E31" s="37" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="19">
-      <c r="A32" s="37" t="n"/>
-      <c r="B32" s="37" t="n"/>
-      <c r="C32" s="37" t="n"/>
-      <c r="D32" s="37" t="n"/>
-      <c r="E32" s="37" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="19">
-      <c r="A33" s="37" t="n"/>
-      <c r="B33" s="37" t="n"/>
-      <c r="C33" s="37" t="n"/>
-      <c r="D33" s="37" t="n"/>
-      <c r="E33" s="37" t="n"/>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="19">
-      <c r="A34" s="37" t="n"/>
-      <c r="B34" s="37" t="n"/>
-      <c r="C34" s="37" t="n"/>
-      <c r="D34" s="37" t="n"/>
-      <c r="E34" s="37" t="n"/>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="19">
-      <c r="A35" s="37" t="n"/>
-      <c r="B35" s="37" t="n"/>
-      <c r="C35" s="37" t="n"/>
-      <c r="D35" s="37" t="n"/>
-      <c r="E35" s="37" t="n"/>
-    </row>
-    <row r="36" ht="15" customHeight="1" s="19">
-      <c r="A36" s="37" t="n"/>
-      <c r="B36" s="37" t="n"/>
-      <c r="C36" s="37" t="n"/>
-      <c r="D36" s="37" t="n"/>
-      <c r="E36" s="37" t="n"/>
-    </row>
-    <row r="37" ht="15" customHeight="1" s="19">
-      <c r="A37" s="37" t="n"/>
-      <c r="B37" s="37" t="n"/>
-      <c r="C37" s="37" t="n"/>
-      <c r="D37" s="37" t="n"/>
-      <c r="E37" s="37" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="19">
-      <c r="A38" s="37" t="n"/>
-      <c r="B38" s="37" t="n"/>
-      <c r="C38" s="37" t="n"/>
-      <c r="D38" s="37" t="n"/>
-      <c r="E38" s="37" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="19">
-      <c r="A39" s="37" t="n"/>
-      <c r="B39" s="37" t="n"/>
-      <c r="C39" s="37" t="n"/>
-      <c r="D39" s="37" t="n"/>
-      <c r="E39" s="37" t="n"/>
-    </row>
-    <row r="40" ht="15" customHeight="1" s="19">
-      <c r="A40" s="37" t="n"/>
-      <c r="B40" s="37" t="n"/>
-      <c r="C40" s="37" t="n"/>
-      <c r="D40" s="37" t="n"/>
-      <c r="E40" s="37" t="n"/>
-    </row>
-    <row r="41" ht="15" customHeight="1" s="19">
-      <c r="A41" s="37" t="n"/>
-      <c r="B41" s="37" t="n"/>
-      <c r="C41" s="37" t="n"/>
-      <c r="D41" s="37" t="n"/>
-      <c r="E41" s="37" t="n"/>
-    </row>
-    <row r="42" ht="15" customHeight="1" s="19">
-      <c r="A42" s="37" t="n"/>
-      <c r="B42" s="37" t="n"/>
-      <c r="C42" s="37" t="n"/>
-      <c r="D42" s="37" t="n"/>
-      <c r="E42" s="37" t="n"/>
-    </row>
-    <row r="43" ht="15" customHeight="1" s="19">
-      <c r="A43" s="37" t="n"/>
-      <c r="B43" s="37" t="n"/>
-      <c r="C43" s="37" t="n"/>
-      <c r="D43" s="37" t="n"/>
-      <c r="E43" s="37" t="n"/>
-    </row>
-    <row r="44" ht="15" customHeight="1" s="19">
-      <c r="A44" s="37" t="n"/>
-      <c r="B44" s="37" t="n"/>
-      <c r="C44" s="37" t="n"/>
-      <c r="D44" s="37" t="n"/>
-      <c r="E44" s="37" t="n"/>
-    </row>
-    <row r="45" ht="15" customHeight="1" s="19">
-      <c r="A45" s="37" t="n"/>
-      <c r="B45" s="37" t="n"/>
-      <c r="C45" s="37" t="n"/>
-      <c r="D45" s="37" t="n"/>
-      <c r="E45" s="37" t="n"/>
-    </row>
-    <row r="46" ht="15" customHeight="1" s="19">
-      <c r="A46" s="37" t="n"/>
-      <c r="B46" s="37" t="n"/>
-      <c r="C46" s="37" t="n"/>
-      <c r="D46" s="37" t="n"/>
-      <c r="E46" s="37" t="n"/>
-    </row>
-    <row r="47" ht="15" customHeight="1" s="19">
-      <c r="A47" s="37" t="n"/>
-      <c r="B47" s="37" t="n"/>
-      <c r="C47" s="37" t="n"/>
-      <c r="D47" s="37" t="n"/>
-      <c r="E47" s="37" t="n"/>
+    <row r="8">
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>E-100 .. E-500</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C8" s="76" t="inlineStr">
+        <is>
+          <t>entity state settled</t>
+        </is>
+      </c>
+      <c r="D8" s="76" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="E8" s="76" t="inlineStr">
+        <is>
+          <t>Capacities, Tags, Tracks and links current before anything reads them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="76" t="inlineStr">
+        <is>
+          <t>M-100</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>turn ownership established</t>
+        </is>
+      </c>
+      <c r="D9" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E9" s="76" t="inlineStr">
+        <is>
+          <t>respond and interrupt are defined in terms of mine/not-mine, so this must be settled before any cost is eligible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="76" t="inlineStr">
+        <is>
+          <t>M-200</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>budget refresh</t>
+        </is>
+      </c>
+      <c r="D10" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E10" s="76" t="inlineStr">
+        <is>
+          <t>Doubloons restored per the Budget. Must precede any payment this Moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="76" t="inlineStr">
+        <is>
+          <t>M-300</t>
+        </is>
+      </c>
+      <c r="B11" s="76" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C11" s="76" t="inlineStr">
+        <is>
+          <t>cap reset</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E11" s="76" t="inlineStr">
+        <is>
+          <t>Per-Moment and per-round cap counters clear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>M-400</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>scope refresh</t>
+        </is>
+      </c>
+      <c r="D12" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E12" s="76" t="inlineStr">
+        <is>
+          <t>Standing vectors re-evaluate what they cover, using positions as of now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="76" t="inlineStr">
+        <is>
+          <t>M-500</t>
+        </is>
+      </c>
+      <c r="B13" s="76" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C13" s="76" t="inlineStr">
+        <is>
+          <t>phenomena emit</t>
+        </is>
+      </c>
+      <c r="D13" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E13" s="76" t="inlineStr">
+        <is>
+          <t>A fire, plague or curse places its vectors into the scope settled at M-400. M-400 BEFORE M-500 IS LOAD-BEARING — a fire covers where you are NOW. And M-500 before C-100 so those vectors exist in time to be gathered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="76" t="inlineStr">
+        <is>
+          <t>C-100 .. C-600</t>
+        </is>
+      </c>
+      <c r="B14" s="76" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C14" s="76" t="inlineStr">
+        <is>
+          <t>vectors created</t>
+        </is>
+      </c>
+      <c r="D14" s="76" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="E14" s="76" t="inlineStr">
+        <is>
+          <t>Direction, magnitude, snapshot modifiers, pin, layer, class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="76" t="inlineStr">
+        <is>
+          <t>R-100 .. R-1400</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C15" s="76" t="inlineStr">
+        <is>
+          <t>vectors resolve, per target</t>
+        </is>
+      </c>
+      <c r="D15" s="76" t="inlineStr">
+        <is>
+          <t>existing · CLOSED in Phase 0</t>
+        </is>
+      </c>
+      <c r="E15" s="76" t="inlineStr">
+        <is>
+          <t>Nineteen slots, each forced by a worked case that failed without it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="76" t="inlineStr">
+        <is>
+          <t>X-100</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C16" s="76" t="inlineStr">
+        <is>
+          <t>direct Verbs apply</t>
+        </is>
+      </c>
+      <c r="D16" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E16" s="76" t="inlineStr">
+        <is>
+          <t>Move, transfer, set, spend. NOT EVERY VERB IS A VECTOR — these have no magnitude to modify and meet no Guards. X-100 AFTER R-1400 so a Listener that produces a movement applies it after resolution, not during.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="76" t="inlineStr">
+        <is>
+          <t>X-200</t>
+        </is>
+      </c>
+      <c r="B17" s="76" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C17" s="76" t="inlineStr">
+        <is>
+          <t>Track restoration</t>
+        </is>
+      </c>
+      <c r="D17" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E17" s="76" t="inlineStr">
+        <is>
+          <t>Natural recovery, per the Landing occupant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="76" t="inlineStr">
+        <is>
+          <t>X-300</t>
+        </is>
+      </c>
+      <c r="B18" s="76" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C18" s="76" t="inlineStr">
+        <is>
+          <t>progression accrues</t>
+        </is>
+      </c>
+      <c r="D18" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E18" s="76" t="inlineStr">
+        <is>
+          <t>Reads final positions, so after X-100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="76" t="inlineStr">
+        <is>
+          <t>X-400</t>
+        </is>
+      </c>
+      <c r="B19" s="76" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C19" s="76" t="inlineStr">
+        <is>
+          <t>knowledge propagates</t>
+        </is>
+      </c>
+      <c r="D19" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E19" s="76" t="inlineStr">
+        <is>
+          <t>Almanac updates from what was observed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="76" t="inlineStr">
+        <is>
+          <t>X-500</t>
+        </is>
+      </c>
+      <c r="B20" s="76" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C20" s="76" t="inlineStr">
+        <is>
+          <t>standing propagates</t>
+        </is>
+      </c>
+      <c r="D20" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E20" s="76" t="inlineStr">
+        <is>
+          <t>Social consequence spreads through Connections. AFTER X-400 — you cannot spread a reputation for something nobody knows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="76" t="inlineStr">
+        <is>
+          <t>X-600</t>
+        </is>
+      </c>
+      <c r="B21" s="76" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C21" s="76" t="inlineStr">
+        <is>
+          <t>cadence emission</t>
+        </is>
+      </c>
+      <c r="D21" s="76" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E21" s="76" t="inlineStr">
+        <is>
+          <t>Dispatch and Chronicle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="76" t="inlineStr">
+        <is>
+          <t>HONESTLY: THIS IS THE LEAST-GROUNDED SETTLED LIST. The R-region slots each came from a worked case that failed without them. M- and X- came from asking "what must be true before R-100" and "what reads the result", which is weaker evidence. EXPECT THESE REGIONS TO GAIN SLOTS IN PHASE 2 AND TREAT THAT AS NORMAL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="71" t="inlineStr">
+        <is>
+          <t>CONSIDERED AND REJECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>running direct Verbs through the R-region</t>
+        </is>
+      </c>
+      <c r="B26" s="72" t="inlineStr"/>
+      <c r="C26" s="72" t="inlineStr"/>
+      <c r="D26" s="72" t="inlineStr"/>
+      <c r="E26" s="72" t="inlineStr">
+        <is>
+          <t>REJECTED — nineteen slots of theatre for a Verb with no magnitude and no Guard. They pin to X-100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="72" t="inlineStr">
+        <is>
+          <t>a separate region for movement</t>
+        </is>
+      </c>
+      <c r="B27" s="72" t="inlineStr"/>
+      <c r="C27" s="72" t="inlineStr"/>
+      <c r="D27" s="72" t="inlineStr"/>
+      <c r="E27" s="72" t="inlineStr">
+        <is>
+          <t>REJECTED — movement is a direct Verb at X-100. A turn contains several Moments, so move-then-attack is two Moments and scope refreshes between them at M-400.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Harden cut; Landing retired as a Socket (two remain); Creature gains integrity and substance; X-100 narrowed to movement and transfer
</commit_message>
<xml_diff>
--- a/docs/substrate-lists.xlsx
+++ b/docs/substrate-lists.xlsx
@@ -7471,7 +7471,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -8030,7 +8029,6 @@
       </c>
       <c r="C32" s="24" t="n"/>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>
@@ -8919,7 +8917,7 @@
       </c>
       <c r="D16" s="76" t="inlineStr">
         <is>
-          <t>HARDEN. Resisting notches a counter making future resistance easier; failing notches the other way. THE ONE GENUINELY NEW MECHANISM — no physical system makes you harder to injure by injuring you; every serious mental system does (Unknown Armies, Delta Green, CoC).</t>
+          <t>HARDEN WAS PROPOSED HERE AND CUT. Resisting making resistance easier is a SNOWBALL IN BOTH DIRECTIONS — the classic death spiral. It works in Unknown Armies and Delta Green because it runs ACROSS A CAMPAIGN, not inside a fight. Within-scene feedback is a snowball; across-campaign feedback is an arc. A horror Component may add it on a session timescale.</t>
         </is>
       </c>
     </row>
@@ -9033,6 +9031,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="76" t="inlineStr">
         <is>
@@ -9040,6 +9039,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="71" t="inlineStr">
         <is>
@@ -9525,7 +9525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="19" min="1" max="1"/>
@@ -9545,7 +9545,7 @@
     <row r="2">
       <c r="A2" s="64" t="inlineStr">
         <is>
-          <t>PENDING · BLOCKING · three, Aug 2026</t>
+          <t>SETTLED · Aug 2026 · TWO</t>
         </is>
       </c>
     </row>
@@ -9559,7 +9559,7 @@
     <row r="4">
       <c r="A4" s="66" t="inlineStr">
         <is>
-          <t>THREE. Time and Budget moved into the Substrate in Aug 2026. Occupants are FROZEN PER SETTING — changing one makes a different Setting.</t>
+          <t>TWO. Time and Budget moved into the Substrate; LANDING WAS RETIRED when the Track merge ate its job. Five became two in a month, and each removal came from finding the hole held nothing up.</t>
         </is>
       </c>
     </row>
@@ -9677,32 +9677,33 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="70" t="inlineStr">
+      <c r="A10" s="72" t="inlineStr">
         <is>
           <t>Landing</t>
         </is>
       </c>
-      <c r="B10" s="70" t="inlineStr">
+      <c r="B10" s="72" t="inlineStr">
         <is>
           <t>What persistent state each Dimension may address (= L25, fourteen rows)</t>
         </is>
       </c>
-      <c r="C10" s="70" t="inlineStr">
+      <c r="C10" s="72" t="inlineStr">
         <is>
           <t>How a landed vector becomes persistent state</t>
         </is>
       </c>
-      <c r="D10" s="70" t="inlineStr">
+      <c r="D10" s="72" t="inlineStr">
         <is>
           <t>Vectors arrive and nothing happens</t>
         </is>
       </c>
-      <c r="E10" s="70" t="inlineStr">
-        <is>
-          <t>Research (lists-research.md §4) says this is a PIPELINE, not one step: buffer -&gt; convert -&gt; name. The buffer belongs to the occupant and is never durable.</t>
-        </is>
-      </c>
-    </row>
+      <c r="E10" s="72" t="inlineStr">
+        <is>
+          <t>RETIRED Aug 2026. Its job was choosing HOW a surviving vector becomes persistent state — pool, wound track, consequence slot, phrase. The Track merge removed the choice: every axis is a Track by construction. What was left is Thresholds, Listeners and Track definitions, all of which exist. A Socket that can be satisfied by doing nothing is not a Socket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="70" t="inlineStr">
         <is>
@@ -9710,6 +9711,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="71" t="inlineStr">
         <is>
@@ -9777,6 +9779,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13960,12 +13963,12 @@
       </c>
       <c r="C11" s="76" t="inlineStr">
         <is>
-          <t>vitality</t>
+          <t>vitality · vigor · mobility · acuity · composure · clarity · will · temperature · integrity · substance</t>
         </is>
       </c>
       <c r="D11" s="76" t="inlineStr">
         <is>
-          <t>posture · awareness · consciousness</t>
+          <t>Specialisations. integrity is bone and structure, substance is flesh and matter — without them a hammer blow against a person would land on nothing.</t>
         </is>
       </c>
       <c r="E11" s="76" t="inlineStr">
@@ -14109,6 +14112,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="76" t="inlineStr">
         <is>
@@ -14116,6 +14120,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="71" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
L26 settled: seven condition forms, cascade depth 32, and the Brush
</commit_message>
<xml_diff>
--- a/docs/substrate-lists.xlsx
+++ b/docs/substrate-lists.xlsx
@@ -288,7 +288,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -503,6 +503,9 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -7471,6 +7474,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -7874,21 +7878,21 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="19">
-      <c r="A24" s="26" t="inlineStr">
+      <c r="A24" s="73" t="inlineStr">
         <is>
           <t>L26 · Listener condition forms</t>
         </is>
       </c>
-      <c r="B24" s="31" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C24" s="26">
+      <c r="B24" s="80" t="inlineStr">
+        <is>
+          <t>SETTLED · Aug 2026</t>
+        </is>
+      </c>
+      <c r="C24" s="73">
         <f>COUNTA('L26 Listener condition forms'!A8:A47)</f>
         <v/>
       </c>
-      <c r="D24" s="26">
+      <c r="D24" s="73">
         <f>IF(C24&gt;0,"started","not started")</f>
         <v/>
       </c>
@@ -8029,6 +8033,7 @@
       </c>
       <c r="C32" s="24" t="n"/>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>
@@ -9031,7 +9036,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="76" t="inlineStr">
         <is>
@@ -9039,7 +9043,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="71" t="inlineStr">
         <is>
@@ -9100,7 +9103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" style="19" min="1" max="1"/>
@@ -9119,7 +9122,7 @@
     <row r="2">
       <c r="A2" s="64" t="inlineStr">
         <is>
-          <t>PENDING · research-seeded Aug 2026</t>
+          <t>SETTLED · Aug 2026</t>
         </is>
       </c>
     </row>
@@ -9511,6 +9514,138 @@
       <c r="D29" s="76" t="inlineStr">
         <is>
           <t>"The next time somebody attacks" is once. "While you are bleeding" is while. No default because the two behave differently enough that a wrong guess is silent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="76" t="inlineStr">
+        <is>
+          <t>cascade depth</t>
+        </is>
+      </c>
+      <c r="B31" s="76" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C31" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="D31" s="76" t="inlineStr">
+        <is>
+          <t>Where the database world settled 20 years ago. Magic terminates without a counter by calling a genuine loop A DRAW — a social rule. We have no table to appeal to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="76" t="inlineStr">
+        <is>
+          <t>at the limit</t>
+        </is>
+      </c>
+      <c r="B32" s="76" t="inlineStr">
+        <is>
+          <t>halt without applying, WRITE A RECORD</t>
+        </is>
+      </c>
+      <c r="C32" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="D32" s="76" t="inlineStr">
+        <is>
+          <t>Rolling back is unavailable (append-only). Silent dropping is what makes board states unexplainable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="76" t="inlineStr">
+        <is>
+          <t>ordering</t>
+        </is>
+      </c>
+      <c r="B33" s="76" t="inlineStr">
+        <is>
+          <t>semantic class first, then (layer, component_id, listener_id, target_entity_id)</t>
+        </is>
+      </c>
+      <c r="C33" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="D33" s="76" t="inlineStr">
+        <is>
+          <t>The key may contain ONLY values that do not move when unrelated content is added. Drools salience is deterministic but NOT STABLE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="76" t="inlineStr">
+        <is>
+          <t>composition</t>
+        </is>
+      </c>
+      <c r="B34" s="76" t="inlineStr">
+        <is>
+          <t>and · or · not</t>
+        </is>
+      </c>
+      <c r="C34" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="D34" s="76" t="inlineStr">
+        <is>
+          <t>"not" is safe — the open-world rule is about absent FIELDS, not unknown STATE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="76" t="inlineStr">
+        <is>
+          <t>firing discipline</t>
+        </is>
+      </c>
+      <c r="B35" s="76" t="inlineStr">
+        <is>
+          <t>once | while — REQUIRED, no default</t>
+        </is>
+      </c>
+      <c r="C35" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="D35" s="76" t="inlineStr">
+        <is>
+          <t>A wrong guess is silent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="76" t="inlineStr">
+        <is>
+          <t>BRUSH</t>
+        </is>
+      </c>
+      <c r="B36" s="76" t="inlineStr">
+        <is>
+          <t>a Threshold crossed and uncrossed inside one Moment</t>
+        </is>
+      </c>
+      <c r="C36" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED · NEW</t>
+        </is>
+      </c>
+      <c r="D36" s="76" t="inlineStr">
+        <is>
+          <t>A creature at 0 vitality at R-1200 healed at R-1250 is NOT DEAD — Listeners evaluate at R-1400. Written on the Resolution Record so a Lens can surface it and a Listener can watch it via the "Record matching a shape" form. SLOTS ARE OBSERVABLE; the order of commutative operations INSIDE a slot is not.</t>
         </is>
       </c>
     </row>
@@ -9525,7 +9660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="19" min="1" max="1"/>
@@ -9703,7 +9838,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="70" t="inlineStr">
         <is>
@@ -9711,7 +9845,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="71" t="inlineStr">
         <is>
@@ -9779,7 +9912,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14112,7 +14244,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="76" t="inlineStr">
         <is>
@@ -14120,7 +14251,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="71" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Phase 1 closed: consistency sweep across all docs, START-HERE handoff, worked-builds, refreshed open questions
</commit_message>
<xml_diff>
--- a/docs/substrate-lists.xlsx
+++ b/docs/substrate-lists.xlsx
@@ -45,7 +45,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -203,6 +203,11 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F3864"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -288,7 +293,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -507,6 +512,30 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -764,9 +793,9 @@
   <dimension ref="A1:C69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="30" customWidth="1" style="18" min="1" max="1"/>
-    <col width="42" customWidth="1" style="18" min="2" max="2"/>
-    <col width="78" customWidth="1" style="18" min="3" max="3"/>
+    <col width="34" customWidth="1" style="18" min="1" max="1"/>
+    <col width="28" customWidth="1" style="18" min="2" max="2"/>
+    <col width="62" customWidth="1" style="18" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.35" customHeight="1" s="19">
@@ -779,7 +808,7 @@
     <row r="2" ht="15" customHeight="1" s="19">
       <c r="A2" s="21" t="inlineStr">
         <is>
-          <t>Everything the Substrate still needs decided. One tab per list. Source of truth: docs/dictionary.md Part 11.</t>
+          <t>Source of truth: docs/dictionary.md Part 11. PHASE 1 CLOSED, AUGUST 2026 — every blocking list is settled except L6 Verbs, which is drafted and closes in Phase 2 against real content.</t>
         </is>
       </c>
     </row>
@@ -839,340 +868,350 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="19">
-      <c r="A10" s="22" t="inlineStr">
-        <is>
-          <t>The order to fill them in</t>
+      <c r="A10" s="81" t="inlineStr">
+        <is>
+          <t>Where each list stands</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="19">
-      <c r="A11" s="25" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="A11" s="82" t="inlineStr">
         <is>
           <t>List</t>
         </is>
       </c>
-      <c r="C11" s="25" t="inlineStr">
-        <is>
-          <t>Why here</t>
+      <c r="B11" s="82" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C11" s="82" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="19">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B12" s="27" t="inlineStr">
-        <is>
-          <t>L29 Capacities</t>
-        </is>
-      </c>
-      <c r="C12" s="26" t="inlineStr">
-        <is>
-          <t>The most load-bearing list. What a character is made of AND the axes an attempt splits across.</t>
+      <c r="A12" s="83" t="inlineStr">
+        <is>
+          <t>L21 Dimension Spaces</t>
+        </is>
+      </c>
+      <c r="B12" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C12" s="83" t="inlineStr">
+        <is>
+          <t>five: physical, mental, social, mystic, attempt</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="19">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B13" s="27" t="inlineStr">
-        <is>
-          <t>L21 Dimension Spaces</t>
-        </is>
-      </c>
-      <c r="C13" s="26" t="inlineStr">
-        <is>
-          <t>Then L22 Dimensions, then L23 Channels. Strictly in that order.</t>
+      <c r="A13" s="83" t="inlineStr">
+        <is>
+          <t>L29 Attempt Domains &amp; Dimensions</t>
+        </is>
+      </c>
+      <c r="B13" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C13" s="83" t="inlineStr">
+        <is>
+          <t>7 Domains, 15 Dimensions, Specialisations</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="19">
-      <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B14" s="27" t="inlineStr">
-        <is>
-          <t>L22 Dimensions, per Space</t>
-        </is>
-      </c>
-      <c r="C14" s="26" t="n"/>
+      <c r="A14" s="83" t="inlineStr">
+        <is>
+          <t>L22 Dimensions</t>
+        </is>
+      </c>
+      <c r="B14" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C14" s="83" t="inlineStr">
+        <is>
+          <t>fourteen, sign convention: negative = less of the target</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="19">
-      <c r="A15" s="26" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B15" s="27" t="inlineStr">
-        <is>
-          <t>L23 Named Channels</t>
-        </is>
-      </c>
-      <c r="C15" s="26" t="n"/>
+      <c r="A15" s="83" t="inlineStr">
+        <is>
+          <t>L23 Channels</t>
+        </is>
+      </c>
+      <c r="B15" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C15" s="83" t="inlineStr">
+        <is>
+          <t>88, hundredths over all fourteen, summing to 100</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="19">
-      <c r="A16" s="26" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B16" s="27" t="inlineStr">
+      <c r="A16" s="83" t="inlineStr">
+        <is>
+          <t>L32 Moment kinds</t>
+        </is>
+      </c>
+      <c r="B16" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C16" s="83" t="inlineStr">
+        <is>
+          <t>nine, every reference carrying a round</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="19">
+      <c r="A17" s="83" t="inlineStr">
+        <is>
+          <t>L31 Timings</t>
+        </is>
+      </c>
+      <c r="B17" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C17" s="83" t="inlineStr">
+        <is>
+          <t>four: own, any, respond, interrupt — plus trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="19">
+      <c r="A18" s="83" t="inlineStr">
         <is>
           <t>L27 Sockets</t>
         </is>
       </c>
-      <c r="C16" s="26" t="inlineStr">
-        <is>
-          <t>Blocks the Component contract.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="19">
-      <c r="A17" s="26" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B17" s="27" t="inlineStr">
-        <is>
-          <t>L28 Economy Units</t>
-        </is>
-      </c>
-      <c r="C17" s="26" t="inlineStr">
-        <is>
-          <t>Blocks every spell and ability ever written.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="19">
-      <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
+      <c r="B18" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C18" s="83" t="inlineStr">
+        <is>
+          <t>TWO: Place and Resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="19">
+      <c r="A19" s="83" t="inlineStr">
+        <is>
+          <t>L28 Economy</t>
+        </is>
+      </c>
+      <c r="B19" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C19" s="83" t="inlineStr">
+        <is>
+          <t>one unit (doubloon); cost = cost + timing + cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="19">
+      <c r="A20" s="83" t="inlineStr">
         <is>
           <t>L1 / L2 / L3</t>
         </is>
       </c>
-      <c r="C18" s="26" t="inlineStr">
-        <is>
-          <t>Categories, then Universal Attributes, then Category Attributes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="19">
-      <c r="A19" s="26" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B19" s="27" t="inlineStr">
-        <is>
-          <t>L4 Tags and L5 State axes</t>
-        </is>
-      </c>
-      <c r="C19" s="26" t="n"/>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="19">
-      <c r="A20" s="26" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B20" s="27" t="inlineStr">
-        <is>
-          <t>L18 Aggregation operators</t>
-        </is>
-      </c>
-      <c r="C20" s="26" t="inlineStr">
-        <is>
-          <t>The single most likely source of a determinism bug.</t>
+      <c r="B20" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C20" s="83" t="inlineStr">
+        <is>
+          <t>nine Categories that compose; eight universal fields</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="19">
-      <c r="A21" s="26" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B21" s="27" t="inlineStr">
-        <is>
-          <t>L25 Conversions</t>
-        </is>
-      </c>
-      <c r="C21" s="26" t="inlineStr">
-        <is>
-          <t>What a surviving vector actually does.</t>
+      <c r="A21" s="83" t="inlineStr">
+        <is>
+          <t>L5 Tracks</t>
+        </is>
+      </c>
+      <c r="B21" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C21" s="83" t="inlineStr">
+        <is>
+          <t>fourteen, one per Dimension; conditions are BANDS</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="19">
-      <c r="A22" s="26" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B22" s="27" t="inlineStr">
-        <is>
-          <t>L7 Layers — the rest</t>
-        </is>
-      </c>
-      <c r="C22" s="26" t="inlineStr">
-        <is>
-          <t>Everything outside resolution: progression, economy, movement, knowledge, standing.</t>
+      <c r="A22" s="83" t="inlineStr">
+        <is>
+          <t>L18 Aggregation</t>
+        </is>
+      </c>
+      <c r="B22" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C22" s="83" t="inlineStr">
+        <is>
+          <t>collapsed to four rules by the Track merge</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="19">
-      <c r="A23" s="26" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B23" s="27" t="inlineStr">
+      <c r="A23" s="83" t="inlineStr">
+        <is>
+          <t>L25 Landing</t>
+        </is>
+      </c>
+      <c r="B23" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C23" s="83" t="inlineStr">
+        <is>
+          <t>a push lands on the Track the Dimension names</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="19">
+      <c r="A24" s="83" t="inlineStr">
+        <is>
+          <t>L7 Layers</t>
+        </is>
+      </c>
+      <c r="B24" s="84" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C24" s="83" t="inlineStr">
+        <is>
+          <t>five regions, 41 slots; M- and X- added</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="76" t="inlineStr">
         <is>
           <t>L26 Listener conditions</t>
         </is>
       </c>
-      <c r="C23" s="26" t="inlineStr">
-        <is>
-          <t>Plus the cascade limit and the evaluation order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="19">
-      <c r="A24" s="26" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B24" s="27" t="inlineStr">
-        <is>
-          <t>L6 VERBS — LAST</t>
-        </is>
-      </c>
-      <c r="C24" s="26" t="inlineStr">
-        <is>
-          <t>Not third, and not an afternoon. Every list above produces the evidence.</t>
+      <c r="B25" s="76" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
+        </is>
+      </c>
+      <c r="C25" s="76" t="inlineStr">
+        <is>
+          <t>seven forms; depth 32; halt-and-Record; the Brush</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="19">
-      <c r="A26" s="22" t="inlineStr">
-        <is>
-          <t>Status key</t>
+      <c r="A26" s="85" t="inlineStr">
+        <is>
+          <t>L4 Tags</t>
+        </is>
+      </c>
+      <c r="B26" s="72" t="inlineStr">
+        <is>
+          <t>PROVISIONAL</t>
+        </is>
+      </c>
+      <c r="C26" s="72" t="inlineStr">
+        <is>
+          <t>22 chosen; full field survey in docs/tags-*.md</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="19">
-      <c r="A27" s="28" t="inlineStr">
-        <is>
-          <t>BLOCKING</t>
-        </is>
-      </c>
-      <c r="B27" s="24" t="inlineStr">
-        <is>
-          <t>Nothing can be built until this is done.</t>
+      <c r="A27" s="86" t="inlineStr">
+        <is>
+          <t>L6 Verbs</t>
+        </is>
+      </c>
+      <c r="B27" s="87" t="inlineStr">
+        <is>
+          <t>DRAFTED — CLOSES IN PHASE 2</t>
+        </is>
+      </c>
+      <c r="C27" s="72" t="inlineStr">
+        <is>
+          <t>Push · Set · Place · Repin · Link · Create · Decide</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="19">
-      <c r="A28" s="29" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="B28" s="24" t="inlineStr">
-        <is>
-          <t>Needed, not yet blocking anything.</t>
+      <c r="A28" s="88" t="inlineStr">
+        <is>
+          <t>L10-L13, L19, L20, L24, L30</t>
+        </is>
+      </c>
+      <c r="B28" s="87" t="inlineStr">
+        <is>
+          <t>PENDING, not blocking</t>
+        </is>
+      </c>
+      <c r="C28" s="72" t="inlineStr">
+        <is>
+          <t>none of these hold anything up</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="19">
-      <c r="A29" s="29" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="B29" s="24" t="inlineStr">
-        <is>
-          <t>Shape decided, contents open.</t>
-        </is>
-      </c>
+      <c r="A29" s="29" t="n"/>
+      <c r="B29" s="24" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="19">
-      <c r="A30" s="28" t="inlineStr">
-        <is>
-          <t>CLOSE LAST</t>
-        </is>
-      </c>
-      <c r="B30" s="24" t="inlineStr">
-        <is>
-          <t>Deliberately not settled yet. Settling it early is the mistake.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A30" s="28" t="n"/>
+      <c r="B30" s="24" t="n"/>
+    </row>
+    <row r="31"/>
     <row r="32">
-      <c r="A32" s="38" t="inlineStr">
-        <is>
-          <t>HOW TO USE THE PROPOSALS — added August 2026</t>
-        </is>
-      </c>
+      <c r="A32" s="38" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="39" t="inlineStr"/>
+      <c r="A33" s="39" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="39" t="inlineStr">
-        <is>
-          <t>Every blocking tab now opens with PROPOSED rows on a pale yellow background. They are a starting position, not an answer.</t>
-        </is>
-      </c>
+      <c r="A34" s="39" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="39" t="inlineStr">
-        <is>
-          <t>Three things to do with each row: accept it, edit it, or cut it. Cutting is the most valuable of the three.</t>
-        </is>
-      </c>
+      <c r="A35" s="39" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="39" t="inlineStr"/>
+      <c r="A36" s="39" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="39" t="inlineStr">
-        <is>
-          <t>When you cut one, move it down to the CONSIDERED AND REJECTED block on the same tab and say why. Nothing above the</t>
-        </is>
-      </c>
+      <c r="A37" s="39" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="39" t="inlineStr">
-        <is>
-          <t>Substrate can put back something the Substrate omitted, and in two years you will not remember whether a thing is missing</t>
-        </is>
-      </c>
+      <c r="A38" s="39" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="39" t="inlineStr">
-        <is>
-          <t>because you decided against it or because you never thought of it.</t>
-        </is>
-      </c>
+      <c r="A39" s="39" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="39" t="inlineStr"/>
@@ -7474,7 +7513,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -8033,7 +8071,6 @@
       </c>
       <c r="C32" s="24" t="n"/>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Reconciliation 2/4: docs aligned to settled state; lint added; L23 regenerated
</commit_message>
<xml_diff>
--- a/docs/substrate-lists.xlsx
+++ b/docs/substrate-lists.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L2 Universal Attributes" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L3 Category Attributes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L4 Core Tag vocabulary" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L5 State axes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L5 Tracks" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L6 Verbs" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L7 Layers" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L10 Challenge Profile axes" sheetId="10" state="visible" r:id="rId10"/>
@@ -27,7 +27,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L22 Dimensions, per Space" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L23 Named Channels" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L24 Guard presets" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L25 Transient-to-Persistent con" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L25 Landing models" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L26 Listener condition forms" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L27 Sockets" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L28 Economy" sheetId="24" state="visible" r:id="rId24"/>
@@ -293,7 +293,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -537,6 +537,20 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1142,7 +1156,7 @@
       </c>
       <c r="C26" s="72" t="inlineStr">
         <is>
-          <t>22 chosen; full field survey in docs/tags-*.md</t>
+          <t>24 chosen (11 Substrate + 13 Ruleset); full field survey in docs/tags-*.md</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1202,6 @@
       <c r="A30" s="28" t="n"/>
       <c r="B30" s="24" t="n"/>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="38" t="n"/>
     </row>
@@ -1233,7 +1246,7 @@
     <row r="43">
       <c r="A43" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">   →  L1 / L2 / L3 (+ the three character sheets)  →  L4 / L5 / L18 / L25  →  L7 Layers  →  L26 Listeners  →  L6 VERBS LAST</t>
+          <t xml:space="preserve">   →  L1 / L2 / L3 (sheets deferred to the Phase 2 paper kit)  →  L4 / L5 / L18 / L25  →  L7 Layers  →  L26 Listeners  →  L6 VERBS LAST</t>
         </is>
       </c>
     </row>
@@ -4028,7 +4041,7 @@
       </c>
       <c r="C7" s="34" t="inlineStr">
         <is>
-          <t>thermal, kinetic, vital</t>
+          <t>temperature, integrity, vitality</t>
         </is>
       </c>
       <c r="D7" s="34" t="inlineStr">
@@ -4060,7 +4073,7 @@
       </c>
       <c r="C8" s="41" t="inlineStr">
         <is>
-          <t>thermal, kinetic, vital, corrosive, vigor?</t>
+          <t>temperature, integrity, substance, vitality, vigor, mobility, acuity</t>
         </is>
       </c>
       <c r="D8" s="41" t="inlineStr">
@@ -4087,7 +4100,7 @@
       </c>
       <c r="C9" s="41" t="inlineStr">
         <is>
-          <t>composure, clarity, will?</t>
+          <t>composure, clarity, will</t>
         </is>
       </c>
       <c r="D9" s="41" t="inlineStr">
@@ -4114,7 +4127,7 @@
       </c>
       <c r="C10" s="41" t="inlineStr">
         <is>
-          <t>regard, standing?</t>
+          <t>regard, standing</t>
         </is>
       </c>
       <c r="D10" s="41" t="inlineStr">
@@ -4141,7 +4154,7 @@
       </c>
       <c r="C11" s="41" t="inlineStr">
         <is>
-          <t>working?, essence?</t>
+          <t>working, essence</t>
         </is>
       </c>
       <c r="D11" s="41" t="inlineStr">
@@ -4248,7 +4261,7 @@
       <c r="D18" s="41" t="inlineStr"/>
       <c r="E18" s="41" t="inlineStr">
         <is>
-          <t>REJECTED: money is a Resource, not a direction. A bribe is a social vector paid for with a Resource</t>
+          <t>REJECTED: money is a payable Track, not a direction. A bribe is a social vector paid for with a Resource</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5289,7 @@
     <row r="3" ht="30" customHeight="1" s="19">
       <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>Positions in HUNDREDTHS. Every row must sum, in absolute value, to exactly 100 (column R checks it). No two Channels may share a position.</t>
+          <t>Positions in HUNDREDTHS. Every row must sum, in absolute value, to exactly 100. CANONICAL SOURCE: docs/channels.py — this tab is generated from it; edit there, regenerate here.</t>
         </is>
       </c>
     </row>
@@ -5375,7 +5388,7 @@
       </c>
     </row>
     <row r="7" ht="46.25" customHeight="1" s="19">
-      <c r="A7" s="49" t="inlineStr">
+      <c r="A7" s="50" t="inlineStr">
         <is>
           <t>FORCE &amp; WEAPONS</t>
         </is>
@@ -5385,36 +5398,29 @@
           <t>impact</t>
         </is>
       </c>
-      <c r="C7" s="34" t="inlineStr">
-        <is>
-          <t>thermal +1.0</t>
-        </is>
-      </c>
-      <c r="D7" s="51" t="n">
+      <c r="C7" s="50" t="n"/>
+      <c r="D7" s="89" t="n">
         <v>-100</v>
       </c>
-      <c r="E7" s="34" t="inlineStr">
-        <is>
-          <t>transient</t>
-        </is>
-      </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>Creating a damage type means placing it. Its relationship to every existing type is then already determined</t>
-        </is>
-      </c>
-      <c r="G7" s="35" t="inlineStr">
-        <is>
-          <t>← example, not data</t>
-        </is>
-      </c>
-      <c r="Q7" s="18">
+      <c r="E7" s="50" t="n"/>
+      <c r="F7" s="50" t="n"/>
+      <c r="G7" s="44" t="n"/>
+      <c r="H7" s="60" t="n"/>
+      <c r="I7" s="60" t="n"/>
+      <c r="J7" s="60" t="n"/>
+      <c r="K7" s="60" t="n"/>
+      <c r="L7" s="60" t="n"/>
+      <c r="M7" s="60" t="n"/>
+      <c r="N7" s="60" t="n"/>
+      <c r="O7" s="60" t="n"/>
+      <c r="P7" s="60" t="n"/>
+      <c r="Q7" s="44">
         <f>IF(SUMPRODUCT(ABS(C7:P7))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="19">
-      <c r="A8" s="52" t="inlineStr">
+      <c r="A8" s="40" t="inlineStr">
         <is>
           <t>FORCE &amp; WEAPONS</t>
         </is>
@@ -5424,29 +5430,31 @@
           <t>pierce</t>
         </is>
       </c>
-      <c r="C8" s="36" t="inlineStr">
-        <is>
-          <t>thermal +1.0</t>
-        </is>
-      </c>
-      <c r="D8" s="53" t="n">
+      <c r="C8" s="40" t="n"/>
+      <c r="D8" s="90" t="n">
         <v>-80</v>
       </c>
-      <c r="E8" s="36" t="inlineStr">
-        <is>
-          <t>transient</t>
-        </is>
-      </c>
-      <c r="F8" s="53" t="n">
+      <c r="E8" s="40" t="n"/>
+      <c r="F8" s="90" t="n">
         <v>-20</v>
       </c>
-      <c r="Q8" s="18">
+      <c r="G8" s="60" t="n"/>
+      <c r="H8" s="60" t="n"/>
+      <c r="I8" s="60" t="n"/>
+      <c r="J8" s="60" t="n"/>
+      <c r="K8" s="60" t="n"/>
+      <c r="L8" s="60" t="n"/>
+      <c r="M8" s="60" t="n"/>
+      <c r="N8" s="60" t="n"/>
+      <c r="O8" s="60" t="n"/>
+      <c r="P8" s="60" t="n"/>
+      <c r="Q8" s="44">
         <f>IF(SUMPRODUCT(ABS(C8:P8))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="19">
-      <c r="A9" s="52" t="inlineStr">
+      <c r="A9" s="40" t="inlineStr">
         <is>
           <t>FORCE &amp; WEAPONS</t>
         </is>
@@ -5456,29 +5464,31 @@
           <t>rend</t>
         </is>
       </c>
-      <c r="C9" s="36" t="inlineStr">
-        <is>
-          <t>thermal −1.0</t>
-        </is>
-      </c>
-      <c r="D9" s="53" t="n">
+      <c r="C9" s="40" t="n"/>
+      <c r="D9" s="90" t="n">
         <v>-60</v>
       </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>transient</t>
-        </is>
-      </c>
-      <c r="F9" s="53" t="n">
+      <c r="E9" s="40" t="n"/>
+      <c r="F9" s="90" t="n">
         <v>-40</v>
       </c>
-      <c r="Q9" s="18">
+      <c r="G9" s="60" t="n"/>
+      <c r="H9" s="60" t="n"/>
+      <c r="I9" s="60" t="n"/>
+      <c r="J9" s="60" t="n"/>
+      <c r="K9" s="60" t="n"/>
+      <c r="L9" s="60" t="n"/>
+      <c r="M9" s="60" t="n"/>
+      <c r="N9" s="60" t="n"/>
+      <c r="O9" s="60" t="n"/>
+      <c r="P9" s="60" t="n"/>
+      <c r="Q9" s="44">
         <f>IF(SUMPRODUCT(ABS(C9:P9))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="19">
-      <c r="A10" s="52" t="inlineStr">
+      <c r="A10" s="40" t="inlineStr">
         <is>
           <t>FORCE &amp; WEAPONS</t>
         </is>
@@ -5488,29 +5498,31 @@
           <t>bleed</t>
         </is>
       </c>
-      <c r="C10" s="36" t="inlineStr">
-        <is>
-          <t>kinetic +1.0</t>
-        </is>
-      </c>
-      <c r="D10" s="53" t="n">
+      <c r="C10" s="40" t="n"/>
+      <c r="D10" s="90" t="n">
         <v>-30</v>
       </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>transient</t>
-        </is>
-      </c>
-      <c r="F10" s="53" t="n">
+      <c r="E10" s="40" t="n"/>
+      <c r="F10" s="90" t="n">
         <v>-70</v>
       </c>
-      <c r="Q10" s="18">
+      <c r="G10" s="60" t="n"/>
+      <c r="H10" s="60" t="n"/>
+      <c r="I10" s="60" t="n"/>
+      <c r="J10" s="60" t="n"/>
+      <c r="K10" s="60" t="n"/>
+      <c r="L10" s="60" t="n"/>
+      <c r="M10" s="60" t="n"/>
+      <c r="N10" s="60" t="n"/>
+      <c r="O10" s="60" t="n"/>
+      <c r="P10" s="60" t="n"/>
+      <c r="Q10" s="44">
         <f>IF(SUMPRODUCT(ABS(C10:P10))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="19">
-      <c r="A11" s="52" t="inlineStr">
+      <c r="A11" s="40" t="inlineStr">
         <is>
           <t>FORCE &amp; WEAPONS</t>
         </is>
@@ -5520,29 +5532,31 @@
           <t>crush</t>
         </is>
       </c>
-      <c r="C11" s="36" t="inlineStr">
-        <is>
-          <t>thermal +0.3, kinetic +0.7</t>
-        </is>
-      </c>
-      <c r="D11" s="53" t="n">
+      <c r="C11" s="40" t="n"/>
+      <c r="D11" s="90" t="n">
         <v>-70</v>
       </c>
-      <c r="E11" s="53" t="n">
+      <c r="E11" s="90" t="n">
         <v>-30</v>
       </c>
-      <c r="F11" s="36" t="inlineStr">
-        <is>
-          <t>PROPOSED. The interior Channel that proves the Space is worth having</t>
-        </is>
-      </c>
-      <c r="Q11" s="18">
+      <c r="F11" s="40" t="n"/>
+      <c r="G11" s="60" t="n"/>
+      <c r="H11" s="60" t="n"/>
+      <c r="I11" s="60" t="n"/>
+      <c r="J11" s="60" t="n"/>
+      <c r="K11" s="60" t="n"/>
+      <c r="L11" s="60" t="n"/>
+      <c r="M11" s="60" t="n"/>
+      <c r="N11" s="60" t="n"/>
+      <c r="O11" s="60" t="n"/>
+      <c r="P11" s="60" t="n"/>
+      <c r="Q11" s="44">
         <f>IF(SUMPRODUCT(ABS(C11:P11))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="19">
-      <c r="A12" s="52" t="inlineStr">
+      <c r="A12" s="40" t="inlineStr">
         <is>
           <t>FORCE &amp; WEAPONS</t>
         </is>
@@ -5552,34 +5566,31 @@
           <t>stagger</t>
         </is>
       </c>
-      <c r="C12" s="36" t="inlineStr">
-        <is>
-          <t>vital +1.0</t>
-        </is>
-      </c>
-      <c r="D12" s="53" t="n">
+      <c r="C12" s="40" t="n"/>
+      <c r="D12" s="90" t="n">
         <v>-50</v>
       </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>persistent</t>
-        </is>
-      </c>
-      <c r="F12" s="36" t="inlineStr">
-        <is>
-          <t>PROPOSED. Persistent — it keeps working</t>
-        </is>
-      </c>
-      <c r="G12" s="54" t="n">
+      <c r="E12" s="40" t="n"/>
+      <c r="F12" s="40" t="n"/>
+      <c r="G12" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q12" s="18">
+      <c r="H12" s="60" t="n"/>
+      <c r="I12" s="60" t="n"/>
+      <c r="J12" s="60" t="n"/>
+      <c r="K12" s="60" t="n"/>
+      <c r="L12" s="60" t="n"/>
+      <c r="M12" s="60" t="n"/>
+      <c r="N12" s="60" t="n"/>
+      <c r="O12" s="60" t="n"/>
+      <c r="P12" s="60" t="n"/>
+      <c r="Q12" s="44">
         <f>IF(SUMPRODUCT(ABS(C12:P12))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="19">
-      <c r="A13" s="52" t="inlineStr">
+      <c r="A13" s="40" t="inlineStr">
         <is>
           <t>FORCE &amp; WEAPONS</t>
         </is>
@@ -5589,34 +5600,31 @@
           <t>concussion</t>
         </is>
       </c>
-      <c r="C13" s="36" t="inlineStr">
-        <is>
-          <t>corrosive +0.7, thermal +0.3</t>
-        </is>
-      </c>
-      <c r="D13" s="53" t="n">
+      <c r="C13" s="40" t="n"/>
+      <c r="D13" s="90" t="n">
         <v>-50</v>
       </c>
-      <c r="E13" s="36" t="inlineStr">
-        <is>
-          <t>persistent</t>
-        </is>
-      </c>
-      <c r="F13" s="36" t="inlineStr">
-        <is>
-          <t>PROPOSED. Second interior Channel</t>
-        </is>
-      </c>
-      <c r="K13" s="54" t="n">
+      <c r="E13" s="40" t="n"/>
+      <c r="F13" s="40" t="n"/>
+      <c r="G13" s="60" t="n"/>
+      <c r="H13" s="60" t="n"/>
+      <c r="I13" s="60" t="n"/>
+      <c r="J13" s="60" t="n"/>
+      <c r="K13" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q13" s="18">
+      <c r="L13" s="60" t="n"/>
+      <c r="M13" s="60" t="n"/>
+      <c r="N13" s="60" t="n"/>
+      <c r="O13" s="60" t="n"/>
+      <c r="P13" s="60" t="n"/>
+      <c r="Q13" s="44">
         <f>IF(SUMPRODUCT(ABS(C13:P13))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="19">
-      <c r="A14" s="52" t="inlineStr">
+      <c r="A14" s="40" t="inlineStr">
         <is>
           <t>FORCE &amp; WEAPONS</t>
         </is>
@@ -5626,34 +5634,31 @@
           <t>knockdown</t>
         </is>
       </c>
-      <c r="C14" s="36" t="inlineStr">
-        <is>
-          <t>thermal +0.6, vital +0.4</t>
-        </is>
-      </c>
-      <c r="D14" s="53" t="n">
+      <c r="C14" s="40" t="n"/>
+      <c r="D14" s="90" t="n">
         <v>-40</v>
       </c>
-      <c r="E14" s="36" t="inlineStr">
-        <is>
-          <t>transient</t>
-        </is>
-      </c>
-      <c r="F14" s="36" t="inlineStr">
-        <is>
-          <t>PROPOSED. Third interior Channel — the target is at least three</t>
-        </is>
-      </c>
-      <c r="H14" s="54" t="n">
+      <c r="E14" s="40" t="n"/>
+      <c r="F14" s="40" t="n"/>
+      <c r="G14" s="60" t="n"/>
+      <c r="H14" s="91" t="n">
         <v>-60</v>
       </c>
-      <c r="Q14" s="18">
+      <c r="I14" s="60" t="n"/>
+      <c r="J14" s="60" t="n"/>
+      <c r="K14" s="60" t="n"/>
+      <c r="L14" s="60" t="n"/>
+      <c r="M14" s="60" t="n"/>
+      <c r="N14" s="60" t="n"/>
+      <c r="O14" s="60" t="n"/>
+      <c r="P14" s="60" t="n"/>
+      <c r="Q14" s="44">
         <f>IF(SUMPRODUCT(ABS(C14:P14))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="19">
-      <c r="A15" s="52" t="inlineStr">
+      <c r="A15" s="40" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5663,31 +5668,29 @@
           <t>fire</t>
         </is>
       </c>
-      <c r="C15" s="55" t="n">
+      <c r="C15" s="92" t="n">
         <v>100</v>
       </c>
-      <c r="D15" s="36" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="E15" s="36" t="inlineStr">
-        <is>
-          <t>transient</t>
-        </is>
-      </c>
-      <c r="F15" s="36" t="inlineStr">
-        <is>
-          <t>PROPOSED. Fear, at the cost of some standing</t>
-        </is>
-      </c>
-      <c r="Q15" s="18">
+      <c r="D15" s="40" t="n"/>
+      <c r="E15" s="40" t="n"/>
+      <c r="F15" s="40" t="n"/>
+      <c r="G15" s="60" t="n"/>
+      <c r="H15" s="60" t="n"/>
+      <c r="I15" s="60" t="n"/>
+      <c r="J15" s="60" t="n"/>
+      <c r="K15" s="60" t="n"/>
+      <c r="L15" s="60" t="n"/>
+      <c r="M15" s="60" t="n"/>
+      <c r="N15" s="60" t="n"/>
+      <c r="O15" s="60" t="n"/>
+      <c r="P15" s="60" t="n"/>
+      <c r="Q15" s="44">
         <f>IF(SUMPRODUCT(ABS(C15:P15))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="19">
-      <c r="A16" s="52" t="inlineStr">
+      <c r="A16" s="40" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5697,31 +5700,29 @@
           <t>frost</t>
         </is>
       </c>
-      <c r="C16" s="53" t="n">
+      <c r="C16" s="90" t="n">
         <v>-100</v>
       </c>
-      <c r="D16" s="36" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="E16" s="36" t="inlineStr">
-        <is>
-          <t>transient</t>
-        </is>
-      </c>
-      <c r="F16" s="36" t="inlineStr">
-        <is>
-          <t>PROPOSED</t>
-        </is>
-      </c>
-      <c r="Q16" s="18">
+      <c r="D16" s="40" t="n"/>
+      <c r="E16" s="40" t="n"/>
+      <c r="F16" s="40" t="n"/>
+      <c r="G16" s="60" t="n"/>
+      <c r="H16" s="60" t="n"/>
+      <c r="I16" s="60" t="n"/>
+      <c r="J16" s="60" t="n"/>
+      <c r="K16" s="60" t="n"/>
+      <c r="L16" s="60" t="n"/>
+      <c r="M16" s="60" t="n"/>
+      <c r="N16" s="60" t="n"/>
+      <c r="O16" s="60" t="n"/>
+      <c r="P16" s="60" t="n"/>
+      <c r="Q16" s="44">
         <f>IF(SUMPRODUCT(ABS(C16:P16))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="19">
-      <c r="A17" s="52" t="inlineStr">
+      <c r="A17" s="40" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5731,21 +5732,31 @@
           <t>lightning</t>
         </is>
       </c>
-      <c r="C17" s="55" t="n">
+      <c r="C17" s="92" t="n">
         <v>30</v>
       </c>
-      <c r="D17" s="53" t="n">
+      <c r="D17" s="90" t="n">
         <v>-70</v>
       </c>
-      <c r="E17" s="36" t="inlineStr"/>
-      <c r="F17" s="36" t="inlineStr"/>
-      <c r="Q17" s="18">
+      <c r="E17" s="40" t="n"/>
+      <c r="F17" s="40" t="n"/>
+      <c r="G17" s="60" t="n"/>
+      <c r="H17" s="60" t="n"/>
+      <c r="I17" s="60" t="n"/>
+      <c r="J17" s="60" t="n"/>
+      <c r="K17" s="60" t="n"/>
+      <c r="L17" s="60" t="n"/>
+      <c r="M17" s="60" t="n"/>
+      <c r="N17" s="60" t="n"/>
+      <c r="O17" s="60" t="n"/>
+      <c r="P17" s="60" t="n"/>
+      <c r="Q17" s="44">
         <f>IF(SUMPRODUCT(ABS(C17:P17))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="19">
-      <c r="A18" s="52" t="inlineStr">
+      <c r="A18" s="40" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5755,21 +5766,31 @@
           <t>blast</t>
         </is>
       </c>
-      <c r="C18" s="55" t="n">
+      <c r="C18" s="92" t="n">
         <v>50</v>
       </c>
-      <c r="D18" s="53" t="n">
+      <c r="D18" s="90" t="n">
         <v>-50</v>
       </c>
-      <c r="E18" s="36" t="inlineStr"/>
-      <c r="F18" s="36" t="inlineStr"/>
-      <c r="Q18" s="18">
+      <c r="E18" s="40" t="n"/>
+      <c r="F18" s="40" t="n"/>
+      <c r="G18" s="60" t="n"/>
+      <c r="H18" s="60" t="n"/>
+      <c r="I18" s="60" t="n"/>
+      <c r="J18" s="60" t="n"/>
+      <c r="K18" s="60" t="n"/>
+      <c r="L18" s="60" t="n"/>
+      <c r="M18" s="60" t="n"/>
+      <c r="N18" s="60" t="n"/>
+      <c r="O18" s="60" t="n"/>
+      <c r="P18" s="60" t="n"/>
+      <c r="Q18" s="44">
         <f>IF(SUMPRODUCT(ABS(C18:P18))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="19">
-      <c r="A19" s="52" t="inlineStr">
+      <c r="A19" s="40" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5779,22 +5800,31 @@
           <t>shockwave</t>
         </is>
       </c>
-      <c r="C19" s="36" t="inlineStr"/>
-      <c r="D19" s="53" t="n">
+      <c r="C19" s="40" t="n"/>
+      <c r="D19" s="90" t="n">
         <v>-60</v>
       </c>
-      <c r="E19" s="36" t="inlineStr"/>
-      <c r="F19" s="36" t="inlineStr"/>
-      <c r="I19" s="54" t="n">
+      <c r="E19" s="40" t="n"/>
+      <c r="F19" s="40" t="n"/>
+      <c r="G19" s="60" t="n"/>
+      <c r="H19" s="60" t="n"/>
+      <c r="I19" s="91" t="n">
         <v>-40</v>
       </c>
-      <c r="Q19" s="18">
+      <c r="J19" s="60" t="n"/>
+      <c r="K19" s="60" t="n"/>
+      <c r="L19" s="60" t="n"/>
+      <c r="M19" s="60" t="n"/>
+      <c r="N19" s="60" t="n"/>
+      <c r="O19" s="60" t="n"/>
+      <c r="P19" s="60" t="n"/>
+      <c r="Q19" s="44">
         <f>IF(SUMPRODUCT(ABS(C19:P19))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="19">
-      <c r="A20" s="56" t="inlineStr">
+      <c r="A20" s="57" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5804,19 +5834,29 @@
           <t>acid</t>
         </is>
       </c>
-      <c r="C20" s="37" t="n"/>
-      <c r="D20" s="37" t="n"/>
-      <c r="E20" s="51" t="n">
+      <c r="C20" s="57" t="n"/>
+      <c r="D20" s="57" t="n"/>
+      <c r="E20" s="89" t="n">
         <v>-100</v>
       </c>
-      <c r="F20" s="37" t="n"/>
-      <c r="Q20" s="18">
+      <c r="F20" s="57" t="n"/>
+      <c r="G20" s="60" t="n"/>
+      <c r="H20" s="60" t="n"/>
+      <c r="I20" s="60" t="n"/>
+      <c r="J20" s="60" t="n"/>
+      <c r="K20" s="60" t="n"/>
+      <c r="L20" s="60" t="n"/>
+      <c r="M20" s="60" t="n"/>
+      <c r="N20" s="60" t="n"/>
+      <c r="O20" s="60" t="n"/>
+      <c r="P20" s="60" t="n"/>
+      <c r="Q20" s="44">
         <f>IF(SUMPRODUCT(ABS(C20:P20))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="19">
-      <c r="A21" s="56" t="inlineStr">
+      <c r="A21" s="57" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5826,21 +5866,31 @@
           <t>molten</t>
         </is>
       </c>
-      <c r="C21" s="58" t="n">
+      <c r="C21" s="93" t="n">
         <v>50</v>
       </c>
-      <c r="D21" s="37" t="n"/>
-      <c r="E21" s="51" t="n">
+      <c r="D21" s="57" t="n"/>
+      <c r="E21" s="89" t="n">
         <v>-50</v>
       </c>
-      <c r="F21" s="37" t="n"/>
-      <c r="Q21" s="18">
+      <c r="F21" s="57" t="n"/>
+      <c r="G21" s="60" t="n"/>
+      <c r="H21" s="60" t="n"/>
+      <c r="I21" s="60" t="n"/>
+      <c r="J21" s="60" t="n"/>
+      <c r="K21" s="60" t="n"/>
+      <c r="L21" s="60" t="n"/>
+      <c r="M21" s="60" t="n"/>
+      <c r="N21" s="60" t="n"/>
+      <c r="O21" s="60" t="n"/>
+      <c r="P21" s="60" t="n"/>
+      <c r="Q21" s="44">
         <f>IF(SUMPRODUCT(ABS(C21:P21))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="19">
-      <c r="A22" s="56" t="inlineStr">
+      <c r="A22" s="57" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5850,21 +5900,31 @@
           <t>scald</t>
         </is>
       </c>
-      <c r="C22" s="58" t="n">
+      <c r="C22" s="93" t="n">
         <v>60</v>
       </c>
-      <c r="D22" s="37" t="n"/>
-      <c r="E22" s="37" t="n"/>
-      <c r="F22" s="51" t="n">
+      <c r="D22" s="57" t="n"/>
+      <c r="E22" s="57" t="n"/>
+      <c r="F22" s="89" t="n">
         <v>-40</v>
       </c>
-      <c r="Q22" s="18">
+      <c r="G22" s="60" t="n"/>
+      <c r="H22" s="60" t="n"/>
+      <c r="I22" s="60" t="n"/>
+      <c r="J22" s="60" t="n"/>
+      <c r="K22" s="60" t="n"/>
+      <c r="L22" s="60" t="n"/>
+      <c r="M22" s="60" t="n"/>
+      <c r="N22" s="60" t="n"/>
+      <c r="O22" s="60" t="n"/>
+      <c r="P22" s="60" t="n"/>
+      <c r="Q22" s="44">
         <f>IF(SUMPRODUCT(ABS(C22:P22))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="19">
-      <c r="A23" s="56" t="inlineStr">
+      <c r="A23" s="57" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5874,21 +5934,31 @@
           <t>frostbite</t>
         </is>
       </c>
-      <c r="C23" s="51" t="n">
+      <c r="C23" s="89" t="n">
         <v>-50</v>
       </c>
-      <c r="D23" s="37" t="n"/>
-      <c r="E23" s="37" t="n"/>
-      <c r="F23" s="51" t="n">
+      <c r="D23" s="57" t="n"/>
+      <c r="E23" s="57" t="n"/>
+      <c r="F23" s="89" t="n">
         <v>-50</v>
       </c>
-      <c r="Q23" s="18">
+      <c r="G23" s="60" t="n"/>
+      <c r="H23" s="60" t="n"/>
+      <c r="I23" s="60" t="n"/>
+      <c r="J23" s="60" t="n"/>
+      <c r="K23" s="60" t="n"/>
+      <c r="L23" s="60" t="n"/>
+      <c r="M23" s="60" t="n"/>
+      <c r="N23" s="60" t="n"/>
+      <c r="O23" s="60" t="n"/>
+      <c r="P23" s="60" t="n"/>
+      <c r="Q23" s="44">
         <f>IF(SUMPRODUCT(ABS(C23:P23))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="19">
-      <c r="A24" s="56" t="inlineStr">
+      <c r="A24" s="57" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5898,22 +5968,31 @@
           <t>exposure</t>
         </is>
       </c>
-      <c r="C24" s="51" t="n">
+      <c r="C24" s="89" t="n">
         <v>-40</v>
       </c>
-      <c r="D24" s="37" t="n"/>
-      <c r="E24" s="37" t="n"/>
-      <c r="F24" s="37" t="n"/>
-      <c r="G24" s="54" t="n">
+      <c r="D24" s="57" t="n"/>
+      <c r="E24" s="57" t="n"/>
+      <c r="F24" s="57" t="n"/>
+      <c r="G24" s="91" t="n">
         <v>-60</v>
       </c>
-      <c r="Q24" s="18">
+      <c r="H24" s="60" t="n"/>
+      <c r="I24" s="60" t="n"/>
+      <c r="J24" s="60" t="n"/>
+      <c r="K24" s="60" t="n"/>
+      <c r="L24" s="60" t="n"/>
+      <c r="M24" s="60" t="n"/>
+      <c r="N24" s="60" t="n"/>
+      <c r="O24" s="60" t="n"/>
+      <c r="P24" s="60" t="n"/>
+      <c r="Q24" s="44">
         <f>IF(SUMPRODUCT(ABS(C24:P24))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="19">
-      <c r="A25" s="56" t="inlineStr">
+      <c r="A25" s="57" t="inlineStr">
         <is>
           <t>ELEMENTS</t>
         </is>
@@ -5923,23 +6002,31 @@
           <t>flash</t>
         </is>
       </c>
-      <c r="C25" s="37" t="n"/>
-      <c r="D25" s="37" t="n"/>
-      <c r="E25" s="37" t="n"/>
-      <c r="F25" s="37" t="n"/>
-      <c r="I25" s="54" t="n">
+      <c r="C25" s="57" t="n"/>
+      <c r="D25" s="57" t="n"/>
+      <c r="E25" s="57" t="n"/>
+      <c r="F25" s="57" t="n"/>
+      <c r="G25" s="60" t="n"/>
+      <c r="H25" s="60" t="n"/>
+      <c r="I25" s="91" t="n">
         <v>-70</v>
       </c>
-      <c r="K25" s="54" t="n">
+      <c r="J25" s="60" t="n"/>
+      <c r="K25" s="91" t="n">
         <v>-30</v>
       </c>
-      <c r="Q25" s="18">
+      <c r="L25" s="60" t="n"/>
+      <c r="M25" s="60" t="n"/>
+      <c r="N25" s="60" t="n"/>
+      <c r="O25" s="60" t="n"/>
+      <c r="P25" s="60" t="n"/>
+      <c r="Q25" s="44">
         <f>IF(SUMPRODUCT(ABS(C25:P25))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="19">
-      <c r="A26" s="56" t="inlineStr">
+      <c r="A26" s="57" t="inlineStr">
         <is>
           <t>AFFLICTION</t>
         </is>
@@ -5949,22 +6036,31 @@
           <t>venom</t>
         </is>
       </c>
-      <c r="C26" s="37" t="n"/>
-      <c r="D26" s="37" t="n"/>
-      <c r="E26" s="37" t="n"/>
-      <c r="F26" s="51" t="n">
+      <c r="C26" s="57" t="n"/>
+      <c r="D26" s="57" t="n"/>
+      <c r="E26" s="57" t="n"/>
+      <c r="F26" s="89" t="n">
         <v>-70</v>
       </c>
-      <c r="K26" s="54" t="n">
+      <c r="G26" s="60" t="n"/>
+      <c r="H26" s="60" t="n"/>
+      <c r="I26" s="60" t="n"/>
+      <c r="J26" s="60" t="n"/>
+      <c r="K26" s="91" t="n">
         <v>-30</v>
       </c>
-      <c r="Q26" s="18">
+      <c r="L26" s="60" t="n"/>
+      <c r="M26" s="60" t="n"/>
+      <c r="N26" s="60" t="n"/>
+      <c r="O26" s="60" t="n"/>
+      <c r="P26" s="60" t="n"/>
+      <c r="Q26" s="44">
         <f>IF(SUMPRODUCT(ABS(C26:P26))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="19">
-      <c r="A27" s="56" t="inlineStr">
+      <c r="A27" s="57" t="inlineStr">
         <is>
           <t>AFFLICTION</t>
         </is>
@@ -5974,21 +6070,31 @@
           <t>blight</t>
         </is>
       </c>
-      <c r="C27" s="37" t="n"/>
-      <c r="D27" s="37" t="n"/>
-      <c r="E27" s="51" t="n">
+      <c r="C27" s="57" t="n"/>
+      <c r="D27" s="57" t="n"/>
+      <c r="E27" s="89" t="n">
         <v>-50</v>
       </c>
-      <c r="F27" s="51" t="n">
+      <c r="F27" s="89" t="n">
         <v>-50</v>
       </c>
-      <c r="Q27" s="18">
+      <c r="G27" s="60" t="n"/>
+      <c r="H27" s="60" t="n"/>
+      <c r="I27" s="60" t="n"/>
+      <c r="J27" s="60" t="n"/>
+      <c r="K27" s="60" t="n"/>
+      <c r="L27" s="60" t="n"/>
+      <c r="M27" s="60" t="n"/>
+      <c r="N27" s="60" t="n"/>
+      <c r="O27" s="60" t="n"/>
+      <c r="P27" s="60" t="n"/>
+      <c r="Q27" s="44">
         <f>IF(SUMPRODUCT(ABS(C27:P27))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="19">
-      <c r="A28" s="56" t="inlineStr">
+      <c r="A28" s="57" t="inlineStr">
         <is>
           <t>AFFLICTION</t>
         </is>
@@ -5998,22 +6104,31 @@
           <t>agony</t>
         </is>
       </c>
-      <c r="C28" s="37" t="n"/>
-      <c r="D28" s="37" t="n"/>
-      <c r="E28" s="37" t="n"/>
-      <c r="F28" s="51" t="n">
+      <c r="C28" s="57" t="n"/>
+      <c r="D28" s="57" t="n"/>
+      <c r="E28" s="57" t="n"/>
+      <c r="F28" s="89" t="n">
         <v>-50</v>
       </c>
-      <c r="K28" s="54" t="n">
+      <c r="G28" s="60" t="n"/>
+      <c r="H28" s="60" t="n"/>
+      <c r="I28" s="60" t="n"/>
+      <c r="J28" s="60" t="n"/>
+      <c r="K28" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q28" s="18">
+      <c r="L28" s="60" t="n"/>
+      <c r="M28" s="60" t="n"/>
+      <c r="N28" s="60" t="n"/>
+      <c r="O28" s="60" t="n"/>
+      <c r="P28" s="60" t="n"/>
+      <c r="Q28" s="44">
         <f>IF(SUMPRODUCT(ABS(C28:P28))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="19">
-      <c r="A29" s="56" t="inlineStr">
+      <c r="A29" s="57" t="inlineStr">
         <is>
           <t>AFFLICTION</t>
         </is>
@@ -6023,23 +6138,31 @@
           <t>fatigue</t>
         </is>
       </c>
-      <c r="C29" s="37" t="n"/>
-      <c r="D29" s="37" t="n"/>
-      <c r="E29" s="37" t="n"/>
-      <c r="F29" s="37" t="n"/>
-      <c r="G29" s="54" t="n">
+      <c r="C29" s="57" t="n"/>
+      <c r="D29" s="57" t="n"/>
+      <c r="E29" s="57" t="n"/>
+      <c r="F29" s="57" t="n"/>
+      <c r="G29" s="91" t="n">
         <v>-70</v>
       </c>
-      <c r="J29" s="54" t="n">
+      <c r="H29" s="60" t="n"/>
+      <c r="I29" s="60" t="n"/>
+      <c r="J29" s="91" t="n">
         <v>-30</v>
       </c>
-      <c r="Q29" s="18">
+      <c r="K29" s="60" t="n"/>
+      <c r="L29" s="60" t="n"/>
+      <c r="M29" s="60" t="n"/>
+      <c r="N29" s="60" t="n"/>
+      <c r="O29" s="60" t="n"/>
+      <c r="P29" s="60" t="n"/>
+      <c r="Q29" s="44">
         <f>IF(SUMPRODUCT(ABS(C29:P29))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="19">
-      <c r="A30" s="56" t="inlineStr">
+      <c r="A30" s="57" t="inlineStr">
         <is>
           <t>AFFLICTION</t>
         </is>
@@ -6049,22 +6172,31 @@
           <t>wither</t>
         </is>
       </c>
-      <c r="C30" s="37" t="n"/>
-      <c r="D30" s="37" t="n"/>
-      <c r="E30" s="37" t="n"/>
-      <c r="F30" s="51" t="n">
+      <c r="C30" s="57" t="n"/>
+      <c r="D30" s="57" t="n"/>
+      <c r="E30" s="57" t="n"/>
+      <c r="F30" s="89" t="n">
         <v>-60</v>
       </c>
-      <c r="G30" s="54" t="n">
+      <c r="G30" s="91" t="n">
         <v>-40</v>
       </c>
-      <c r="Q30" s="18">
+      <c r="H30" s="60" t="n"/>
+      <c r="I30" s="60" t="n"/>
+      <c r="J30" s="60" t="n"/>
+      <c r="K30" s="60" t="n"/>
+      <c r="L30" s="60" t="n"/>
+      <c r="M30" s="60" t="n"/>
+      <c r="N30" s="60" t="n"/>
+      <c r="O30" s="60" t="n"/>
+      <c r="P30" s="60" t="n"/>
+      <c r="Q30" s="44">
         <f>IF(SUMPRODUCT(ABS(C30:P30))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="19">
-      <c r="A31" s="56" t="inlineStr">
+      <c r="A31" s="57" t="inlineStr">
         <is>
           <t>AFFLICTION</t>
         </is>
@@ -6074,22 +6206,31 @@
           <t>rot</t>
         </is>
       </c>
-      <c r="C31" s="37" t="n"/>
-      <c r="D31" s="37" t="n"/>
-      <c r="E31" s="51" t="n">
+      <c r="C31" s="57" t="n"/>
+      <c r="D31" s="57" t="n"/>
+      <c r="E31" s="89" t="n">
         <v>-60</v>
       </c>
-      <c r="F31" s="37" t="n"/>
-      <c r="G31" s="54" t="n">
+      <c r="F31" s="57" t="n"/>
+      <c r="G31" s="91" t="n">
         <v>-40</v>
       </c>
-      <c r="Q31" s="18">
+      <c r="H31" s="60" t="n"/>
+      <c r="I31" s="60" t="n"/>
+      <c r="J31" s="60" t="n"/>
+      <c r="K31" s="60" t="n"/>
+      <c r="L31" s="60" t="n"/>
+      <c r="M31" s="60" t="n"/>
+      <c r="N31" s="60" t="n"/>
+      <c r="O31" s="60" t="n"/>
+      <c r="P31" s="60" t="n"/>
+      <c r="Q31" s="44">
         <f>IF(SUMPRODUCT(ABS(C31:P31))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="19">
-      <c r="A32" s="56" t="inlineStr">
+      <c r="A32" s="57" t="inlineStr">
         <is>
           <t>AFFLICTION</t>
         </is>
@@ -6099,23 +6240,31 @@
           <t>numb</t>
         </is>
       </c>
-      <c r="C32" s="37" t="n"/>
-      <c r="D32" s="37" t="n"/>
-      <c r="E32" s="37" t="n"/>
-      <c r="F32" s="37" t="n"/>
-      <c r="H32" s="54" t="n">
+      <c r="C32" s="57" t="n"/>
+      <c r="D32" s="57" t="n"/>
+      <c r="E32" s="57" t="n"/>
+      <c r="F32" s="57" t="n"/>
+      <c r="G32" s="60" t="n"/>
+      <c r="H32" s="91" t="n">
         <v>-40</v>
       </c>
-      <c r="I32" s="54" t="n">
+      <c r="I32" s="91" t="n">
         <v>-60</v>
       </c>
-      <c r="Q32" s="18">
+      <c r="J32" s="60" t="n"/>
+      <c r="K32" s="60" t="n"/>
+      <c r="L32" s="60" t="n"/>
+      <c r="M32" s="60" t="n"/>
+      <c r="N32" s="60" t="n"/>
+      <c r="O32" s="60" t="n"/>
+      <c r="P32" s="60" t="n"/>
+      <c r="Q32" s="44">
         <f>IF(SUMPRODUCT(ABS(C32:P32))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="19">
-      <c r="A33" s="56" t="inlineStr">
+      <c r="A33" s="57" t="inlineStr">
         <is>
           <t>BINDING &amp; MOVEMENT</t>
         </is>
@@ -6125,20 +6274,29 @@
           <t>slow</t>
         </is>
       </c>
-      <c r="C33" s="37" t="n"/>
-      <c r="D33" s="37" t="n"/>
-      <c r="E33" s="37" t="n"/>
-      <c r="F33" s="37" t="n"/>
-      <c r="H33" s="54" t="n">
+      <c r="C33" s="57" t="n"/>
+      <c r="D33" s="57" t="n"/>
+      <c r="E33" s="57" t="n"/>
+      <c r="F33" s="57" t="n"/>
+      <c r="G33" s="60" t="n"/>
+      <c r="H33" s="91" t="n">
         <v>-100</v>
       </c>
-      <c r="Q33" s="18">
+      <c r="I33" s="60" t="n"/>
+      <c r="J33" s="60" t="n"/>
+      <c r="K33" s="60" t="n"/>
+      <c r="L33" s="60" t="n"/>
+      <c r="M33" s="60" t="n"/>
+      <c r="N33" s="60" t="n"/>
+      <c r="O33" s="60" t="n"/>
+      <c r="P33" s="60" t="n"/>
+      <c r="Q33" s="44">
         <f>IF(SUMPRODUCT(ABS(C33:P33))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="19">
-      <c r="A34" s="56" t="inlineStr">
+      <c r="A34" s="57" t="inlineStr">
         <is>
           <t>BINDING &amp; MOVEMENT</t>
         </is>
@@ -6148,23 +6306,31 @@
           <t>entangle</t>
         </is>
       </c>
-      <c r="C34" s="37" t="n"/>
-      <c r="D34" s="37" t="n"/>
-      <c r="E34" s="37" t="n"/>
-      <c r="F34" s="37" t="n"/>
-      <c r="G34" s="54" t="n">
+      <c r="C34" s="57" t="n"/>
+      <c r="D34" s="57" t="n"/>
+      <c r="E34" s="57" t="n"/>
+      <c r="F34" s="57" t="n"/>
+      <c r="G34" s="91" t="n">
         <v>-30</v>
       </c>
-      <c r="H34" s="54" t="n">
+      <c r="H34" s="91" t="n">
         <v>-70</v>
       </c>
-      <c r="Q34" s="18">
+      <c r="I34" s="60" t="n"/>
+      <c r="J34" s="60" t="n"/>
+      <c r="K34" s="60" t="n"/>
+      <c r="L34" s="60" t="n"/>
+      <c r="M34" s="60" t="n"/>
+      <c r="N34" s="60" t="n"/>
+      <c r="O34" s="60" t="n"/>
+      <c r="P34" s="60" t="n"/>
+      <c r="Q34" s="44">
         <f>IF(SUMPRODUCT(ABS(C34:P34))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="19">
-      <c r="A35" s="56" t="inlineStr">
+      <c r="A35" s="57" t="inlineStr">
         <is>
           <t>BINDING &amp; MOVEMENT</t>
         </is>
@@ -6174,22 +6340,31 @@
           <t>snare</t>
         </is>
       </c>
-      <c r="C35" s="37" t="n"/>
-      <c r="D35" s="37" t="n"/>
-      <c r="E35" s="37" t="n"/>
-      <c r="F35" s="51" t="n">
+      <c r="C35" s="57" t="n"/>
+      <c r="D35" s="57" t="n"/>
+      <c r="E35" s="57" t="n"/>
+      <c r="F35" s="89" t="n">
         <v>-20</v>
       </c>
-      <c r="H35" s="54" t="n">
+      <c r="G35" s="60" t="n"/>
+      <c r="H35" s="91" t="n">
         <v>-80</v>
       </c>
-      <c r="Q35" s="18">
+      <c r="I35" s="60" t="n"/>
+      <c r="J35" s="60" t="n"/>
+      <c r="K35" s="60" t="n"/>
+      <c r="L35" s="60" t="n"/>
+      <c r="M35" s="60" t="n"/>
+      <c r="N35" s="60" t="n"/>
+      <c r="O35" s="60" t="n"/>
+      <c r="P35" s="60" t="n"/>
+      <c r="Q35" s="44">
         <f>IF(SUMPRODUCT(ABS(C35:P35))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="19">
-      <c r="A36" s="56" t="inlineStr">
+      <c r="A36" s="57" t="inlineStr">
         <is>
           <t>BINDING &amp; MOVEMENT</t>
         </is>
@@ -6199,22 +6374,31 @@
           <t>cripple</t>
         </is>
       </c>
-      <c r="C36" s="37" t="n"/>
-      <c r="D36" s="37" t="n"/>
-      <c r="E36" s="37" t="n"/>
-      <c r="F36" s="51" t="n">
+      <c r="C36" s="57" t="n"/>
+      <c r="D36" s="57" t="n"/>
+      <c r="E36" s="57" t="n"/>
+      <c r="F36" s="89" t="n">
         <v>-40</v>
       </c>
-      <c r="H36" s="54" t="n">
+      <c r="G36" s="60" t="n"/>
+      <c r="H36" s="91" t="n">
         <v>-60</v>
       </c>
-      <c r="Q36" s="18">
+      <c r="I36" s="60" t="n"/>
+      <c r="J36" s="60" t="n"/>
+      <c r="K36" s="60" t="n"/>
+      <c r="L36" s="60" t="n"/>
+      <c r="M36" s="60" t="n"/>
+      <c r="N36" s="60" t="n"/>
+      <c r="O36" s="60" t="n"/>
+      <c r="P36" s="60" t="n"/>
+      <c r="Q36" s="44">
         <f>IF(SUMPRODUCT(ABS(C36:P36))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="19">
-      <c r="A37" s="56" t="inlineStr">
+      <c r="A37" s="57" t="inlineStr">
         <is>
           <t>BINDING &amp; MOVEMENT</t>
         </is>
@@ -6224,22 +6408,31 @@
           <t>pin</t>
         </is>
       </c>
-      <c r="C37" s="37" t="n"/>
-      <c r="D37" s="51" t="n">
+      <c r="C37" s="57" t="n"/>
+      <c r="D37" s="89" t="n">
         <v>-50</v>
       </c>
-      <c r="E37" s="37" t="n"/>
-      <c r="F37" s="37" t="n"/>
-      <c r="H37" s="54" t="n">
+      <c r="E37" s="57" t="n"/>
+      <c r="F37" s="57" t="n"/>
+      <c r="G37" s="60" t="n"/>
+      <c r="H37" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q37" s="18">
+      <c r="I37" s="60" t="n"/>
+      <c r="J37" s="60" t="n"/>
+      <c r="K37" s="60" t="n"/>
+      <c r="L37" s="60" t="n"/>
+      <c r="M37" s="60" t="n"/>
+      <c r="N37" s="60" t="n"/>
+      <c r="O37" s="60" t="n"/>
+      <c r="P37" s="60" t="n"/>
+      <c r="Q37" s="44">
         <f>IF(SUMPRODUCT(ABS(C37:P37))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="19">
-      <c r="A38" s="56" t="inlineStr">
+      <c r="A38" s="57" t="inlineStr">
         <is>
           <t>BINDING &amp; MOVEMENT</t>
         </is>
@@ -6249,22 +6442,31 @@
           <t>petrify</t>
         </is>
       </c>
-      <c r="C38" s="37" t="n"/>
-      <c r="D38" s="58" t="n">
+      <c r="C38" s="57" t="n"/>
+      <c r="D38" s="93" t="n">
         <v>40</v>
       </c>
-      <c r="E38" s="37" t="n"/>
-      <c r="F38" s="37" t="n"/>
-      <c r="H38" s="54" t="n">
+      <c r="E38" s="57" t="n"/>
+      <c r="F38" s="57" t="n"/>
+      <c r="G38" s="60" t="n"/>
+      <c r="H38" s="91" t="n">
         <v>-60</v>
       </c>
-      <c r="Q38" s="18">
+      <c r="I38" s="60" t="n"/>
+      <c r="J38" s="60" t="n"/>
+      <c r="K38" s="60" t="n"/>
+      <c r="L38" s="60" t="n"/>
+      <c r="M38" s="60" t="n"/>
+      <c r="N38" s="60" t="n"/>
+      <c r="O38" s="60" t="n"/>
+      <c r="P38" s="60" t="n"/>
+      <c r="Q38" s="44">
         <f>IF(SUMPRODUCT(ABS(C38:P38))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="19">
-      <c r="A39" s="56" t="inlineStr">
+      <c r="A39" s="57" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6274,20 +6476,29 @@
           <t>dread</t>
         </is>
       </c>
-      <c r="C39" s="37" t="n"/>
-      <c r="D39" s="37" t="n"/>
-      <c r="E39" s="37" t="n"/>
-      <c r="F39" s="37" t="n"/>
-      <c r="J39" s="54" t="n">
+      <c r="C39" s="57" t="n"/>
+      <c r="D39" s="57" t="n"/>
+      <c r="E39" s="57" t="n"/>
+      <c r="F39" s="57" t="n"/>
+      <c r="G39" s="60" t="n"/>
+      <c r="H39" s="60" t="n"/>
+      <c r="I39" s="60" t="n"/>
+      <c r="J39" s="91" t="n">
         <v>-100</v>
       </c>
-      <c r="Q39" s="18">
+      <c r="K39" s="60" t="n"/>
+      <c r="L39" s="60" t="n"/>
+      <c r="M39" s="60" t="n"/>
+      <c r="N39" s="60" t="n"/>
+      <c r="O39" s="60" t="n"/>
+      <c r="P39" s="60" t="n"/>
+      <c r="Q39" s="44">
         <f>IF(SUMPRODUCT(ABS(C39:P39))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="19">
-      <c r="A40" s="56" t="inlineStr">
+      <c r="A40" s="57" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6297,23 +6508,31 @@
           <t>terror</t>
         </is>
       </c>
-      <c r="C40" s="37" t="n"/>
-      <c r="D40" s="37" t="n"/>
-      <c r="E40" s="37" t="n"/>
-      <c r="F40" s="37" t="n"/>
-      <c r="G40" s="54" t="n">
+      <c r="C40" s="57" t="n"/>
+      <c r="D40" s="57" t="n"/>
+      <c r="E40" s="57" t="n"/>
+      <c r="F40" s="57" t="n"/>
+      <c r="G40" s="91" t="n">
         <v>-30</v>
       </c>
-      <c r="J40" s="54" t="n">
+      <c r="H40" s="60" t="n"/>
+      <c r="I40" s="60" t="n"/>
+      <c r="J40" s="91" t="n">
         <v>-70</v>
       </c>
-      <c r="Q40" s="18">
+      <c r="K40" s="60" t="n"/>
+      <c r="L40" s="60" t="n"/>
+      <c r="M40" s="60" t="n"/>
+      <c r="N40" s="60" t="n"/>
+      <c r="O40" s="60" t="n"/>
+      <c r="P40" s="60" t="n"/>
+      <c r="Q40" s="44">
         <f>IF(SUMPRODUCT(ABS(C40:P40))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="19">
-      <c r="A41" s="56" t="inlineStr">
+      <c r="A41" s="57" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6323,20 +6542,29 @@
           <t>confusion</t>
         </is>
       </c>
-      <c r="C41" s="37" t="n"/>
-      <c r="D41" s="37" t="n"/>
-      <c r="E41" s="37" t="n"/>
-      <c r="F41" s="37" t="n"/>
-      <c r="K41" s="54" t="n">
+      <c r="C41" s="57" t="n"/>
+      <c r="D41" s="57" t="n"/>
+      <c r="E41" s="57" t="n"/>
+      <c r="F41" s="57" t="n"/>
+      <c r="G41" s="60" t="n"/>
+      <c r="H41" s="60" t="n"/>
+      <c r="I41" s="60" t="n"/>
+      <c r="J41" s="60" t="n"/>
+      <c r="K41" s="91" t="n">
         <v>-100</v>
       </c>
-      <c r="Q41" s="18">
+      <c r="L41" s="60" t="n"/>
+      <c r="M41" s="60" t="n"/>
+      <c r="N41" s="60" t="n"/>
+      <c r="O41" s="60" t="n"/>
+      <c r="P41" s="60" t="n"/>
+      <c r="Q41" s="44">
         <f>IF(SUMPRODUCT(ABS(C41:P41))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="19">
-      <c r="A42" s="56" t="inlineStr">
+      <c r="A42" s="57" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6346,23 +6574,31 @@
           <t>panic</t>
         </is>
       </c>
-      <c r="C42" s="37" t="n"/>
-      <c r="D42" s="37" t="n"/>
-      <c r="E42" s="37" t="n"/>
-      <c r="F42" s="37" t="n"/>
-      <c r="J42" s="54" t="n">
+      <c r="C42" s="57" t="n"/>
+      <c r="D42" s="57" t="n"/>
+      <c r="E42" s="57" t="n"/>
+      <c r="F42" s="57" t="n"/>
+      <c r="G42" s="60" t="n"/>
+      <c r="H42" s="60" t="n"/>
+      <c r="I42" s="60" t="n"/>
+      <c r="J42" s="91" t="n">
         <v>-60</v>
       </c>
-      <c r="K42" s="54" t="n">
+      <c r="K42" s="91" t="n">
         <v>-40</v>
       </c>
-      <c r="Q42" s="18">
+      <c r="L42" s="60" t="n"/>
+      <c r="M42" s="60" t="n"/>
+      <c r="N42" s="60" t="n"/>
+      <c r="O42" s="60" t="n"/>
+      <c r="P42" s="60" t="n"/>
+      <c r="Q42" s="44">
         <f>IF(SUMPRODUCT(ABS(C42:P42))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="19">
-      <c r="A43" s="56" t="inlineStr">
+      <c r="A43" s="57" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6372,23 +6608,31 @@
           <t>charm</t>
         </is>
       </c>
-      <c r="C43" s="37" t="n"/>
-      <c r="D43" s="37" t="n"/>
-      <c r="E43" s="37" t="n"/>
-      <c r="F43" s="37" t="n"/>
-      <c r="K43" s="54" t="n">
+      <c r="C43" s="57" t="n"/>
+      <c r="D43" s="57" t="n"/>
+      <c r="E43" s="57" t="n"/>
+      <c r="F43" s="57" t="n"/>
+      <c r="G43" s="60" t="n"/>
+      <c r="H43" s="60" t="n"/>
+      <c r="I43" s="60" t="n"/>
+      <c r="J43" s="60" t="n"/>
+      <c r="K43" s="91" t="n">
         <v>-30</v>
       </c>
-      <c r="L43" s="54" t="n">
+      <c r="L43" s="91" t="n">
         <v>-70</v>
       </c>
-      <c r="Q43" s="18">
+      <c r="M43" s="60" t="n"/>
+      <c r="N43" s="60" t="n"/>
+      <c r="O43" s="60" t="n"/>
+      <c r="P43" s="60" t="n"/>
+      <c r="Q43" s="44">
         <f>IF(SUMPRODUCT(ABS(C43:P43))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="19">
-      <c r="A44" s="56" t="inlineStr">
+      <c r="A44" s="57" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6398,20 +6642,29 @@
           <t>domination</t>
         </is>
       </c>
-      <c r="C44" s="37" t="n"/>
-      <c r="D44" s="37" t="n"/>
-      <c r="E44" s="37" t="n"/>
-      <c r="F44" s="37" t="n"/>
-      <c r="L44" s="54" t="n">
+      <c r="C44" s="57" t="n"/>
+      <c r="D44" s="57" t="n"/>
+      <c r="E44" s="57" t="n"/>
+      <c r="F44" s="57" t="n"/>
+      <c r="G44" s="60" t="n"/>
+      <c r="H44" s="60" t="n"/>
+      <c r="I44" s="60" t="n"/>
+      <c r="J44" s="60" t="n"/>
+      <c r="K44" s="60" t="n"/>
+      <c r="L44" s="91" t="n">
         <v>-100</v>
       </c>
-      <c r="Q44" s="18">
+      <c r="M44" s="60" t="n"/>
+      <c r="N44" s="60" t="n"/>
+      <c r="O44" s="60" t="n"/>
+      <c r="P44" s="60" t="n"/>
+      <c r="Q44" s="44">
         <f>IF(SUMPRODUCT(ABS(C44:P44))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="19">
-      <c r="A45" s="56" t="inlineStr">
+      <c r="A45" s="57" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6421,23 +6674,31 @@
           <t>despair</t>
         </is>
       </c>
-      <c r="C45" s="37" t="n"/>
-      <c r="D45" s="37" t="n"/>
-      <c r="E45" s="37" t="n"/>
-      <c r="F45" s="37" t="n"/>
-      <c r="J45" s="54" t="n">
+      <c r="C45" s="57" t="n"/>
+      <c r="D45" s="57" t="n"/>
+      <c r="E45" s="57" t="n"/>
+      <c r="F45" s="57" t="n"/>
+      <c r="G45" s="60" t="n"/>
+      <c r="H45" s="60" t="n"/>
+      <c r="I45" s="60" t="n"/>
+      <c r="J45" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="L45" s="54" t="n">
+      <c r="K45" s="60" t="n"/>
+      <c r="L45" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q45" s="18">
+      <c r="M45" s="60" t="n"/>
+      <c r="N45" s="60" t="n"/>
+      <c r="O45" s="60" t="n"/>
+      <c r="P45" s="60" t="n"/>
+      <c r="Q45" s="44">
         <f>IF(SUMPRODUCT(ABS(C45:P45))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="19">
-      <c r="A46" s="56" t="inlineStr">
+      <c r="A46" s="57" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6447,23 +6708,31 @@
           <t>compel</t>
         </is>
       </c>
-      <c r="C46" s="37" t="n"/>
-      <c r="D46" s="37" t="n"/>
-      <c r="E46" s="37" t="n"/>
-      <c r="F46" s="37" t="n"/>
-      <c r="L46" s="54" t="n">
+      <c r="C46" s="57" t="n"/>
+      <c r="D46" s="57" t="n"/>
+      <c r="E46" s="57" t="n"/>
+      <c r="F46" s="57" t="n"/>
+      <c r="G46" s="60" t="n"/>
+      <c r="H46" s="60" t="n"/>
+      <c r="I46" s="60" t="n"/>
+      <c r="J46" s="60" t="n"/>
+      <c r="K46" s="60" t="n"/>
+      <c r="L46" s="91" t="n">
         <v>-60</v>
       </c>
-      <c r="N46" s="54" t="n">
+      <c r="M46" s="60" t="n"/>
+      <c r="N46" s="91" t="n">
         <v>-40</v>
       </c>
-      <c r="Q46" s="18">
+      <c r="O46" s="60" t="n"/>
+      <c r="P46" s="60" t="n"/>
+      <c r="Q46" s="44">
         <f>IF(SUMPRODUCT(ABS(C46:P46))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="19">
-      <c r="A47" s="56" t="inlineStr">
+      <c r="A47" s="57" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6473,23 +6742,31 @@
           <t>daze</t>
         </is>
       </c>
-      <c r="C47" s="37" t="n"/>
-      <c r="D47" s="37" t="n"/>
-      <c r="E47" s="37" t="n"/>
-      <c r="F47" s="37" t="n"/>
-      <c r="I47" s="54" t="n">
+      <c r="C47" s="57" t="n"/>
+      <c r="D47" s="57" t="n"/>
+      <c r="E47" s="57" t="n"/>
+      <c r="F47" s="57" t="n"/>
+      <c r="G47" s="60" t="n"/>
+      <c r="H47" s="60" t="n"/>
+      <c r="I47" s="91" t="n">
         <v>-40</v>
       </c>
-      <c r="K47" s="54" t="n">
+      <c r="J47" s="60" t="n"/>
+      <c r="K47" s="91" t="n">
         <v>-60</v>
       </c>
-      <c r="Q47" s="18">
+      <c r="L47" s="60" t="n"/>
+      <c r="M47" s="60" t="n"/>
+      <c r="N47" s="60" t="n"/>
+      <c r="O47" s="60" t="n"/>
+      <c r="P47" s="60" t="n"/>
+      <c r="Q47" s="44">
         <f>IF(SUMPRODUCT(ABS(C47:P47))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="59" t="inlineStr">
+      <c r="A48" s="60" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6499,19 +6776,31 @@
           <t>madness</t>
         </is>
       </c>
-      <c r="J48" s="54" t="n">
+      <c r="C48" s="60" t="n"/>
+      <c r="D48" s="60" t="n"/>
+      <c r="E48" s="60" t="n"/>
+      <c r="F48" s="60" t="n"/>
+      <c r="G48" s="60" t="n"/>
+      <c r="H48" s="60" t="n"/>
+      <c r="I48" s="60" t="n"/>
+      <c r="J48" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="K48" s="54" t="n">
+      <c r="K48" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q48" s="18">
+      <c r="L48" s="60" t="n"/>
+      <c r="M48" s="60" t="n"/>
+      <c r="N48" s="60" t="n"/>
+      <c r="O48" s="60" t="n"/>
+      <c r="P48" s="60" t="n"/>
+      <c r="Q48" s="44">
         <f>IF(SUMPRODUCT(ABS(C48:P48))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="59" t="inlineStr">
+      <c r="A49" s="60" t="inlineStr">
         <is>
           <t>FEAR &amp; MIND</t>
         </is>
@@ -6521,19 +6810,31 @@
           <t>transfix</t>
         </is>
       </c>
-      <c r="H49" s="54" t="n">
+      <c r="C49" s="60" t="n"/>
+      <c r="D49" s="60" t="n"/>
+      <c r="E49" s="60" t="n"/>
+      <c r="F49" s="60" t="n"/>
+      <c r="G49" s="60" t="n"/>
+      <c r="H49" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="J49" s="54" t="n">
+      <c r="I49" s="60" t="n"/>
+      <c r="J49" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q49" s="18">
+      <c r="K49" s="60" t="n"/>
+      <c r="L49" s="60" t="n"/>
+      <c r="M49" s="60" t="n"/>
+      <c r="N49" s="60" t="n"/>
+      <c r="O49" s="60" t="n"/>
+      <c r="P49" s="60" t="n"/>
+      <c r="Q49" s="44">
         <f>IF(SUMPRODUCT(ABS(C49:P49))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="59" t="inlineStr">
+      <c r="A50" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6543,16 +6844,29 @@
           <t>praise</t>
         </is>
       </c>
-      <c r="M50" s="61" t="n">
+      <c r="C50" s="60" t="n"/>
+      <c r="D50" s="60" t="n"/>
+      <c r="E50" s="60" t="n"/>
+      <c r="F50" s="60" t="n"/>
+      <c r="G50" s="60" t="n"/>
+      <c r="H50" s="60" t="n"/>
+      <c r="I50" s="60" t="n"/>
+      <c r="J50" s="60" t="n"/>
+      <c r="K50" s="60" t="n"/>
+      <c r="L50" s="60" t="n"/>
+      <c r="M50" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q50" s="18">
+      <c r="N50" s="60" t="n"/>
+      <c r="O50" s="60" t="n"/>
+      <c r="P50" s="60" t="n"/>
+      <c r="Q50" s="44">
         <f>IF(SUMPRODUCT(ABS(C50:P50))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="59" t="inlineStr">
+      <c r="A51" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6562,16 +6876,29 @@
           <t>scorn</t>
         </is>
       </c>
-      <c r="M51" s="54" t="n">
+      <c r="C51" s="60" t="n"/>
+      <c r="D51" s="60" t="n"/>
+      <c r="E51" s="60" t="n"/>
+      <c r="F51" s="60" t="n"/>
+      <c r="G51" s="60" t="n"/>
+      <c r="H51" s="60" t="n"/>
+      <c r="I51" s="60" t="n"/>
+      <c r="J51" s="60" t="n"/>
+      <c r="K51" s="60" t="n"/>
+      <c r="L51" s="60" t="n"/>
+      <c r="M51" s="91" t="n">
         <v>-100</v>
       </c>
-      <c r="Q51" s="18">
+      <c r="N51" s="60" t="n"/>
+      <c r="O51" s="60" t="n"/>
+      <c r="P51" s="60" t="n"/>
+      <c r="Q51" s="44">
         <f>IF(SUMPRODUCT(ABS(C51:P51))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="59" t="inlineStr">
+      <c r="A52" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6581,16 +6908,29 @@
           <t>endorse</t>
         </is>
       </c>
-      <c r="N52" s="61" t="n">
+      <c r="C52" s="60" t="n"/>
+      <c r="D52" s="60" t="n"/>
+      <c r="E52" s="60" t="n"/>
+      <c r="F52" s="60" t="n"/>
+      <c r="G52" s="60" t="n"/>
+      <c r="H52" s="60" t="n"/>
+      <c r="I52" s="60" t="n"/>
+      <c r="J52" s="60" t="n"/>
+      <c r="K52" s="60" t="n"/>
+      <c r="L52" s="60" t="n"/>
+      <c r="M52" s="60" t="n"/>
+      <c r="N52" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q52" s="18">
+      <c r="O52" s="60" t="n"/>
+      <c r="P52" s="60" t="n"/>
+      <c r="Q52" s="44">
         <f>IF(SUMPRODUCT(ABS(C52:P52))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="59" t="inlineStr">
+      <c r="A53" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6600,16 +6940,29 @@
           <t>discredit</t>
         </is>
       </c>
-      <c r="N53" s="54" t="n">
+      <c r="C53" s="60" t="n"/>
+      <c r="D53" s="60" t="n"/>
+      <c r="E53" s="60" t="n"/>
+      <c r="F53" s="60" t="n"/>
+      <c r="G53" s="60" t="n"/>
+      <c r="H53" s="60" t="n"/>
+      <c r="I53" s="60" t="n"/>
+      <c r="J53" s="60" t="n"/>
+      <c r="K53" s="60" t="n"/>
+      <c r="L53" s="60" t="n"/>
+      <c r="M53" s="60" t="n"/>
+      <c r="N53" s="91" t="n">
         <v>-100</v>
       </c>
-      <c r="Q53" s="18">
+      <c r="O53" s="60" t="n"/>
+      <c r="P53" s="60" t="n"/>
+      <c r="Q53" s="44">
         <f>IF(SUMPRODUCT(ABS(C53:P53))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="59" t="inlineStr">
+      <c r="A54" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6619,19 +6972,31 @@
           <t>champion</t>
         </is>
       </c>
-      <c r="M54" s="61" t="n">
+      <c r="C54" s="60" t="n"/>
+      <c r="D54" s="60" t="n"/>
+      <c r="E54" s="60" t="n"/>
+      <c r="F54" s="60" t="n"/>
+      <c r="G54" s="60" t="n"/>
+      <c r="H54" s="60" t="n"/>
+      <c r="I54" s="60" t="n"/>
+      <c r="J54" s="60" t="n"/>
+      <c r="K54" s="60" t="n"/>
+      <c r="L54" s="60" t="n"/>
+      <c r="M54" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="N54" s="61" t="n">
+      <c r="N54" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q54" s="18">
+      <c r="O54" s="60" t="n"/>
+      <c r="P54" s="60" t="n"/>
+      <c r="Q54" s="44">
         <f>IF(SUMPRODUCT(ABS(C54:P54))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="59" t="inlineStr">
+      <c r="A55" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6641,19 +7006,31 @@
           <t>slander</t>
         </is>
       </c>
-      <c r="M55" s="54" t="n">
+      <c r="C55" s="60" t="n"/>
+      <c r="D55" s="60" t="n"/>
+      <c r="E55" s="60" t="n"/>
+      <c r="F55" s="60" t="n"/>
+      <c r="G55" s="60" t="n"/>
+      <c r="H55" s="60" t="n"/>
+      <c r="I55" s="60" t="n"/>
+      <c r="J55" s="60" t="n"/>
+      <c r="K55" s="60" t="n"/>
+      <c r="L55" s="60" t="n"/>
+      <c r="M55" s="91" t="n">
         <v>-70</v>
       </c>
-      <c r="N55" s="54" t="n">
+      <c r="N55" s="91" t="n">
         <v>-30</v>
       </c>
-      <c r="Q55" s="18">
+      <c r="O55" s="60" t="n"/>
+      <c r="P55" s="60" t="n"/>
+      <c r="Q55" s="44">
         <f>IF(SUMPRODUCT(ABS(C55:P55))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="59" t="inlineStr">
+      <c r="A56" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6663,19 +7040,31 @@
           <t>denounce</t>
         </is>
       </c>
-      <c r="M56" s="54" t="n">
+      <c r="C56" s="60" t="n"/>
+      <c r="D56" s="60" t="n"/>
+      <c r="E56" s="60" t="n"/>
+      <c r="F56" s="60" t="n"/>
+      <c r="G56" s="60" t="n"/>
+      <c r="H56" s="60" t="n"/>
+      <c r="I56" s="60" t="n"/>
+      <c r="J56" s="60" t="n"/>
+      <c r="K56" s="60" t="n"/>
+      <c r="L56" s="60" t="n"/>
+      <c r="M56" s="91" t="n">
         <v>-20</v>
       </c>
-      <c r="N56" s="54" t="n">
+      <c r="N56" s="91" t="n">
         <v>-80</v>
       </c>
-      <c r="Q56" s="18">
+      <c r="O56" s="60" t="n"/>
+      <c r="P56" s="60" t="n"/>
+      <c r="Q56" s="44">
         <f>IF(SUMPRODUCT(ABS(C56:P56))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="59" t="inlineStr">
+      <c r="A57" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6685,19 +7074,31 @@
           <t>humble</t>
         </is>
       </c>
-      <c r="M57" s="61" t="n">
+      <c r="C57" s="60" t="n"/>
+      <c r="D57" s="60" t="n"/>
+      <c r="E57" s="60" t="n"/>
+      <c r="F57" s="60" t="n"/>
+      <c r="G57" s="60" t="n"/>
+      <c r="H57" s="60" t="n"/>
+      <c r="I57" s="60" t="n"/>
+      <c r="J57" s="60" t="n"/>
+      <c r="K57" s="60" t="n"/>
+      <c r="L57" s="60" t="n"/>
+      <c r="M57" s="94" t="n">
         <v>50</v>
       </c>
-      <c r="N57" s="54" t="n">
+      <c r="N57" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q57" s="18">
+      <c r="O57" s="60" t="n"/>
+      <c r="P57" s="60" t="n"/>
+      <c r="Q57" s="44">
         <f>IF(SUMPRODUCT(ABS(C57:P57))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="59" t="inlineStr">
+      <c r="A58" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6707,19 +7108,31 @@
           <t>menace</t>
         </is>
       </c>
-      <c r="M58" s="54" t="n">
+      <c r="C58" s="60" t="n"/>
+      <c r="D58" s="60" t="n"/>
+      <c r="E58" s="60" t="n"/>
+      <c r="F58" s="60" t="n"/>
+      <c r="G58" s="60" t="n"/>
+      <c r="H58" s="60" t="n"/>
+      <c r="I58" s="60" t="n"/>
+      <c r="J58" s="60" t="n"/>
+      <c r="K58" s="60" t="n"/>
+      <c r="L58" s="60" t="n"/>
+      <c r="M58" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="N58" s="61" t="n">
+      <c r="N58" s="94" t="n">
         <v>50</v>
       </c>
-      <c r="Q58" s="18">
+      <c r="O58" s="60" t="n"/>
+      <c r="P58" s="60" t="n"/>
+      <c r="Q58" s="44">
         <f>IF(SUMPRODUCT(ABS(C58:P58))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="59" t="inlineStr">
+      <c r="A59" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6729,19 +7142,31 @@
           <t>humiliate</t>
         </is>
       </c>
-      <c r="J59" s="54" t="n">
+      <c r="C59" s="60" t="n"/>
+      <c r="D59" s="60" t="n"/>
+      <c r="E59" s="60" t="n"/>
+      <c r="F59" s="60" t="n"/>
+      <c r="G59" s="60" t="n"/>
+      <c r="H59" s="60" t="n"/>
+      <c r="I59" s="60" t="n"/>
+      <c r="J59" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="N59" s="54" t="n">
+      <c r="K59" s="60" t="n"/>
+      <c r="L59" s="60" t="n"/>
+      <c r="M59" s="60" t="n"/>
+      <c r="N59" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q59" s="18">
+      <c r="O59" s="60" t="n"/>
+      <c r="P59" s="60" t="n"/>
+      <c r="Q59" s="44">
         <f>IF(SUMPRODUCT(ABS(C59:P59))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="59" t="inlineStr">
+      <c r="A60" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6751,19 +7176,31 @@
           <t>embolden</t>
         </is>
       </c>
-      <c r="J60" s="61" t="n">
+      <c r="C60" s="60" t="n"/>
+      <c r="D60" s="60" t="n"/>
+      <c r="E60" s="60" t="n"/>
+      <c r="F60" s="60" t="n"/>
+      <c r="G60" s="60" t="n"/>
+      <c r="H60" s="60" t="n"/>
+      <c r="I60" s="60" t="n"/>
+      <c r="J60" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="N60" s="61" t="n">
+      <c r="K60" s="60" t="n"/>
+      <c r="L60" s="60" t="n"/>
+      <c r="M60" s="60" t="n"/>
+      <c r="N60" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q60" s="18">
+      <c r="O60" s="60" t="n"/>
+      <c r="P60" s="60" t="n"/>
+      <c r="Q60" s="44">
         <f>IF(SUMPRODUCT(ABS(C60:P60))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="59" t="inlineStr">
+      <c r="A61" s="60" t="inlineStr">
         <is>
           <t>STANDING</t>
         </is>
@@ -6773,19 +7210,31 @@
           <t>enthrall</t>
         </is>
       </c>
-      <c r="L61" s="54" t="n">
+      <c r="C61" s="60" t="n"/>
+      <c r="D61" s="60" t="n"/>
+      <c r="E61" s="60" t="n"/>
+      <c r="F61" s="60" t="n"/>
+      <c r="G61" s="60" t="n"/>
+      <c r="H61" s="60" t="n"/>
+      <c r="I61" s="60" t="n"/>
+      <c r="J61" s="60" t="n"/>
+      <c r="K61" s="60" t="n"/>
+      <c r="L61" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="M61" s="61" t="n">
+      <c r="M61" s="94" t="n">
         <v>50</v>
       </c>
-      <c r="Q61" s="18">
+      <c r="N61" s="60" t="n"/>
+      <c r="O61" s="60" t="n"/>
+      <c r="P61" s="60" t="n"/>
+      <c r="Q61" s="44">
         <f>IF(SUMPRODUCT(ABS(C61:P61))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="59" t="inlineStr">
+      <c r="A62" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -6795,16 +7244,29 @@
           <t>enchant</t>
         </is>
       </c>
-      <c r="O62" s="61" t="n">
+      <c r="C62" s="60" t="n"/>
+      <c r="D62" s="60" t="n"/>
+      <c r="E62" s="60" t="n"/>
+      <c r="F62" s="60" t="n"/>
+      <c r="G62" s="60" t="n"/>
+      <c r="H62" s="60" t="n"/>
+      <c r="I62" s="60" t="n"/>
+      <c r="J62" s="60" t="n"/>
+      <c r="K62" s="60" t="n"/>
+      <c r="L62" s="60" t="n"/>
+      <c r="M62" s="60" t="n"/>
+      <c r="N62" s="60" t="n"/>
+      <c r="O62" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q62" s="18">
+      <c r="P62" s="60" t="n"/>
+      <c r="Q62" s="44">
         <f>IF(SUMPRODUCT(ABS(C62:P62))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="59" t="inlineStr">
+      <c r="A63" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -6814,16 +7276,29 @@
           <t>dispel</t>
         </is>
       </c>
-      <c r="O63" s="54" t="n">
+      <c r="C63" s="60" t="n"/>
+      <c r="D63" s="60" t="n"/>
+      <c r="E63" s="60" t="n"/>
+      <c r="F63" s="60" t="n"/>
+      <c r="G63" s="60" t="n"/>
+      <c r="H63" s="60" t="n"/>
+      <c r="I63" s="60" t="n"/>
+      <c r="J63" s="60" t="n"/>
+      <c r="K63" s="60" t="n"/>
+      <c r="L63" s="60" t="n"/>
+      <c r="M63" s="60" t="n"/>
+      <c r="N63" s="60" t="n"/>
+      <c r="O63" s="91" t="n">
         <v>-100</v>
       </c>
-      <c r="Q63" s="18">
+      <c r="P63" s="60" t="n"/>
+      <c r="Q63" s="44">
         <f>IF(SUMPRODUCT(ABS(C63:P63))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="59" t="inlineStr">
+      <c r="A64" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -6833,16 +7308,29 @@
           <t>infuse</t>
         </is>
       </c>
-      <c r="P64" s="61" t="n">
+      <c r="C64" s="60" t="n"/>
+      <c r="D64" s="60" t="n"/>
+      <c r="E64" s="60" t="n"/>
+      <c r="F64" s="60" t="n"/>
+      <c r="G64" s="60" t="n"/>
+      <c r="H64" s="60" t="n"/>
+      <c r="I64" s="60" t="n"/>
+      <c r="J64" s="60" t="n"/>
+      <c r="K64" s="60" t="n"/>
+      <c r="L64" s="60" t="n"/>
+      <c r="M64" s="60" t="n"/>
+      <c r="N64" s="60" t="n"/>
+      <c r="O64" s="60" t="n"/>
+      <c r="P64" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q64" s="18">
+      <c r="Q64" s="44">
         <f>IF(SUMPRODUCT(ABS(C64:P64))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="59" t="inlineStr">
+      <c r="A65" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -6852,16 +7340,29 @@
           <t>drain</t>
         </is>
       </c>
-      <c r="P65" s="54" t="n">
+      <c r="C65" s="60" t="n"/>
+      <c r="D65" s="60" t="n"/>
+      <c r="E65" s="60" t="n"/>
+      <c r="F65" s="60" t="n"/>
+      <c r="G65" s="60" t="n"/>
+      <c r="H65" s="60" t="n"/>
+      <c r="I65" s="60" t="n"/>
+      <c r="J65" s="60" t="n"/>
+      <c r="K65" s="60" t="n"/>
+      <c r="L65" s="60" t="n"/>
+      <c r="M65" s="60" t="n"/>
+      <c r="N65" s="60" t="n"/>
+      <c r="O65" s="60" t="n"/>
+      <c r="P65" s="91" t="n">
         <v>-100</v>
       </c>
-      <c r="Q65" s="18">
+      <c r="Q65" s="44">
         <f>IF(SUMPRODUCT(ABS(C65:P65))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="59" t="inlineStr">
+      <c r="A66" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -6871,19 +7372,31 @@
           <t>ward</t>
         </is>
       </c>
-      <c r="O66" s="61" t="n">
+      <c r="C66" s="60" t="n"/>
+      <c r="D66" s="60" t="n"/>
+      <c r="E66" s="60" t="n"/>
+      <c r="F66" s="60" t="n"/>
+      <c r="G66" s="60" t="n"/>
+      <c r="H66" s="60" t="n"/>
+      <c r="I66" s="60" t="n"/>
+      <c r="J66" s="60" t="n"/>
+      <c r="K66" s="60" t="n"/>
+      <c r="L66" s="60" t="n"/>
+      <c r="M66" s="60" t="n"/>
+      <c r="N66" s="60" t="n"/>
+      <c r="O66" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="P66" s="61" t="n">
+      <c r="P66" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q66" s="18">
+      <c r="Q66" s="44">
         <f>IF(SUMPRODUCT(ABS(C66:P66))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="59" t="inlineStr">
+      <c r="A67" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -6893,19 +7406,31 @@
           <t>siphon</t>
         </is>
       </c>
-      <c r="O67" s="54" t="n">
+      <c r="C67" s="60" t="n"/>
+      <c r="D67" s="60" t="n"/>
+      <c r="E67" s="60" t="n"/>
+      <c r="F67" s="60" t="n"/>
+      <c r="G67" s="60" t="n"/>
+      <c r="H67" s="60" t="n"/>
+      <c r="I67" s="60" t="n"/>
+      <c r="J67" s="60" t="n"/>
+      <c r="K67" s="60" t="n"/>
+      <c r="L67" s="60" t="n"/>
+      <c r="M67" s="60" t="n"/>
+      <c r="N67" s="60" t="n"/>
+      <c r="O67" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="P67" s="54" t="n">
+      <c r="P67" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q67" s="18">
+      <c r="Q67" s="44">
         <f>IF(SUMPRODUCT(ABS(C67:P67))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="59" t="inlineStr">
+      <c r="A68" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -6915,19 +7440,31 @@
           <t>bind</t>
         </is>
       </c>
-      <c r="O68" s="61" t="n">
+      <c r="C68" s="60" t="n"/>
+      <c r="D68" s="60" t="n"/>
+      <c r="E68" s="60" t="n"/>
+      <c r="F68" s="60" t="n"/>
+      <c r="G68" s="60" t="n"/>
+      <c r="H68" s="60" t="n"/>
+      <c r="I68" s="60" t="n"/>
+      <c r="J68" s="60" t="n"/>
+      <c r="K68" s="60" t="n"/>
+      <c r="L68" s="60" t="n"/>
+      <c r="M68" s="60" t="n"/>
+      <c r="N68" s="60" t="n"/>
+      <c r="O68" s="94" t="n">
         <v>70</v>
       </c>
-      <c r="P68" s="54" t="n">
+      <c r="P68" s="91" t="n">
         <v>-30</v>
       </c>
-      <c r="Q68" s="18">
+      <c r="Q68" s="44">
         <f>IF(SUMPRODUCT(ABS(C68:P68))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="59" t="inlineStr">
+      <c r="A69" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -6937,19 +7474,31 @@
           <t>surge</t>
         </is>
       </c>
-      <c r="O69" s="54" t="n">
+      <c r="C69" s="60" t="n"/>
+      <c r="D69" s="60" t="n"/>
+      <c r="E69" s="60" t="n"/>
+      <c r="F69" s="60" t="n"/>
+      <c r="G69" s="60" t="n"/>
+      <c r="H69" s="60" t="n"/>
+      <c r="I69" s="60" t="n"/>
+      <c r="J69" s="60" t="n"/>
+      <c r="K69" s="60" t="n"/>
+      <c r="L69" s="60" t="n"/>
+      <c r="M69" s="60" t="n"/>
+      <c r="N69" s="60" t="n"/>
+      <c r="O69" s="91" t="n">
         <v>-40</v>
       </c>
-      <c r="P69" s="61" t="n">
+      <c r="P69" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="Q69" s="18">
+      <c r="Q69" s="44">
         <f>IF(SUMPRODUCT(ABS(C69:P69))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="59" t="inlineStr">
+      <c r="A70" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -6959,22 +7508,33 @@
           <t>curse</t>
         </is>
       </c>
-      <c r="F70" s="54" t="n">
+      <c r="C70" s="60" t="n"/>
+      <c r="D70" s="60" t="n"/>
+      <c r="E70" s="60" t="n"/>
+      <c r="F70" s="91" t="n">
         <v>-30</v>
       </c>
-      <c r="M70" s="54" t="n">
+      <c r="G70" s="60" t="n"/>
+      <c r="H70" s="60" t="n"/>
+      <c r="I70" s="60" t="n"/>
+      <c r="J70" s="60" t="n"/>
+      <c r="K70" s="60" t="n"/>
+      <c r="L70" s="60" t="n"/>
+      <c r="M70" s="91" t="n">
         <v>-30</v>
       </c>
-      <c r="O70" s="61" t="n">
+      <c r="N70" s="60" t="n"/>
+      <c r="O70" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q70" s="18">
+      <c r="P70" s="60" t="n"/>
+      <c r="Q70" s="44">
         <f>IF(SUMPRODUCT(ABS(C70:P70))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="59" t="inlineStr">
+      <c r="A71" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -6984,22 +7544,33 @@
           <t>blessing</t>
         </is>
       </c>
-      <c r="F71" s="61" t="n">
+      <c r="C71" s="60" t="n"/>
+      <c r="D71" s="60" t="n"/>
+      <c r="E71" s="60" t="n"/>
+      <c r="F71" s="94" t="n">
         <v>30</v>
       </c>
-      <c r="J71" s="61" t="n">
+      <c r="G71" s="60" t="n"/>
+      <c r="H71" s="60" t="n"/>
+      <c r="I71" s="60" t="n"/>
+      <c r="J71" s="94" t="n">
         <v>30</v>
       </c>
-      <c r="O71" s="61" t="n">
+      <c r="K71" s="60" t="n"/>
+      <c r="L71" s="60" t="n"/>
+      <c r="M71" s="60" t="n"/>
+      <c r="N71" s="60" t="n"/>
+      <c r="O71" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q71" s="18">
+      <c r="P71" s="60" t="n"/>
+      <c r="Q71" s="44">
         <f>IF(SUMPRODUCT(ABS(C71:P71))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="59" t="inlineStr">
+      <c r="A72" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -7009,19 +7580,31 @@
           <t>soulburn</t>
         </is>
       </c>
-      <c r="F72" s="54" t="n">
+      <c r="C72" s="60" t="n"/>
+      <c r="D72" s="60" t="n"/>
+      <c r="E72" s="60" t="n"/>
+      <c r="F72" s="91" t="n">
         <v>-40</v>
       </c>
-      <c r="P72" s="54" t="n">
+      <c r="G72" s="60" t="n"/>
+      <c r="H72" s="60" t="n"/>
+      <c r="I72" s="60" t="n"/>
+      <c r="J72" s="60" t="n"/>
+      <c r="K72" s="60" t="n"/>
+      <c r="L72" s="60" t="n"/>
+      <c r="M72" s="60" t="n"/>
+      <c r="N72" s="60" t="n"/>
+      <c r="O72" s="60" t="n"/>
+      <c r="P72" s="91" t="n">
         <v>-60</v>
       </c>
-      <c r="Q72" s="18">
+      <c r="Q72" s="44">
         <f>IF(SUMPRODUCT(ABS(C72:P72))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="59" t="inlineStr">
+      <c r="A73" s="60" t="inlineStr">
         <is>
           <t>MYSTIC</t>
         </is>
@@ -7031,19 +7614,31 @@
           <t>hallow</t>
         </is>
       </c>
-      <c r="J73" s="61" t="n">
+      <c r="C73" s="60" t="n"/>
+      <c r="D73" s="60" t="n"/>
+      <c r="E73" s="60" t="n"/>
+      <c r="F73" s="60" t="n"/>
+      <c r="G73" s="60" t="n"/>
+      <c r="H73" s="60" t="n"/>
+      <c r="I73" s="60" t="n"/>
+      <c r="J73" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="O73" s="61" t="n">
+      <c r="K73" s="60" t="n"/>
+      <c r="L73" s="60" t="n"/>
+      <c r="M73" s="60" t="n"/>
+      <c r="N73" s="60" t="n"/>
+      <c r="O73" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="Q73" s="18">
+      <c r="P73" s="60" t="n"/>
+      <c r="Q73" s="44">
         <f>IF(SUMPRODUCT(ABS(C73:P73))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="59" t="inlineStr">
+      <c r="A74" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7053,16 +7648,29 @@
           <t>mend</t>
         </is>
       </c>
-      <c r="F74" s="61" t="n">
+      <c r="C74" s="60" t="n"/>
+      <c r="D74" s="60" t="n"/>
+      <c r="E74" s="60" t="n"/>
+      <c r="F74" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q74" s="18">
+      <c r="G74" s="60" t="n"/>
+      <c r="H74" s="60" t="n"/>
+      <c r="I74" s="60" t="n"/>
+      <c r="J74" s="60" t="n"/>
+      <c r="K74" s="60" t="n"/>
+      <c r="L74" s="60" t="n"/>
+      <c r="M74" s="60" t="n"/>
+      <c r="N74" s="60" t="n"/>
+      <c r="O74" s="60" t="n"/>
+      <c r="P74" s="60" t="n"/>
+      <c r="Q74" s="44">
         <f>IF(SUMPRODUCT(ABS(C74:P74))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="59" t="inlineStr">
+      <c r="A75" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7072,16 +7680,29 @@
           <t>rally</t>
         </is>
       </c>
-      <c r="G75" s="61" t="n">
+      <c r="C75" s="60" t="n"/>
+      <c r="D75" s="60" t="n"/>
+      <c r="E75" s="60" t="n"/>
+      <c r="F75" s="60" t="n"/>
+      <c r="G75" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q75" s="18">
+      <c r="H75" s="60" t="n"/>
+      <c r="I75" s="60" t="n"/>
+      <c r="J75" s="60" t="n"/>
+      <c r="K75" s="60" t="n"/>
+      <c r="L75" s="60" t="n"/>
+      <c r="M75" s="60" t="n"/>
+      <c r="N75" s="60" t="n"/>
+      <c r="O75" s="60" t="n"/>
+      <c r="P75" s="60" t="n"/>
+      <c r="Q75" s="44">
         <f>IF(SUMPRODUCT(ABS(C75:P75))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="59" t="inlineStr">
+      <c r="A76" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7091,16 +7712,29 @@
           <t>courage</t>
         </is>
       </c>
-      <c r="J76" s="61" t="n">
+      <c r="C76" s="60" t="n"/>
+      <c r="D76" s="60" t="n"/>
+      <c r="E76" s="60" t="n"/>
+      <c r="F76" s="60" t="n"/>
+      <c r="G76" s="60" t="n"/>
+      <c r="H76" s="60" t="n"/>
+      <c r="I76" s="60" t="n"/>
+      <c r="J76" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q76" s="18">
+      <c r="K76" s="60" t="n"/>
+      <c r="L76" s="60" t="n"/>
+      <c r="M76" s="60" t="n"/>
+      <c r="N76" s="60" t="n"/>
+      <c r="O76" s="60" t="n"/>
+      <c r="P76" s="60" t="n"/>
+      <c r="Q76" s="44">
         <f>IF(SUMPRODUCT(ABS(C76:P76))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="59" t="inlineStr">
+      <c r="A77" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7110,16 +7744,29 @@
           <t>lucidity</t>
         </is>
       </c>
-      <c r="K77" s="61" t="n">
+      <c r="C77" s="60" t="n"/>
+      <c r="D77" s="60" t="n"/>
+      <c r="E77" s="60" t="n"/>
+      <c r="F77" s="60" t="n"/>
+      <c r="G77" s="60" t="n"/>
+      <c r="H77" s="60" t="n"/>
+      <c r="I77" s="60" t="n"/>
+      <c r="J77" s="60" t="n"/>
+      <c r="K77" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q77" s="18">
+      <c r="L77" s="60" t="n"/>
+      <c r="M77" s="60" t="n"/>
+      <c r="N77" s="60" t="n"/>
+      <c r="O77" s="60" t="n"/>
+      <c r="P77" s="60" t="n"/>
+      <c r="Q77" s="44">
         <f>IF(SUMPRODUCT(ABS(C77:P77))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="59" t="inlineStr">
+      <c r="A78" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7129,16 +7776,29 @@
           <t>unbind</t>
         </is>
       </c>
-      <c r="L78" s="61" t="n">
+      <c r="C78" s="60" t="n"/>
+      <c r="D78" s="60" t="n"/>
+      <c r="E78" s="60" t="n"/>
+      <c r="F78" s="60" t="n"/>
+      <c r="G78" s="60" t="n"/>
+      <c r="H78" s="60" t="n"/>
+      <c r="I78" s="60" t="n"/>
+      <c r="J78" s="60" t="n"/>
+      <c r="K78" s="60" t="n"/>
+      <c r="L78" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q78" s="18">
+      <c r="M78" s="60" t="n"/>
+      <c r="N78" s="60" t="n"/>
+      <c r="O78" s="60" t="n"/>
+      <c r="P78" s="60" t="n"/>
+      <c r="Q78" s="44">
         <f>IF(SUMPRODUCT(ABS(C78:P78))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="59" t="inlineStr">
+      <c r="A79" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7148,16 +7808,29 @@
           <t>brace</t>
         </is>
       </c>
-      <c r="D79" s="61" t="n">
+      <c r="C79" s="60" t="n"/>
+      <c r="D79" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q79" s="18">
+      <c r="E79" s="60" t="n"/>
+      <c r="F79" s="60" t="n"/>
+      <c r="G79" s="60" t="n"/>
+      <c r="H79" s="60" t="n"/>
+      <c r="I79" s="60" t="n"/>
+      <c r="J79" s="60" t="n"/>
+      <c r="K79" s="60" t="n"/>
+      <c r="L79" s="60" t="n"/>
+      <c r="M79" s="60" t="n"/>
+      <c r="N79" s="60" t="n"/>
+      <c r="O79" s="60" t="n"/>
+      <c r="P79" s="60" t="n"/>
+      <c r="Q79" s="44">
         <f>IF(SUMPRODUCT(ABS(C79:P79))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="59" t="inlineStr">
+      <c r="A80" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7167,16 +7840,29 @@
           <t>seal</t>
         </is>
       </c>
-      <c r="E80" s="61" t="n">
+      <c r="C80" s="60" t="n"/>
+      <c r="D80" s="60" t="n"/>
+      <c r="E80" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q80" s="18">
+      <c r="F80" s="60" t="n"/>
+      <c r="G80" s="60" t="n"/>
+      <c r="H80" s="60" t="n"/>
+      <c r="I80" s="60" t="n"/>
+      <c r="J80" s="60" t="n"/>
+      <c r="K80" s="60" t="n"/>
+      <c r="L80" s="60" t="n"/>
+      <c r="M80" s="60" t="n"/>
+      <c r="N80" s="60" t="n"/>
+      <c r="O80" s="60" t="n"/>
+      <c r="P80" s="60" t="n"/>
+      <c r="Q80" s="44">
         <f>IF(SUMPRODUCT(ABS(C80:P80))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="59" t="inlineStr">
+      <c r="A81" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7186,16 +7872,29 @@
           <t>haste</t>
         </is>
       </c>
-      <c r="H81" s="61" t="n">
+      <c r="C81" s="60" t="n"/>
+      <c r="D81" s="60" t="n"/>
+      <c r="E81" s="60" t="n"/>
+      <c r="F81" s="60" t="n"/>
+      <c r="G81" s="60" t="n"/>
+      <c r="H81" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q81" s="18">
+      <c r="I81" s="60" t="n"/>
+      <c r="J81" s="60" t="n"/>
+      <c r="K81" s="60" t="n"/>
+      <c r="L81" s="60" t="n"/>
+      <c r="M81" s="60" t="n"/>
+      <c r="N81" s="60" t="n"/>
+      <c r="O81" s="60" t="n"/>
+      <c r="P81" s="60" t="n"/>
+      <c r="Q81" s="44">
         <f>IF(SUMPRODUCT(ABS(C81:P81))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="59" t="inlineStr">
+      <c r="A82" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7205,16 +7904,29 @@
           <t>keen</t>
         </is>
       </c>
-      <c r="I82" s="61" t="n">
+      <c r="C82" s="60" t="n"/>
+      <c r="D82" s="60" t="n"/>
+      <c r="E82" s="60" t="n"/>
+      <c r="F82" s="60" t="n"/>
+      <c r="G82" s="60" t="n"/>
+      <c r="H82" s="60" t="n"/>
+      <c r="I82" s="94" t="n">
         <v>100</v>
       </c>
-      <c r="Q82" s="18">
+      <c r="J82" s="60" t="n"/>
+      <c r="K82" s="60" t="n"/>
+      <c r="L82" s="60" t="n"/>
+      <c r="M82" s="60" t="n"/>
+      <c r="N82" s="60" t="n"/>
+      <c r="O82" s="60" t="n"/>
+      <c r="P82" s="60" t="n"/>
+      <c r="Q82" s="44">
         <f>IF(SUMPRODUCT(ABS(C82:P82))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="59" t="inlineStr">
+      <c r="A83" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7224,19 +7936,31 @@
           <t>regenerate</t>
         </is>
       </c>
-      <c r="F83" s="61" t="n">
+      <c r="C83" s="60" t="n"/>
+      <c r="D83" s="60" t="n"/>
+      <c r="E83" s="60" t="n"/>
+      <c r="F83" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="G83" s="61" t="n">
+      <c r="G83" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q83" s="18">
+      <c r="H83" s="60" t="n"/>
+      <c r="I83" s="60" t="n"/>
+      <c r="J83" s="60" t="n"/>
+      <c r="K83" s="60" t="n"/>
+      <c r="L83" s="60" t="n"/>
+      <c r="M83" s="60" t="n"/>
+      <c r="N83" s="60" t="n"/>
+      <c r="O83" s="60" t="n"/>
+      <c r="P83" s="60" t="n"/>
+      <c r="Q83" s="44">
         <f>IF(SUMPRODUCT(ABS(C83:P83))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="59" t="inlineStr">
+      <c r="A84" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7246,19 +7970,31 @@
           <t>fortify</t>
         </is>
       </c>
-      <c r="D84" s="61" t="n">
+      <c r="C84" s="60" t="n"/>
+      <c r="D84" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="E84" s="61" t="n">
+      <c r="E84" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q84" s="18">
+      <c r="F84" s="60" t="n"/>
+      <c r="G84" s="60" t="n"/>
+      <c r="H84" s="60" t="n"/>
+      <c r="I84" s="60" t="n"/>
+      <c r="J84" s="60" t="n"/>
+      <c r="K84" s="60" t="n"/>
+      <c r="L84" s="60" t="n"/>
+      <c r="M84" s="60" t="n"/>
+      <c r="N84" s="60" t="n"/>
+      <c r="O84" s="60" t="n"/>
+      <c r="P84" s="60" t="n"/>
+      <c r="Q84" s="44">
         <f>IF(SUMPRODUCT(ABS(C84:P84))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="59" t="inlineStr">
+      <c r="A85" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7268,19 +8004,31 @@
           <t>bolster</t>
         </is>
       </c>
-      <c r="D85" s="61" t="n">
+      <c r="C85" s="60" t="n"/>
+      <c r="D85" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="F85" s="61" t="n">
+      <c r="E85" s="60" t="n"/>
+      <c r="F85" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q85" s="18">
+      <c r="G85" s="60" t="n"/>
+      <c r="H85" s="60" t="n"/>
+      <c r="I85" s="60" t="n"/>
+      <c r="J85" s="60" t="n"/>
+      <c r="K85" s="60" t="n"/>
+      <c r="L85" s="60" t="n"/>
+      <c r="M85" s="60" t="n"/>
+      <c r="N85" s="60" t="n"/>
+      <c r="O85" s="60" t="n"/>
+      <c r="P85" s="60" t="n"/>
+      <c r="Q85" s="44">
         <f>IF(SUMPRODUCT(ABS(C85:P85))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="59" t="inlineStr">
+      <c r="A86" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7290,19 +8038,31 @@
           <t>preserve</t>
         </is>
       </c>
-      <c r="E86" s="61" t="n">
+      <c r="C86" s="60" t="n"/>
+      <c r="D86" s="60" t="n"/>
+      <c r="E86" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="F86" s="61" t="n">
+      <c r="F86" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q86" s="18">
+      <c r="G86" s="60" t="n"/>
+      <c r="H86" s="60" t="n"/>
+      <c r="I86" s="60" t="n"/>
+      <c r="J86" s="60" t="n"/>
+      <c r="K86" s="60" t="n"/>
+      <c r="L86" s="60" t="n"/>
+      <c r="M86" s="60" t="n"/>
+      <c r="N86" s="60" t="n"/>
+      <c r="O86" s="60" t="n"/>
+      <c r="P86" s="60" t="n"/>
+      <c r="Q86" s="44">
         <f>IF(SUMPRODUCT(ABS(C86:P86))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="59" t="inlineStr">
+      <c r="A87" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7312,19 +8072,31 @@
           <t>steady</t>
         </is>
       </c>
-      <c r="J87" s="61" t="n">
+      <c r="C87" s="60" t="n"/>
+      <c r="D87" s="60" t="n"/>
+      <c r="E87" s="60" t="n"/>
+      <c r="F87" s="60" t="n"/>
+      <c r="G87" s="60" t="n"/>
+      <c r="H87" s="60" t="n"/>
+      <c r="I87" s="60" t="n"/>
+      <c r="J87" s="94" t="n">
         <v>50</v>
       </c>
-      <c r="K87" s="61" t="n">
+      <c r="K87" s="94" t="n">
         <v>50</v>
       </c>
-      <c r="Q87" s="18">
+      <c r="L87" s="60" t="n"/>
+      <c r="M87" s="60" t="n"/>
+      <c r="N87" s="60" t="n"/>
+      <c r="O87" s="60" t="n"/>
+      <c r="P87" s="60" t="n"/>
+      <c r="Q87" s="44">
         <f>IF(SUMPRODUCT(ABS(C87:P87))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="59" t="inlineStr">
+      <c r="A88" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7334,19 +8106,31 @@
           <t>soothe</t>
         </is>
       </c>
-      <c r="G88" s="61" t="n">
+      <c r="C88" s="60" t="n"/>
+      <c r="D88" s="60" t="n"/>
+      <c r="E88" s="60" t="n"/>
+      <c r="F88" s="60" t="n"/>
+      <c r="G88" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="J88" s="61" t="n">
+      <c r="H88" s="60" t="n"/>
+      <c r="I88" s="60" t="n"/>
+      <c r="J88" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="Q88" s="18">
+      <c r="K88" s="60" t="n"/>
+      <c r="L88" s="60" t="n"/>
+      <c r="M88" s="60" t="n"/>
+      <c r="N88" s="60" t="n"/>
+      <c r="O88" s="60" t="n"/>
+      <c r="P88" s="60" t="n"/>
+      <c r="Q88" s="44">
         <f>IF(SUMPRODUCT(ABS(C88:P88))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="59" t="inlineStr">
+      <c r="A89" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7356,19 +8140,31 @@
           <t>sharpen</t>
         </is>
       </c>
-      <c r="I89" s="61" t="n">
+      <c r="C89" s="60" t="n"/>
+      <c r="D89" s="60" t="n"/>
+      <c r="E89" s="60" t="n"/>
+      <c r="F89" s="60" t="n"/>
+      <c r="G89" s="60" t="n"/>
+      <c r="H89" s="60" t="n"/>
+      <c r="I89" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="K89" s="61" t="n">
+      <c r="J89" s="60" t="n"/>
+      <c r="K89" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="Q89" s="18">
+      <c r="L89" s="60" t="n"/>
+      <c r="M89" s="60" t="n"/>
+      <c r="N89" s="60" t="n"/>
+      <c r="O89" s="60" t="n"/>
+      <c r="P89" s="60" t="n"/>
+      <c r="Q89" s="44">
         <f>IF(SUMPRODUCT(ABS(C89:P89))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="59" t="inlineStr">
+      <c r="A90" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7378,19 +8174,31 @@
           <t>vigilance</t>
         </is>
       </c>
-      <c r="I90" s="61" t="n">
+      <c r="C90" s="60" t="n"/>
+      <c r="D90" s="60" t="n"/>
+      <c r="E90" s="60" t="n"/>
+      <c r="F90" s="60" t="n"/>
+      <c r="G90" s="60" t="n"/>
+      <c r="H90" s="60" t="n"/>
+      <c r="I90" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="K90" s="61" t="n">
+      <c r="J90" s="60" t="n"/>
+      <c r="K90" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q90" s="18">
+      <c r="L90" s="60" t="n"/>
+      <c r="M90" s="60" t="n"/>
+      <c r="N90" s="60" t="n"/>
+      <c r="O90" s="60" t="n"/>
+      <c r="P90" s="60" t="n"/>
+      <c r="Q90" s="44">
         <f>IF(SUMPRODUCT(ABS(C90:P90))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="59" t="inlineStr">
+      <c r="A91" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7400,19 +8208,31 @@
           <t>quicken</t>
         </is>
       </c>
-      <c r="H91" s="61" t="n">
+      <c r="C91" s="60" t="n"/>
+      <c r="D91" s="60" t="n"/>
+      <c r="E91" s="60" t="n"/>
+      <c r="F91" s="60" t="n"/>
+      <c r="G91" s="60" t="n"/>
+      <c r="H91" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="I91" s="61" t="n">
+      <c r="I91" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q91" s="18">
+      <c r="J91" s="60" t="n"/>
+      <c r="K91" s="60" t="n"/>
+      <c r="L91" s="60" t="n"/>
+      <c r="M91" s="60" t="n"/>
+      <c r="N91" s="60" t="n"/>
+      <c r="O91" s="60" t="n"/>
+      <c r="P91" s="60" t="n"/>
+      <c r="Q91" s="44">
         <f>IF(SUMPRODUCT(ABS(C91:P91))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="59" t="inlineStr">
+      <c r="A92" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7422,19 +8242,31 @@
           <t>steel</t>
         </is>
       </c>
-      <c r="J92" s="61" t="n">
+      <c r="C92" s="60" t="n"/>
+      <c r="D92" s="60" t="n"/>
+      <c r="E92" s="60" t="n"/>
+      <c r="F92" s="60" t="n"/>
+      <c r="G92" s="60" t="n"/>
+      <c r="H92" s="60" t="n"/>
+      <c r="I92" s="60" t="n"/>
+      <c r="J92" s="94" t="n">
         <v>50</v>
       </c>
-      <c r="L92" s="61" t="n">
+      <c r="K92" s="60" t="n"/>
+      <c r="L92" s="94" t="n">
         <v>50</v>
       </c>
-      <c r="Q92" s="18">
+      <c r="M92" s="60" t="n"/>
+      <c r="N92" s="60" t="n"/>
+      <c r="O92" s="60" t="n"/>
+      <c r="P92" s="60" t="n"/>
+      <c r="Q92" s="44">
         <f>IF(SUMPRODUCT(ABS(C92:P92))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="59" t="inlineStr">
+      <c r="A93" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7444,19 +8276,31 @@
           <t>freedom</t>
         </is>
       </c>
-      <c r="H93" s="61" t="n">
+      <c r="C93" s="60" t="n"/>
+      <c r="D93" s="60" t="n"/>
+      <c r="E93" s="60" t="n"/>
+      <c r="F93" s="60" t="n"/>
+      <c r="G93" s="60" t="n"/>
+      <c r="H93" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="L93" s="61" t="n">
+      <c r="I93" s="60" t="n"/>
+      <c r="J93" s="60" t="n"/>
+      <c r="K93" s="60" t="n"/>
+      <c r="L93" s="94" t="n">
         <v>40</v>
       </c>
-      <c r="Q93" s="18">
+      <c r="M93" s="60" t="n"/>
+      <c r="N93" s="60" t="n"/>
+      <c r="O93" s="60" t="n"/>
+      <c r="P93" s="60" t="n"/>
+      <c r="Q93" s="44">
         <f>IF(SUMPRODUCT(ABS(C93:P93))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="59" t="inlineStr">
+      <c r="A94" s="60" t="inlineStr">
         <is>
           <t>RESTORE &amp; PROTECT</t>
         </is>
@@ -7466,13 +8310,25 @@
           <t>cleanse</t>
         </is>
       </c>
-      <c r="F94" s="61" t="n">
+      <c r="C94" s="60" t="n"/>
+      <c r="D94" s="60" t="n"/>
+      <c r="E94" s="60" t="n"/>
+      <c r="F94" s="94" t="n">
         <v>50</v>
       </c>
-      <c r="O94" s="54" t="n">
+      <c r="G94" s="60" t="n"/>
+      <c r="H94" s="60" t="n"/>
+      <c r="I94" s="60" t="n"/>
+      <c r="J94" s="60" t="n"/>
+      <c r="K94" s="60" t="n"/>
+      <c r="L94" s="60" t="n"/>
+      <c r="M94" s="60" t="n"/>
+      <c r="N94" s="60" t="n"/>
+      <c r="O94" s="91" t="n">
         <v>-50</v>
       </c>
-      <c r="Q94" s="18">
+      <c r="P94" s="60" t="n"/>
+      <c r="Q94" s="44">
         <f>IF(SUMPRODUCT(ABS(C94:P94))=100,"ok","*** FIX ***")</f>
         <v/>
       </c>
@@ -7603,7 +8459,7 @@
       </c>
       <c r="B8" s="74" t="inlineStr">
         <is>
-          <t>PROVISIONAL · 22 chosen</t>
+          <t>PROVISIONAL · 24 chosen</t>
         </is>
       </c>
       <c r="C8" s="73">
@@ -7627,7 +8483,7 @@
         </is>
       </c>
       <c r="C9" s="73">
-        <f>COUNTA('L5 State axes'!A8:A47)</f>
+        <f>COUNTA('L5 Tracks'!A8:A47)</f>
         <v/>
       </c>
       <c r="D9" s="73">
@@ -7643,7 +8499,7 @@
       </c>
       <c r="B10" s="30" t="inlineStr">
         <is>
-          <t>PRELIMINARY · CLOSE LAST</t>
+          <t>DRAFTED · seven · CLOSES IN PHASE 2</t>
         </is>
       </c>
       <c r="C10" s="26">
@@ -7907,7 +8763,7 @@
         </is>
       </c>
       <c r="C23" s="73">
-        <f>COUNTA('L25 Transient-to-Persistent con'!A8:A47)</f>
+        <f>COUNTA('L25 Landing models'!A8:A47)</f>
         <v/>
       </c>
       <c r="D23" s="73">
@@ -7943,7 +8799,7 @@
       </c>
       <c r="B25" s="74" t="inlineStr">
         <is>
-          <t>SHAPE SETTLED · three · Aug 2026</t>
+          <t>SETTLED · two · Aug 2026</t>
         </is>
       </c>
       <c r="C25" s="73">
@@ -9234,7 +10090,7 @@
       </c>
       <c r="B8" s="70" t="inlineStr">
         <is>
-          <t>vitality Resource ≤ 0</t>
+          <t>vitality Track &lt;= 0</t>
         </is>
       </c>
       <c r="C8" s="70" t="inlineStr">
@@ -9269,12 +10125,12 @@
     <row r="10">
       <c r="A10" s="70" t="inlineStr">
         <is>
-          <t>an Entity holds a State</t>
+          <t>an Entity's Track is in a named band</t>
         </is>
       </c>
       <c r="B10" s="70" t="inlineStr">
         <is>
-          <t>is prone</t>
+          <t>mobility in its "prone" band</t>
         </is>
       </c>
       <c r="C10" s="70" t="inlineStr">
@@ -9375,7 +10231,7 @@
     <row r="16">
       <c r="A16" s="70" t="inlineStr">
         <is>
-          <t>THREE BLANKS THAT MUST BE FILLED HERE, NOT LATER — and research now proposes all three. (1) DEPTH LIMIT: 32. (2) AT THE LIMIT: halt without applying, and WRITE A RECORD. (3) ORDER: (class, layer, component_id, listener_id, target_entity_id).</t>
+          <t>THE THREE BLANKS, FILLED AUG 2026 — see the SETTLED rows below.</t>
         </is>
       </c>
     </row>
@@ -9409,7 +10265,7 @@
       <c r="B20" s="72" t="inlineStr"/>
       <c r="C20" s="72" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>ADOPTED</t>
         </is>
       </c>
       <c r="D20" s="72" t="inlineStr">
@@ -9455,7 +10311,7 @@
       <c r="B23" s="72" t="inlineStr"/>
       <c r="C23" s="72" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>ADOPTED</t>
         </is>
       </c>
       <c r="D23" s="72" t="inlineStr">
@@ -9487,7 +10343,7 @@
       <c r="B25" s="72" t="inlineStr"/>
       <c r="C25" s="72" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>ADOPTED</t>
         </is>
       </c>
       <c r="D25" s="72" t="inlineStr">
@@ -9878,7 +10734,7 @@
     <row r="12">
       <c r="A12" s="70" t="inlineStr">
         <is>
-          <t>THREE IS THE TARGET AND THE CEILING. Every Socket is a permanent dependency for every Component ever written AND a hole in the documentation. A capability belongs here only if the Substrate cannot function without it AND freezing one answer would make a whole class of Setting impossible.</t>
+          <t>TWO IS THE NUMBER, AND IT WAS EARNED. Every Socket is a hole in the explanation as well as the code — Time, Budget and Landing each failed that test and were resolved into the Substrate or the base Ruleset.</t>
         </is>
       </c>
     </row>
@@ -13524,7 +14380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="19" min="1" max="1"/>
@@ -13543,14 +14399,14 @@
     <row r="2">
       <c r="A2" s="64" t="inlineStr">
         <is>
-          <t>SETTLED · Aug 2026 · nine</t>
+          <t>SETTLED · Aug 2026 · eight</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="65" t="inlineStr">
         <is>
-          <t>What EVERY Entity has, no exceptions. Six structural fields plus one slot per Noun kind.</t>
+          <t>What EVERY Entity has, no exceptions. Six structural fields plus two Noun slots — capacities and tracks. Tag membership rides the structural tags field; Relationship is an Entity and needs no slot.</t>
         </is>
       </c>
     </row>
@@ -13663,7 +14519,7 @@
       </c>
       <c r="C10" s="76" t="inlineStr">
         <is>
-          <t>zero or more, optional magnitude</t>
+          <t>zero or more, magnitude declared per Tag</t>
         </is>
       </c>
       <c r="D10" s="76" t="inlineStr">
@@ -13734,7 +14590,7 @@
       </c>
       <c r="D13" s="76" t="inlineStr">
         <is>
-          <t>The escape hatch: anything that is NOT one of the five Noun kinds. WATCH THIS — anything put here that another Component must read is a missing Noun slot in disguise.</t>
+          <t>The escape hatch: anything that is NOT one of the four Noun kinds. WATCH THIS — anything put here that another Component must read is a missing Noun slot in disguise.</t>
         </is>
       </c>
     </row>
@@ -13763,7 +14619,7 @@
     <row r="15">
       <c r="A15" s="76" t="inlineStr">
         <is>
-          <t>states</t>
+          <t>tracks</t>
         </is>
       </c>
       <c r="B15" s="76" t="inlineStr">
@@ -13773,158 +14629,136 @@
       </c>
       <c r="C15" s="76" t="inlineStr">
         <is>
-          <t>axis -&gt; State ID, optional magnitude</t>
+          <t>Track ID -&gt; current, bounded by a max</t>
         </is>
       </c>
       <c r="D15" s="76" t="inlineStr">
         <is>
-          <t>Aggregates by MAX, never sum (PF2e's rule; additive stacking makes any repeatable source unbounded).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="76" t="inlineStr">
-        <is>
-          <t>resources</t>
-        </is>
-      </c>
-      <c r="B16" s="76" t="inlineStr">
-        <is>
-          <t>Noun slot</t>
-        </is>
-      </c>
-      <c r="C16" s="76" t="inlineStr">
-        <is>
-          <t>Resource ID -&gt; value, with Thresholds</t>
-        </is>
-      </c>
-      <c r="D16" s="76" t="inlineStr">
-        <is>
-          <t>Aggregates by CLAMP. The Substrate ships none.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="76" t="inlineStr">
+          <t>Merged from the old states + resources slots, Aug 2026. Aggregates by CLAMP; named conditions are BANDS on a Track, never things; payable is a flag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="76" t="inlineStr">
         <is>
           <t>RELATIONSHIP NEEDS NO SLOT — it is an Entity.</t>
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="71" t="inlineStr">
+        <is>
+          <t>CONSIDERED AND REJECTED</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
-      <c r="A20" s="71" t="inlineStr">
-        <is>
-          <t>CONSIDERED AND REJECTED</t>
+      <c r="A20" s="72" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="B20" s="72" t="inlineStr"/>
+      <c r="C20" s="72" t="inlineStr"/>
+      <c r="D20" s="72" t="inlineStr">
+        <is>
+          <t>SPLIT. Destruction is a BAND on a lifecycle Track; retraction is a COMPENSATING RECORD, so the Entity is simply not produced by the Fold. No boolean, no default, no predicate to forget. Under "absent is not zero" a boolean would be three-valued with an INVERTED safe default.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="72" t="inlineStr">
         <is>
-          <t>exists</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B21" s="72" t="inlineStr"/>
       <c r="C21" s="72" t="inlineStr"/>
       <c r="D21" s="72" t="inlineStr">
         <is>
-          <t>SPLIT. Destruction is a STATE on a lifecycle axis; retraction is a COMPENSATING RECORD, so the Entity is simply not produced by the Fold. No boolean, no default, no predicate to forget. Under "absent is not zero" a boolean would be three-valued with an INVERTED safe default.</t>
+          <t>The PLACE SOCKET's Facet. Only the occupant interprets it; the Substrate never needs to.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="72" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B22" s="72" t="inlineStr"/>
       <c r="C22" s="72" t="inlineStr"/>
       <c r="D22" s="72" t="inlineStr">
         <is>
-          <t>The PLACE SOCKET's Facet. Only the occupant interprets it; the Substrate never needs to.</t>
+          <t>A LENS concern. Setting-specific, and the likeliest place for rule 10 (PII) to be violated.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="72" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>mass / bulk</t>
         </is>
       </c>
       <c r="B23" s="72" t="inlineStr"/>
       <c r="C23" s="72" t="inlineStr"/>
       <c r="D23" s="72" t="inlineStr">
         <is>
-          <t>A LENS concern. Setting-specific, and the likeliest place for rule 10 (PII) to be violated.</t>
+          <t>TAGS, with magnitudes.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="72" t="inlineStr">
         <is>
-          <t>mass / bulk</t>
+          <t>hardness</t>
         </is>
       </c>
       <c r="B24" s="72" t="inlineStr"/>
       <c r="C24" s="72" t="inlineStr"/>
       <c r="D24" s="72" t="inlineStr">
         <is>
-          <t>TAGS, with magnitudes.</t>
+          <t>A FLAT GUARD at R-850. Not an attribute at all.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="72" t="inlineStr">
         <is>
-          <t>hardness</t>
+          <t>the fourteen Dimensions</t>
         </is>
       </c>
       <c r="B25" s="72" t="inlineStr"/>
       <c r="C25" s="72" t="inlineStr"/>
       <c r="D25" s="72" t="inlineStr">
         <is>
-          <t>A FLAT GUARD at R-850. Not an attribute at all.</t>
+          <t>Axes a VECTOR travels on, never fields on a target.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="72" t="inlineStr">
         <is>
-          <t>the fourteen Dimensions</t>
+          <t>the inverse of any link</t>
         </is>
       </c>
       <c r="B26" s="72" t="inlineStr"/>
       <c r="C26" s="72" t="inlineStr"/>
       <c r="D26" s="72" t="inlineStr">
         <is>
-          <t>Axes a VECTOR travels on, never fields on a target.</t>
+          <t>DERIVED by the Fold. Writing both directions is denormalisation, and denormalisation desyncs.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="72" t="inlineStr">
         <is>
-          <t>the inverse of any link</t>
+          <t>generation / version counter</t>
         </is>
       </c>
       <c r="B27" s="72" t="inlineStr"/>
       <c r="C27" s="72" t="inlineStr"/>
       <c r="D27" s="72" t="inlineStr">
-        <is>
-          <t>DERIVED by the Fold. Writing both directions is denormalisation, and denormalisation desyncs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="72" t="inlineStr">
-        <is>
-          <t>generation / version counter</t>
-        </is>
-      </c>
-      <c r="B28" s="72" t="inlineStr"/>
-      <c r="C28" s="72" t="inlineStr"/>
-      <c r="D28" s="72" t="inlineStr">
         <is>
           <t>Not needed — generational indices exist to stop a RECYCLED id pointing at a new entity. Never reusing ids removes the precondition, and a Record from 400 Moments ago then needs one integer rather than two forever.</t>
         </is>
@@ -13992,12 +14826,12 @@
       </c>
       <c r="C6" s="67" t="inlineStr">
         <is>
-          <t>Resources</t>
+          <t>Tracks</t>
         </is>
       </c>
       <c r="D6" s="67" t="inlineStr">
         <is>
-          <t>State axes</t>
+          <t>Collapsed axes -&gt; bands</t>
         </is>
       </c>
       <c r="E6" s="67" t="inlineStr">
@@ -14132,12 +14966,12 @@
       </c>
       <c r="C11" s="76" t="inlineStr">
         <is>
-          <t>vitality · vigor · mobility · acuity · composure · clarity · will · temperature · integrity · substance</t>
+          <t>vitality · vigor · mobility · acuity · composure · clarity · will (+ essence in mystic Settings)</t>
         </is>
       </c>
       <c r="D11" s="76" t="inlineStr">
         <is>
-          <t>Specialisations. integrity is bone and structure, substance is flesh and matter — without them a hammer blow against a person would land on nothing.</t>
+          <t>conditions are bands on these Tracks — prone is a band on mobility</t>
         </is>
       </c>
       <c r="E11" s="76" t="inlineStr">
@@ -14159,12 +14993,12 @@
       </c>
       <c r="C12" s="76" t="inlineStr">
         <is>
-          <t>integrity</t>
+          <t>integrity · substance (+ temperature)</t>
         </is>
       </c>
       <c r="D12" s="76" t="inlineStr">
         <is>
-          <t>access</t>
+          <t>the old access axis collapsed into bands (L5)</t>
         </is>
       </c>
       <c r="E12" s="76" t="inlineStr">
@@ -14186,14 +15020,10 @@
       </c>
       <c r="C13" s="76" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D13" s="76" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="D13" s="76" t="n"/>
       <c r="E13" s="76" t="inlineStr">
         <is>
           <t>extent and containment, per the Place Socket</t>
@@ -14213,12 +15043,12 @@
       </c>
       <c r="C14" s="76" t="inlineStr">
         <is>
-          <t>standing</t>
+          <t>standing · vitality (as cohesion)</t>
         </is>
       </c>
       <c r="D14" s="76" t="inlineStr">
         <is>
-          <t>posture</t>
+          <t>the old posture axis collapsed into bands (L5)</t>
         </is>
       </c>
       <c r="E14" s="76" t="inlineStr">
@@ -14240,12 +15070,12 @@
       </c>
       <c r="C15" s="76" t="inlineStr">
         <is>
-          <t>credibility</t>
+          <t>standing (how believed)</t>
         </is>
       </c>
       <c r="D15" s="76" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>the old spread axis collapsed into bands (L5)</t>
         </is>
       </c>
       <c r="E15" s="76" t="inlineStr">
@@ -14267,12 +15097,12 @@
       </c>
       <c r="C16" s="76" t="inlineStr">
         <is>
-          <t>fuel</t>
+          <t>vigor (its fuel) · working (if magical)</t>
         </is>
       </c>
       <c r="D16" s="76" t="inlineStr">
         <is>
-          <t>intensity</t>
+          <t>the old intensity axis collapsed into bands (L5)</t>
         </is>
       </c>
       <c r="E16" s="76" t="inlineStr">
@@ -14341,7 +15171,7 @@
     <row r="2">
       <c r="A2" s="64" t="inlineStr">
         <is>
-          <t>PENDING · BLOCKING · research-seeded Aug 2026</t>
+          <t>PROVISIONAL · Aug 2026 · twenty-four (11 Substrate + 13 Ruleset) · closes against content</t>
         </is>
       </c>
     </row>
@@ -14549,7 +15379,7 @@
       </c>
       <c r="E12" s="70" t="inlineStr">
         <is>
-          <t>Feeds integer apportionment. Not a Resource — not depletable by the Substrate</t>
+          <t>Feeds integer apportionment. Not a Track — not depletable by the Substrate</t>
         </is>
       </c>
     </row>
@@ -14788,7 +15618,7 @@
       </c>
       <c r="E21" s="70" t="inlineStr">
         <is>
-          <t>Not a Resource — the label the Resource system keys on</t>
+          <t>Not a Track — the label expenditure keys on</t>
         </is>
       </c>
     </row>
@@ -15076,7 +15906,7 @@
       <c r="C38" s="72" t="inlineStr"/>
       <c r="D38" s="72" t="inlineStr">
         <is>
-          <t>ARGUE — PROPOSED CHANGE. Make it declared PER TAG, permanently from mint: "carries no magnitude" or "carries a magnitude in unit U". Optional per instance means every reader writes if(magnitude !== undefined), which turns "absent is not zero" into a per-call-site judgement. Lancer: 19 of 67 tags carry a value, and the value TYPE varies per tag — Reliable is a floor, Blast a radius, Overkill a DIE FACE. Nothing generic can be written over "the magnitude."</t>
+          <t>ADOPTED — magnitude is declared PER TAG, permanently from mint: "carries no magnitude" or "carries a magnitude in unit U". Optional per instance means every reader writes if(magnitude !== undefined), which turns "absent is not zero" into a per-call-site judgement. Lancer: 19 of 67 tags carry a value, and the value TYPE varies per tag — Reliable is a floor, Blast a radius, Overkill a DIE FACE. Nothing generic can be written over "the magnitude."</t>
         </is>
       </c>
       <c r="E38" s="72" t="inlineStr"/>
@@ -15717,7 +16547,7 @@
     <row r="2" ht="15" customHeight="1" s="19">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>PRELIMINARY · CLOSE LAST</t>
+          <t>DRAFTED · seven · CLOSES LAST, IN PHASE 2</t>
         </is>
       </c>
     </row>
@@ -15795,53 +16625,193 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="19">
-      <c r="A8" s="37" t="n"/>
-      <c r="B8" s="37" t="n"/>
-      <c r="C8" s="37" t="n"/>
-      <c r="D8" s="37" t="n"/>
-      <c r="E8" s="37" t="n"/>
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="B8" s="37" t="inlineStr">
+        <is>
+          <t>a Track moved by a magnitude</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>harm lands; a cost is paid; healing arrives</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="inlineStr">
+        <is>
+          <t>No — the fundamental operation</t>
+        </is>
+      </c>
+      <c r="E8" s="37" t="inlineStr">
+        <is>
+          <t>drafted — argument owed</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="19">
-      <c r="A9" s="37" t="n"/>
-      <c r="B9" s="37" t="n"/>
-      <c r="C9" s="37" t="n"/>
-      <c r="D9" s="37" t="n"/>
-      <c r="E9" s="37" t="n"/>
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+      <c r="B9" s="37" t="inlineStr">
+        <is>
+          <t>a value set outright, not moved</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>a door is barred; a flag flips</t>
+        </is>
+      </c>
+      <c r="D9" s="37" t="inlineStr">
+        <is>
+          <t>Not by Push — absolute, not relative</t>
+        </is>
+      </c>
+      <c r="E9" s="37" t="inlineStr">
+        <is>
+          <t>drafted — argument owed</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="19">
-      <c r="A10" s="37" t="n"/>
-      <c r="B10" s="37" t="n"/>
-      <c r="C10" s="37" t="n"/>
-      <c r="D10" s="37" t="n"/>
-      <c r="E10" s="37" t="n"/>
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>Place</t>
+        </is>
+      </c>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>position or containment changed</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>a creature moves; a coin enters a purse</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>No — a destination is not a magnitude (rule 27)</t>
+        </is>
+      </c>
+      <c r="E10" s="37" t="inlineStr">
+        <is>
+          <t>drafted — argument owed</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="19">
-      <c r="A11" s="37" t="n"/>
-      <c r="B11" s="37" t="n"/>
-      <c r="C11" s="37" t="n"/>
-      <c r="D11" s="37" t="n"/>
-      <c r="E11" s="37" t="n"/>
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>Repin</t>
+        </is>
+      </c>
+      <c r="B11" s="37" t="inlineStr">
+        <is>
+          <t>a pending vector's Moment changed</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>a blow is delayed; a spell is hastened</t>
+        </is>
+      </c>
+      <c r="D11" s="37" t="inlineStr">
+        <is>
+          <t>No — and it must name a doubloon cost (rule 16)</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="inlineStr">
+        <is>
+          <t>drafted — reasoning in Part 12</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="19">
-      <c r="A12" s="37" t="n"/>
-      <c r="B12" s="37" t="n"/>
-      <c r="C12" s="37" t="n"/>
-      <c r="D12" s="37" t="n"/>
-      <c r="E12" s="37" t="n"/>
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B12" s="37" t="inlineStr">
+        <is>
+          <t>a (relation, target) pair added or removed</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>an oath sworn; a part attached</t>
+        </is>
+      </c>
+      <c r="D12" s="37" t="inlineStr">
+        <is>
+          <t>No — relations are their own state</t>
+        </is>
+      </c>
+      <c r="E12" s="37" t="inlineStr">
+        <is>
+          <t>drafted — argument owed</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="19">
-      <c r="A13" s="37" t="n"/>
-      <c r="B13" s="37" t="n"/>
-      <c r="C13" s="37" t="n"/>
-      <c r="D13" s="37" t="n"/>
-      <c r="E13" s="37" t="n"/>
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>an Entity exists that did not</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>a rumour starts; a wall is conjured</t>
+        </is>
+      </c>
+      <c r="D13" s="37" t="inlineStr">
+        <is>
+          <t>No — existence precedes every other change</t>
+        </is>
+      </c>
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t>drafted — argument owed</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="19">
-      <c r="A14" s="37" t="n"/>
-      <c r="B14" s="37" t="n"/>
-      <c r="C14" s="37" t="n"/>
-      <c r="D14" s="37" t="n"/>
-      <c r="E14" s="37" t="n"/>
+      <c r="A14" s="37" t="inlineStr">
+        <is>
+          <t>Decide</t>
+        </is>
+      </c>
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>a Proposal resolved</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>a player chooses; a default fires</t>
+        </is>
+      </c>
+      <c r="D14" s="37" t="inlineStr">
+        <is>
+          <t>No — the bridge from pending to actual</t>
+        </is>
+      </c>
+      <c r="E14" s="37" t="inlineStr">
+        <is>
+          <t>drafted — argument owed</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="19">
       <c r="A15" s="37" t="n"/>
@@ -15851,7 +16821,11 @@
       <c r="E15" s="37" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="19">
-      <c r="A16" s="37" t="n"/>
+      <c r="A16" s="37" t="inlineStr">
+        <is>
+          <t>SUPERSEDES the 19-candidate list. Only Repin and the shape arguments are on record — the per-verb arguments for the other six are OWED before the Phase 2 closing procedure runs.</t>
+        </is>
+      </c>
       <c r="B16" s="37" t="n"/>
       <c r="C16" s="37" t="n"/>
       <c r="D16" s="37" t="n"/>

</xml_diff>

<commit_message>
Beta pivot 2/2: Phase 2 is the beta; 21 decisions recorded; beta-spec + brand-drafts; L6 arguments; Attempt Points
</commit_message>
<xml_diff>
--- a/docs/substrate-lists.xlsx
+++ b/docs/substrate-lists.xlsx
@@ -10462,7 +10462,7 @@
       </c>
       <c r="B33" s="76" t="inlineStr">
         <is>
-          <t>semantic class first, then (layer, component_id, listener_id, target_entity_id)</t>
+          <t>semantic class (substrate -&gt; mandatory -&gt; elective), then (layer, component_id, listener_id, target_entity_id, source_record_id)</t>
         </is>
       </c>
       <c r="C33" s="76" t="inlineStr">
@@ -10472,7 +10472,7 @@
       </c>
       <c r="D33" s="76" t="inlineStr">
         <is>
-          <t>The key may contain ONLY values that do not move when unrelated content is added. Drools salience is deterministic but NOT STABLE.</t>
+          <t>Settled Aug 2026 (Q3.8). source_record_id makes it a total order. The key may contain ONLY values that do not move when unrelated content is added.</t>
         </is>
       </c>
     </row>

</xml_diff>